<commit_message>
ZZPRDAT: zzprdat-kontext, Wochen-Todo und lastchange nachziehen
Eine Gegenpruefung hat gezeigt, dass saptasks/zzprdat-kontext.md noch den
Kurzstand vom 04.09. mit 'Technisch ist nichts mehr offen' fuehrte. Genau der
Fall, den CLAUDE.md Abschnitt 3.2 meint: der Nachtrag stand anderswo, diese
Datei widersprach ihm.

Der Kurzstand nennt jetzt den Befund, die Korrektur, die wiederholte Messreihe
und ausdruecklich die beiden Punkte, die NICHT behoben sind: der ungemessene
Druckzeitpunkt gegenueber der V2-Verbuchung und Z_ZZPRDAT_CHECK, der jeden
abweichenden Wert als 'Write-once nachgewiesen' meldet.

Das Wochen-Todo fuehrte bei beiden PM-03-Zeilen noch den Stand vor der
Korrektur; lastchange.md kannte die ganze ZZPRDAT- und ZC12-Arbeit vom 03. bis
07.09. ueberhaupt nicht, obwohl die Datei zu Sitzungsbeginn als zweites
geladen wird und die letzten sieben Tage abdecken soll.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -1901,12 +1901,12 @@
       <c r="I12" s="38" t="inlineStr"/>
       <c r="J12" s="38" t="inlineStr">
         <is>
-          <t>Loesung in T76 gebaut, im Paket ZPP1 und im Transportauftrag T76K912490. Auf sieben Wegen nachgetestet: CO01, CO02, COHV Sammelfreigabe, CO40 Umsetzung, Auftragsart PP22, MD04 und CO41. Write-once belegt. Auftrag bewusst nicht freigegeben, nichts nach P76 transportiert.</t>
+          <t>Loesung in T76 gebaut, im Paket ZPP1 und im Transportauftrag T76K912490. Am 07.09.2026 kam eine Korrektur dazu: BEFORE_UPDATE lief bei jedem Sichern und hätte Altaufträge ungewollt nachgefüllt; jetzt wird AFKO-FTRMI vorher geprüft. Danach alle sieben Wege plus Altauftragsfall und Write-once erneut gemessen, Aufträge 1241824 bis 1241830, Werte direkt aus AUFK.</t>
         </is>
       </c>
       <c r="K12" s="38" t="inlineStr">
         <is>
-          <t>04.09.2026</t>
+          <t>07.09.2026</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       <c r="I13" s="38" t="inlineStr"/>
       <c r="J13" s="38" t="inlineStr">
         <is>
-          <t>Anschreiben ist geschrieben und liegt als Outlook-Entwurf mit Betreff und angehängtem Lösungsdokument. Vor dem Versand fehlen zwei Handgriffe: Empfängeradressen für Lucas Castro, Florian Wächter, Marco Di Menco und Fabio Palma eintragen (in docs/ANSPRECHPARTNER.md nicht hinterlegt) und den Text aus docs/ZZPRDAT_Mail_Abnahme_2026-09-04.html hineinkopieren, weil Outlook hier jede Zuweisung an den Nachrichtentext verwirft. Danach zwei Rückmeldungen abwarten: fachliche Abnahme und Marcos Prüfung von Etikett und Typenschild. Erst dann den Auftrag T76K912490 freigeben, getrennt davon das Nachfüllen der Altbestände.</t>
+          <t>Anschreiben liegt als Outlook-Entwurf mit Betreff und angehängtem Lösungsdokument; vor dem Versand die Empfängeradressen eintragen und den Text aus docs/ZZPRDAT_Mail_Abnahme_2026-09-04.html hineinkopieren. Das Dokument hat seit 07.09.2026 die Kapitel 'So testen Sie es selbst' und 'Nachmessung vom 7. September'. Marco prüft Etikett und Typenschild und dabei neu auch den Zeitpunkt: der Verbuchungsbaustein läuft als V2 nach der Standardverbuchung, ein unmittelbarer Druck könnte das Feld noch leer sehen. Nicht behoben ist ausserdem, dass Z_ZZPRDAT_CHECK jeden abweichenden Wert als 'Write-once nachgewiesen' meldet.</t>
         </is>
       </c>
       <c r="K13" s="38" t="inlineStr"/>

</xml_diff>

<commit_message>
Document German railway deployment
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -466,7 +466,7 @@
     <x:t>08.09.2026</x:t>
   </x:si>
   <x:si>
-    <x:t>Produktive Quelle am 08.09. geprüft: SharePoint ist tagesaktuell, die Kopfdatei liefert aber nur die interne RechnungsAdressenID. Der App-Leser für AdressNummer-Kunde, Name Kunde, Land Kunde und Branche ist umgesetzt und getestet. Benötigt wird ein neuer Alphaplan-Kopfexport mit beiden Schlüsseln und den vier Kundenfeldern; danach TRDE gesichert neu laden und Füllgrade prüfen. Details: docs/BAHNMARKT_DE_ANBINDUNG_2026-09-08.md</x:t>
+    <x:t>App-seitig produktiv seit 08.09. 23:51: AdressNummer-Kunde, Name Kunde, Land Kunde und Branche werden gelesen; Bahnbranchen werden automatisch bestätigt. 680/680 Tests grün. SharePoint ist tagesaktuell, der Alphaplan-Rohkopf liefert aber weiterhin nur RechnungsAdressenID. Benötigt wird ein neuer Kopfexport mit beiden Schlüsseln und den vier Kundenfeldern; danach TRDE neu laden und Füllgrade prüfen. Details: docs/BAHNMARKT_DE_ANBINDUNG_2026-09-08.md</x:t>
   </x:si>
   <x:si>
     <x:t>25</x:t>
@@ -1819,7 +1819,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{be9ed5ab-e556-4294-948c-d3a637ae89ab}</x14:id>
+          <x14:id>{87c7b6d1-6a95-4379-8345-deb33b90197f}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -1833,7 +1833,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{be9ed5ab-e556-4294-948c-d3a637ae89ab}">
+          <x14:cfRule type="dataBar" id="{87c7b6d1-6a95-4379-8345-deb33b90197f}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
Document the journal clearing fields and the two measurements behind them
Marks the superseded sentence in the 08.09. section instead of leaving it
standing: it said the fields had deliberately not been built, which is no
longer true. What still holds - no derived date paid - is stated explicitly.

Records both live findings so the next session does not repeat them: the
unusable JDT1.IntrnMatch, and the multiple reconciliations per line that
force aggregation before the join. Issue log and weekly todo carry the open
decision for Andreas, and the RAG summary carries the warning, since a stale
line there starts the next session wrong.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -1318,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2937,6 +2937,55 @@
         </is>
       </c>
       <c r="K32" s="38" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C33" s="38" t="inlineStr">
+        <is>
+          <t>Finance Journal</t>
+        </is>
+      </c>
+      <c r="D33" s="38" t="inlineStr">
+        <is>
+          <t>ISS-006.1</t>
+        </is>
+      </c>
+      <c r="E33" s="38" t="inlineStr">
+        <is>
+          <t>Ausgleichsfelder eingebaut, Bedeutung von date paid entscheiden</t>
+        </is>
+      </c>
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>Andreas / Ingo</t>
+        </is>
+      </c>
+      <c r="G33" s="38" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H33" s="50" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I33" s="38" t="inlineStr"/>
+      <c r="J33" s="38" t="inlineStr">
+        <is>
+          <t>Andreas entscheiden lassen: Zahlungsbuchungsdatum, Ueberweisungsdatum, letzter Ausgleich oder erst vollstaendiger Ausgleich; Felder sind seit 09.09.2026 in Journal und Finance_All vorhanden, aber noch nicht deployed</t>
+        </is>
+      </c>
+      <c r="K33" s="38" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K32">

</xml_diff>

<commit_message>
Bring the project status back in line with what the docs already recorded
PM-08 still said "two blockers, both proven" from 2026-08-27, while the
first one had been solved on 2026-09-09: Rohail's invoice file carried the
business address number, and the production backfill lifted the German
sales rows from 4'549 to 7'592 of 7'622. The deadline passed with nothing
sent, so that is stated rather than quietly re-dated.

PM-04 gains the purchasing snapshot and the label deploy, including the
three status labels that were never committed and so never shipped. PM-05
gains the clearing fields that went live on 2026-09-10. PM-07 is left
alone because HR genuinely has nothing new.

Three new weekly rows: the unshipped labels, the industry-to-segment
decision that no code can make, and two defects in the German customer
master. The summary sheet is pulled along so the workbook does not argue
with itself.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -1093,12 +1093,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>SAP-Direktanbindung produktiv seit 12.08.2026, Materialtext MAKTX seit 18.08.2026.</t>
+          <t>SAP-Direktanbindung produktiv seit 12.08.2026, Materialtext MAKTX seit 18.08.2026. Seit 03.09.2026 teilen alle 15 Routen einen filterabhaengigen Snapshot, warme Aufrufe statt 9-11 s jetzt 0,05-0,14 s. Am 10.09.2026 verstaendlichere Kennzahlen und SAP-Quellenhilfe produktiv, dabei blieben drei Statusbeschriftungen uncommittet und damit unausgeliefert.</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren.</t>
+          <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren, die drei Statusbeschriftungen nachziehen und die neuen Texte produktiv sichtpruefen.</t>
         </is>
       </c>
     </row>
@@ -1119,16 +1119,16 @@
         </is>
       </c>
       <c r="D6" s="37" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Produktiv; Detailarbeit laeuft im Finance-Issue-Log. ISS-003.4 ist als Option produktiv, Andreas entscheidet die Ausnahme.</t>
+          <t>Produktiv; Detailarbeit laeuft im Finance-Issue-Log. Die fuenf Ausgleichsfelder sind seit 10.09.2026 08:53 produktiv (Journal von 29 auf 34 Spalten), Finance_All am selben Tag mit 470’499 Zeilen neu erzeugt. TR-IT-Bewertungsmethode am 09.09.2026 entschieden und zurueckgestellt.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Ueber das Finance-Issue-Log weiterfuehren; CH/AT-Option mit Andreas entscheiden.</t>
+          <t>Ueber das Finance-Issue-Log weiterfuehren; CH/AT-Option und die Bedeutung von date paid mit Andreas entscheiden.</t>
         </is>
       </c>
     </row>
@@ -1239,16 +1239,16 @@
         </is>
       </c>
       <c r="D10" s="37" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Spaltenzuordnung und Nachtrag Januar-Mai sind erledigt; Tagesprozess extern offen.</t>
+          <t>Erledigt. Entscheid vom 02.09.2026: die 7-Tage-Version bleibt im Einsatz, Finance verwendet fuer Spanien InvoiceDate. Kein Wechsel auf die 35-Tage-Version.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Wartet auf serverseitigen Tausch der Sage-Exportversion (7 auf 35 Tage).</t>
+          <t>Keiner.</t>
         </is>
       </c>
     </row>
@@ -1268,14 +1268,17 @@
           <t>Hoch</t>
         </is>
       </c>
+      <c r="D11" t="n">
+        <v>0.8</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4'549 Zeilen direkt belegt; historische Kandidaten und Restliste offen.</t>
+          <t>Blocker 1 am 09.09.2026 geloest: Rohails Rechnungsdatei lieferte die fachliche Adressnummer, produktiver Nachzug um 14:37 auf 7’592 von 7’622 Zeilen und 24 bestaetigte Segmente. Deutscher Bahnumsatz erstmals belegbar. Termin 08.09.2026 ueberschritten, nichts versendet.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aktuellen internen/fachlichen Adressschluessel abgleichen, Rohail-Datei und Dashboard nachpruefen.</t>
+          <t>Neues Zieldatum mit Rohail vereinbaren; 30 Gutschriftenzeilen und drei Doppelnummern klaeren; Patrik die 171 uebrigen Vorschlaege pruefen lassen.</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2178,7 +2181,7 @@
       <c r="I17" s="38" t="inlineStr"/>
       <c r="J17" s="38" t="inlineStr">
         <is>
-          <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren</t>
+          <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren. Am 11.09.2026 gegen docs/rag/PURCHASING.md geprueft: beide Punkte stehen unveraendert offen, ohne Betriebsauswirkung. Das Dashboard selbst ist seit 03.09.2026 durch den Filter-Snapshot beschleunigt (Commits 756e931, 2444731).</t>
         </is>
       </c>
       <c r="K17" s="38" t="n"/>
@@ -2578,7 +2581,7 @@
       </c>
       <c r="J25" s="38" t="inlineStr">
         <is>
-          <t>09.09.: Belegbruecke produktiv (687 Tests). 4'549 von 7'615 DE-Zeilen direkt belegt nachgezogen. 2'427 historische Kandidaten bleiben ungeprueft; 639 Zeilen ohne eindeutigen Treffer (darunter 15 Konfliktzeilen). Aktueller Alphaplan-ID/AdressNr-Abgleich bleibt erforderlich. Details: docs/BAHNMARKT_DE_ANBINDUNG_2026-09-08.md</t>
+          <t>Ueberholt den Stand vom 09.09. 07:20. Rohail Munirs Rechnungen_20260909.xlsx loeste den Schluessel: 60'539 Rechnungen mit fachlicher Adressnr._R, die interne RechnungsAdressenID wird nicht mehr gebraucht. Produktiver Nachzug am 09.09.2026 um 14:37, 3'043 Zeilen in einer Transaktion, fachliche Nummern von 4'549 auf 7'592 von 7'622, Segmente von 19 auf 24, quick_check ok, SalesPriceValue unveraendert. Deutscher Bahnumsatz erstmals belegbar: 2025 rund 578'636 EUR, 2026 bis 09.09. rund 432'237 EUR. OFFEN: 30 Gutschriftenzeilen ohne fachliche Nummer, weil Rohails Datei keine Gutschriften enthaelt, und die 40 Zeilen der drei Doppelnummern Sonepar, EMS und Magnetic Sense. Der Termin 08.09.2026 ist ueberschritten, neues Zieldatum offen.</t>
         </is>
       </c>
       <c r="K25" s="38" t="n"/>
@@ -2631,7 +2634,7 @@
       </c>
       <c r="J26" s="38" t="inlineStr">
         <is>
-          <t>171 offene Vorschlaege der anderen Standorte bleiben fachlich zu pruefen. Rohails DE-Stamm bestaetigt keine auslaendischen Kundenschluessel. DE nur direkte Belegzuordnung und reine Bahnbranche automatisch bestaetigen.</t>
+          <t>171 offene Vorschlaege der anderen Standorte bleiben fachlich zu pruefen. Rohails DE-Stamm bestaetigt keine auslaendischen Kundenschluessel. DE nur direkte Belegzuordnung und reine Bahnbranche automatisch bestaetigen. Am 10.09.2026 produktiv nachgemessen und unveraendert: von 196 Zuordnungen sind 25 bestaetigt, davon 24 aus TRDE; die 171 uebrigen bleiben Namensabgleich-Vorschlaege.</t>
         </is>
       </c>
       <c r="K26" s="38" t="n"/>
@@ -2982,10 +2985,157 @@
       <c r="I33" s="38" t="inlineStr"/>
       <c r="J33" s="38" t="inlineStr">
         <is>
-          <t>Query am 09.09.2026 live gegengezaehlt, keine Zeilenvervielfachung. Jetzt Andreas entscheiden lassen: Zahlungsbuchungsdatum, Ueberweisungsdatum, letzter Ausgleich oder erst vollstaendiger Ausgleich; Felder sind seit 09.09.2026 in Journal und Finance_All vorhanden, aber noch nicht deployed</t>
+          <t>Query am 09.09.2026 live gegengezaehlt, keine Zeilenvervielfachung. Die fuenf Felder sind seit dem Deploy vom 10.09.2026 um 08:53 PRODUKTIV, die Schemamigration hat das Journal von 29 auf 34 Spalten erweitert, 691/691 Tests gruen. Finance_All ist am selben Tag neu erzeugt worden, due date darin vollstaendig belegt. OFFEN ist nur noch der fachliche Entscheid von Andreas, was date paid bedeuten soll: Zahlungsbuchungsdatum, Ueberweisungsdatum, letzter Ausgleich oder erst vollstaendiger Ausgleich.</t>
         </is>
       </c>
       <c r="K33" s="38" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C34" s="38" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D34" s="38" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E34" s="38" t="inlineStr">
+        <is>
+          <t>Einkauf-Beschriftungen: drei Statustexte nicht ausgeliefert</t>
+        </is>
+      </c>
+      <c r="F34" s="38" t="inlineStr">
+        <is>
+          <t>Codex / Ingo</t>
+        </is>
+      </c>
+      <c r="G34" s="38" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H34" s="50" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I34" s="38" t="inlineStr"/>
+      <c r="J34" s="38" t="inlineStr">
+        <is>
+          <t>Beim Deploy vom 10.09.2026 um 09:40 wurde Commit d5bc321 ausgeliefert. Die zuletzt geaenderten drei Statusbeschriftungen waren NICHT committet und sind damit nicht produktiv: "Gebuchter Spend" statt "Bestellwert im Zeitraum" und "Einteilungen" statt "Einteilungen im Zeitraum". Der alte Text steht weiter an vier Stellen in PurchasingDashboard.razor und sechs in PurchasingUiTextCatalog.cs. Nachziehen und ausliefern. Ausserdem steht die produktive Sichtpruefung der neuen Kacheln und der Quellenhilfe noch aus.</t>
+        </is>
+      </c>
+      <c r="K34" s="38" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C35" s="38" t="inlineStr">
+        <is>
+          <t>Marktsegmente</t>
+        </is>
+      </c>
+      <c r="D35" s="38" t="inlineStr">
+        <is>
+          <t>ISS-014</t>
+        </is>
+      </c>
+      <c r="E35" s="38" t="inlineStr">
+        <is>
+          <t>Branche auf Segment abbilden, rund 38 Werte</t>
+        </is>
+      </c>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>Vertrieb / Andreas</t>
+        </is>
+      </c>
+      <c r="G35" s="38" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H35" s="50" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I35" s="38" t="inlineStr"/>
+      <c r="J35" s="38" t="inlineStr">
+        <is>
+          <t>Am 10.09.2026 produktiv gemessen: die Segmentzuweisung laeuft fuer Deutschland automatisch, fuer die anderen acht Standorte nicht, weil dort das Branchenfeld im Quellsystem fehlt. ZSCHWEIZ ist mit 52'276 Zeilen der groesste Standort ohne jede Branche. Die 543 deutschen Kunden verteilen sich auf 38 Branchenwerte und decken 97,9 Prozent des DE-Umsatzes ab; genutzt werden bisher nur die 24 mit "00 Bahn", und in CustomerMarketSegments existiert ueberhaupt nur der Segmentwert Railway. Der naechste Schritt ist kein Code, sondern ein fachlicher Entscheid ueber rund 38 Zeilen. Details: docs/MARKTSEGMENTE_RAILWAY_2026-08-13.md Abschnitt 18.</t>
+        </is>
+      </c>
+      <c r="K35" s="38" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C36" s="38" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="D36" s="38" t="inlineStr">
+        <is>
+          <t>ISS-014.1</t>
+        </is>
+      </c>
+      <c r="E36" s="38" t="inlineStr">
+        <is>
+          <t>Zwei Datenmaengel im deutschen Kundenstamm</t>
+        </is>
+      </c>
+      <c r="F36" s="38" t="inlineStr">
+        <is>
+          <t>Rohail / Ingo</t>
+        </is>
+      </c>
+      <c r="G36" s="38" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H36" s="50" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I36" s="38" t="inlineStr"/>
+      <c r="J36" s="38" t="inlineStr">
+        <is>
+          <t>Am 10.09.2026 beim Branchenabgleich gefunden: Kundennummer 52 traegt zwei verschiedene Bezeichnungen, und zwei Branchenwerte enden auf ein Komma. Zusammen neun Kunden betroffen. Mit Rohail klaeren.</t>
+        </is>
+      </c>
+      <c r="K36" s="38" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K32">

</xml_diff>

<commit_message>
Record the export dashboard and SQLite cache changes
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -744,7 +744,7 @@
     <x:t>Tempo der Webapp (größter Kritikpunkt)</x:t>
   </x:si>
   <x:si>
-    <x:t>Erledigt am 28.09.: Oberfläche erscheint sofort (4f2c62f), Einkauf-Standardansicht vorgewärmt (d32a6aa), Management-Cockpit lokal 41 s -&gt; 3,7 s (5a26596, Deploy nach dem Mittagslauf). Offen: Export-Dashboard (lokal 2-3 s), Server rechnet rund achtmal langsamer als der Entwicklungsrechner. Details docs/PLATTFORM_TEMPO_2026-09-28.md.</x:t>
+    <x:t>Erledigt am 28.09.: Oberfläche erscheint sofort (4f2c62f), Einkauf-Standardansicht vorgewärmt (d32a6aa), Management-Cockpit lokal 41 s -&gt; 3,3 s (5a26596), Export-Dashboard 2,3 s -&gt; 0,07 s und SQLite-Cache (c35d3fa), Deploy um 13:31 nach dem Einkauf-Delta. Offen: ob der SQLite-Cache die achtfache Serverlangsamkeit behebt (Vorwärmzeit im Log, Vergleich 104,7 s). Details docs/PLATTFORM_TEMPO_2026-09-28.md.</x:t>
   </x:si>
   <x:si>
     <x:t>38</x:t>
@@ -2322,7 +2322,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7fe1e117-c917-4a67-b1c8-383b9c147275}</x14:id>
+          <x14:id>{0d07a64c-8cdd-48d2-849c-5156dfd7c961}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -2336,7 +2336,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7fe1e117-c917-4a67-b1c8-383b9c147275}">
+          <x14:cfRule type="dataBar" id="{0d07a64c-8cdd-48d2-849c-5156dfd7c961}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
Record the 13:32 deploy: the server now computes the purchasing view in 24 s instead of 100 s
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -744,7 +744,7 @@
     <x:t>Tempo der Webapp (größter Kritikpunkt)</x:t>
   </x:si>
   <x:si>
-    <x:t>Erledigt am 28.09.: Oberfläche erscheint sofort (4f2c62f), Einkauf-Standardansicht vorgewärmt (d32a6aa), Management-Cockpit lokal 41 s -&gt; 3,3 s (5a26596), Export-Dashboard 2,3 s -&gt; 0,07 s und SQLite-Cache (c35d3fa), Deploy um 13:31 nach dem Einkauf-Delta. Offen: ob der SQLite-Cache die achtfache Serverlangsamkeit behebt (Vorwärmzeit im Log, Vergleich 104,7 s). Details docs/PLATTFORM_TEMPO_2026-09-28.md.</x:t>
+    <x:t>Erledigt am 28.09.: Oberfläche erscheint sofort (4f2c62f), Einkauf-Standardansicht vorgewärmt (d32a6aa), Management-Cockpit lokal 41 s -&gt; 3,3 s (5a26596), Export-Dashboard 2,3 s -&gt; 0,07 s und SQLite-Cache (c35d3fa), Alles produktiv seit 28.09. 13:32; Server-Einkaufsberechnung 104,7 s -&gt; 24,4 s durch den SQLite-Cache. Offen: Finanzvergleich ohne CSV-Cache (2,4 s lokal), Rest-Faktor 2 der VM. Details docs/PLATTFORM_TEMPO_2026-09-28.md.</x:t>
   </x:si>
   <x:si>
     <x:t>38</x:t>
@@ -2322,7 +2322,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0d07a64c-8cdd-48d2-849c-5156dfd7c961}</x14:id>
+          <x14:id>{9d7aabf7-abd6-47f6-b4a8-87e7181e5bdc}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -2336,7 +2336,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0d07a64c-8cdd-48d2-849c-5156dfd7c961}">
+          <x14:cfRule type="dataBar" id="{9d7aabf7-abd6-47f6-b4a8-87e7181e5bdc}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
Bring project status, summaries and indexes up to date for 28.09.
Project status gains PM-09 (webapp speed and a reliable nightly run) and
the 28.09. state of PM-04 (stock value trend) and PM-07 (HR answers).
ISS-017 records the proof that the code workaround holds, the weekly todo
the mail draft to Sonja, and baum.md the new tempo document. Two stale
"not deployed" statements are marked as superseded.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -771,7 +771,7 @@
     <x:t>nächster Call</x:t>
   </x:si>
   <x:si>
-    <x:t>Rexx-Absenzdatei hat pro Person nur Summen, periodengenau nur mit auf den Zeitraum eingegrenztem Export. Dateien auf dem Server sind vom 08.07. (Rexx) und 26.05. (SAP), neue Exporte anfordern.</x:t>
+    <x:t>Mail-Entwurf an Sonja mit dem Umsetzungsstand liegt vor (28.09.), Versand durch Ingo. Rexx-Absenzdatei hat pro Person nur Summen, periodengenau nur mit auf den Zeitraum eingegrenztem Export. Dateien auf dem Server sind vom 08.07. (Rexx) und 26.05. (SAP), neue Exporte anfordern.</x:t>
   </x:si>
   <x:si>
     <x:t>Hinweis</x:t>
@@ -2322,7 +2322,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9d7aabf7-abd6-47f6-b4a8-87e7181e5bdc}</x14:id>
+          <x14:id>{2496d04f-dbcb-41d1-9fe1-66264e75deac}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -2336,7 +2336,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9d7aabf7-abd6-47f6-b4a8-87e7181e5bdc}">
+          <x14:cfRule type="dataBar" id="{2496d04f-dbcb-41d1-9fe1-66264e75deac}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
Add a HERMES view for management to the weekly todo workbook
New Vorhaben_HERMES.tsv lists the nine work packages with tier, sponsor,
user representative, the three decision points (release, acceptance,
closure) and a traffic light. Wochen_Todo gains Vorhaben and HERMES-Stufe
columns. The generator now writes a first sheet "HERMES Übersicht" with
tiles, status symbols, data bars, a pie and a bar chart, plus one-page
templates for the project order and the acceptance record. Roles marked
"Vorschlag" are derived from the docs and not yet confirmed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -6,16 +6,21 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Zusammenfassung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wochen-Todo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legende" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Erläuterungen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="HERMES Übersicht" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Zusammenfassung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wochen-Todo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Legende" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Erläuterungen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vorlage Projektauftrag" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Vorlage Abnahmeprotokoll" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Wochen-Todo'!$A$1:$K$40</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Wochen-Todo'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Wochen-Todo'!$A$1:$K$40</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Erläuterungen'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$43</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="125725" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=""/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="47">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -210,8 +215,147 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E8B57"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C9A100"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C9A100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="007F7F7F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E8B57"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E8B57"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -323,8 +467,73 @@
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E8B57"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left>
         <color rgb="FF000000"/>
@@ -376,11 +585,120 @@
         <color rgb="FF000000"/>
       </diagonal>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="002F5597"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="002E8B57"/>
+      </bottom>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom>
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom>
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <top>
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left>
+        <color rgb="FF000000"/>
+      </left>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="136">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -598,6 +916,175 @@
     <xf numFmtId="164" fontId="8" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="25" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="30" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="31" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="29" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="34" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="28" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="25" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="32" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="28" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -680,6 +1167,249 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ampel der Vorhaben</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'HERMES Übersicht'!Q7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E8B57"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="C9A100"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'HERMES Übersicht'!$P$8:$P$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'HERMES Übersicht'!$Q$8:$Q$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="0"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Offene Aufgaben je Vorhaben</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'HERMES Übersicht'!J7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="5B9BD5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'HERMES Übersicht'!$A$8:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'HERMES Übersicht'!$J$8:$J$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3600000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -987,6 +1717,983 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F3864"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Q29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="48" min="1" max="1"/>
+    <col width="36" customWidth="1" style="48" min="2" max="2"/>
+    <col width="13" customWidth="1" style="48" min="3" max="3"/>
+    <col width="11" customWidth="1" style="48" min="4" max="4"/>
+    <col width="22" customWidth="1" style="48" min="5" max="5"/>
+    <col width="26" customWidth="1" style="48" min="6" max="6"/>
+    <col width="13" customWidth="1" style="48" min="7" max="7"/>
+    <col width="15" customWidth="1" style="48" min="8" max="8"/>
+    <col width="13" customWidth="1" style="48" min="9" max="9"/>
+    <col width="10" customWidth="1" style="48" min="10" max="10"/>
+    <col width="46" customWidth="1" style="48" min="11" max="11"/>
+    <col width="38" customWidth="1" style="48" min="12" max="12"/>
+    <col width="42" customWidth="1" style="48" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" style="48" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" style="48" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1" s="48">
+      <c r="A1" s="73" t="inlineStr">
+        <is>
+          <t>Vorhaben nach HERMES  ·  Übersicht für die Geschäftsleitung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="48">
+      <c r="A2" s="74" t="inlineStr">
+        <is>
+          <t>Stand 29.09.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="48">
+      <c r="A4" s="75" t="inlineStr">
+        <is>
+          <t>VORHABEN</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="n"/>
+      <c r="C4" s="77" t="inlineStr">
+        <is>
+          <t>● IM PLAN</t>
+        </is>
+      </c>
+      <c r="D4" s="78" t="n"/>
+      <c r="E4" s="79" t="inlineStr">
+        <is>
+          <t>● ACHTUNG</t>
+        </is>
+      </c>
+      <c r="F4" s="80" t="n"/>
+      <c r="G4" s="81" t="inlineStr">
+        <is>
+          <t>● KRITISCH</t>
+        </is>
+      </c>
+      <c r="H4" s="82" t="n"/>
+      <c r="I4" s="83" t="inlineStr">
+        <is>
+          <t>FREIGABE FEHLT</t>
+        </is>
+      </c>
+      <c r="J4" s="84" t="n"/>
+      <c r="K4" s="83" t="inlineStr">
+        <is>
+          <t>ROLLE OFFEN</t>
+        </is>
+      </c>
+      <c r="L4" s="84" t="n"/>
+    </row>
+    <row r="5" ht="38" customHeight="1" s="48">
+      <c r="A5" s="85" t="n">
+        <v>9</v>
+      </c>
+      <c r="B5" s="76" t="n"/>
+      <c r="C5" s="86" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="78" t="n"/>
+      <c r="E5" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="80" t="n"/>
+      <c r="G5" s="88" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="82" t="n"/>
+      <c r="I5" s="89" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" s="84" t="n"/>
+      <c r="K5" s="90" t="n">
+        <v>10</v>
+      </c>
+      <c r="L5" s="84" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="48">
+      <c r="A7" s="91" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B7" s="91" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="C7" s="91" t="inlineStr">
+        <is>
+          <t>HERMES-Stufe</t>
+        </is>
+      </c>
+      <c r="D7" s="91" t="inlineStr">
+        <is>
+          <t>Ampel</t>
+        </is>
+      </c>
+      <c r="E7" s="91" t="inlineStr">
+        <is>
+          <t>Auftraggeber</t>
+        </is>
+      </c>
+      <c r="F7" s="91" t="inlineStr">
+        <is>
+          <t>Anwendervertreter</t>
+        </is>
+      </c>
+      <c r="G7" s="91" t="inlineStr">
+        <is>
+          <t>① Freigabe</t>
+        </is>
+      </c>
+      <c r="H7" s="91" t="inlineStr">
+        <is>
+          <t>② Abnahme</t>
+        </is>
+      </c>
+      <c r="I7" s="91" t="inlineStr">
+        <is>
+          <t>③ Abschluss</t>
+        </is>
+      </c>
+      <c r="J7" s="91" t="inlineStr">
+        <is>
+          <t>Offene Aufgaben</t>
+        </is>
+      </c>
+      <c r="K7" s="91" t="inlineStr">
+        <is>
+          <t>Stand in einem Satz</t>
+        </is>
+      </c>
+      <c r="L7" s="91" t="inlineStr">
+        <is>
+          <t>Nächster Entscheid</t>
+        </is>
+      </c>
+      <c r="M7" s="91" t="inlineStr">
+        <is>
+          <t>Erledigt, wenn</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Ampel</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" s="48">
+      <c r="A8" s="92" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="B8" s="93" t="inlineStr">
+        <is>
+          <t>ZLO03: Auswertung auslaufender Materialien korrigieren</t>
+        </is>
+      </c>
+      <c r="C8" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="inlineStr">
+        <is>
+          <t>●  Gelb</t>
+        </is>
+      </c>
+      <c r="E8" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F8" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen (Vorschlag: Ann-Katrin Michel)</t>
+        </is>
+      </c>
+      <c r="G8" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H8" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I8" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J8" s="98" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="99" t="inlineStr">
+        <is>
+          <t>Die Korrektur ist fertig; Test und Übernahme ins Produktivsystem stehen seit dem 14.08.2026 aus.</t>
+        </is>
+      </c>
+      <c r="L8" s="99" t="inlineStr">
+        <is>
+          <t>Anwendervertreter und Abnahmekriterien nachträglich festlegen, dann testen und abnehmen.</t>
+        </is>
+      </c>
+      <c r="M8" s="99" t="inlineStr">
+        <is>
+          <t>Mengen und Materialliste stimmen im Produktivsystem mit einer vereinbarten Stichprobe überein.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Grün</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" s="48">
+      <c r="A9" s="100" t="inlineStr">
+        <is>
+          <t>PM-02</t>
+        </is>
+      </c>
+      <c r="B9" s="101" t="inlineStr">
+        <is>
+          <t>ZC12: Fehler bei Nullmengen</t>
+        </is>
+      </c>
+      <c r="C9" s="102" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+      <c r="D9" s="103" t="inlineStr">
+        <is>
+          <t>●  Rot</t>
+        </is>
+      </c>
+      <c r="E9" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F9" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="G9" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="H9" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="I9" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="J9" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="107" t="inlineStr">
+        <is>
+          <t>Die Ursache ist eingegrenzt und eine korrigierte Fassung vorbereitet, aber noch nicht im System.</t>
+        </is>
+      </c>
+      <c r="L9" s="107" t="inlineStr">
+        <is>
+          <t>Korrigierte Fassung einspielen und den Fall nachtesten.</t>
+        </is>
+      </c>
+      <c r="M9" s="107" t="inlineStr">
+        <is>
+          <t>Nullmengen werden korrekt angezeigt.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Gelb</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="48">
+      <c r="A10" s="92" t="inlineStr">
+        <is>
+          <t>PM-03</t>
+        </is>
+      </c>
+      <c r="B10" s="93" t="inlineStr">
+        <is>
+          <t>ZZPRDAT: Produktionsdatum am Fertigungsauftrag</t>
+        </is>
+      </c>
+      <c r="C10" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D10" s="95" t="inlineStr">
+        <is>
+          <t>●  Gelb</t>
+        </is>
+      </c>
+      <c r="E10" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F10" s="108" t="inlineStr">
+        <is>
+          <t>Vorschlag: Lucas Castro, Florian Waechter</t>
+        </is>
+      </c>
+      <c r="G10" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H10" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I10" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J10" s="98" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="99" t="inlineStr">
+        <is>
+          <t>Die Lösung ist gebaut und im Testsystem vollständig geprüft; die Abnahmeanfrage ist vorbereitet, aber noch nicht versendet.</t>
+        </is>
+      </c>
+      <c r="L10" s="99" t="inlineStr">
+        <is>
+          <t>Abnahmeanfrage versenden.</t>
+        </is>
+      </c>
+      <c r="M10" s="99" t="inlineStr">
+        <is>
+          <t>Die Abnahme liegt schriftlich vor, Etikett und Typenschild sind geprüft.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Rot</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="48">
+      <c r="A11" s="100" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="B11" s="101" t="inlineStr">
+        <is>
+          <t>Einkaufs-Dashboard mit Drilldown und Lagerwert</t>
+        </is>
+      </c>
+      <c r="C11" s="109" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+      <c r="D11" s="110" t="inlineStr">
+        <is>
+          <t>●  Grün</t>
+        </is>
+      </c>
+      <c r="E11" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F11" s="111" t="inlineStr">
+        <is>
+          <t>Vorschlag: Einkauf (Marco, Armin)</t>
+        </is>
+      </c>
+      <c r="G11" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H11" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I11" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J11" s="106" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="107" t="inlineStr">
+        <is>
+          <t>Produktiv; zwei Nacharbeiten im SAP und drei Beschriftungen sind offen.</t>
+        </is>
+      </c>
+      <c r="L11" s="107" t="inlineStr">
+        <is>
+          <t>Nacharbeiten im SAP anstossen.</t>
+        </is>
+      </c>
+      <c r="M11" s="107" t="inlineStr">
+        <is>
+          <t>Der Einkauf nutzt das Dashboard ohne Rückfragen, der Lagerwert ist gegen SAP abgestimmt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" s="48">
+      <c r="A12" s="92" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="B12" s="93" t="inlineStr">
+        <is>
+          <t>Finance: Gruppenreporting Umsatz und Marge</t>
+        </is>
+      </c>
+      <c r="C12" s="109" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+      <c r="D12" s="95" t="inlineStr">
+        <is>
+          <t>●  Gelb</t>
+        </is>
+      </c>
+      <c r="E12" s="108" t="inlineStr">
+        <is>
+          <t>Vorschlag: Andreas Stoller</t>
+        </is>
+      </c>
+      <c r="F12" s="108" t="inlineStr">
+        <is>
+          <t>Vorschlag: Andreas Stoller</t>
+        </is>
+      </c>
+      <c r="G12" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H12" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I12" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J12" s="98" t="n">
+        <v>15</v>
+      </c>
+      <c r="K12" s="99" t="inlineStr">
+        <is>
+          <t>Produktiv; mehrere Fachentscheide zu Marge, Umsatzbegriff und Kostenregeln sind offen.</t>
+        </is>
+      </c>
+      <c r="L12" s="99" t="inlineStr">
+        <is>
+          <t>Offene Fachentscheide mit Andreas Stoller abschliessen.</t>
+        </is>
+      </c>
+      <c r="M12" s="99" t="inlineStr">
+        <is>
+          <t>Andreas Stoller gibt Gruppenmarge und Umsatzdefinition schriftlich frei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" s="48">
+      <c r="A13" s="100" t="inlineStr">
+        <is>
+          <t>PM-06</t>
+        </is>
+      </c>
+      <c r="B13" s="101" t="inlineStr">
+        <is>
+          <t>PPWR: Stoffcompliance über SAP-Klassifizierung</t>
+        </is>
+      </c>
+      <c r="C13" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D13" s="110" t="inlineStr">
+        <is>
+          <t>●  Grün</t>
+        </is>
+      </c>
+      <c r="E13" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F13" s="111" t="inlineStr">
+        <is>
+          <t>Vorschlag: Adil</t>
+        </is>
+      </c>
+      <c r="G13" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H13" s="113" t="inlineStr">
+        <is>
+          <t>✔  20.08.2026</t>
+        </is>
+      </c>
+      <c r="I13" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J13" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="107" t="inlineStr">
+        <is>
+          <t>Pilotmaterialien sind zugeordnet und laut Ingo abgenommen; die Übernahme ins Produktivsystem folgt nach Plan.</t>
+        </is>
+      </c>
+      <c r="L13" s="107" t="inlineStr">
+        <is>
+          <t>Übergabe in den Betrieb dokumentieren.</t>
+        </is>
+      </c>
+      <c r="M13" s="107" t="inlineStr">
+        <is>
+          <t>Die Klassifizierung ist produktiv und dokumentiert übergeben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" s="48">
+      <c r="A14" s="92" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="B14" s="93" t="inlineStr">
+        <is>
+          <t>HR: automatische Auswertung der Personaldaten</t>
+        </is>
+      </c>
+      <c r="C14" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D14" s="95" t="inlineStr">
+        <is>
+          <t>●  Gelb</t>
+        </is>
+      </c>
+      <c r="E14" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F14" s="108" t="inlineStr">
+        <is>
+          <t>Vorschlag: Sonja Richter</t>
+        </is>
+      </c>
+      <c r="G14" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H14" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I14" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J14" s="98" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="99" t="inlineStr">
+        <is>
+          <t>Die fachlichen Wünsche sind umgesetzt; es fehlt die Exportschnittstelle der externen Firma.</t>
+        </is>
+      </c>
+      <c r="L14" s="99" t="inlineStr">
+        <is>
+          <t>Termin der externen Firma einfordern.</t>
+        </is>
+      </c>
+      <c r="M14" s="99" t="inlineStr">
+        <is>
+          <t>Die monatliche Auswertung läuft ohne Handarbeit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" s="48">
+      <c r="A15" s="100" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="B15" s="101" t="inlineStr">
+        <is>
+          <t>Bahnmarkt: Railway-Auswertung für Deutschland und die Standorte</t>
+        </is>
+      </c>
+      <c r="C15" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D15" s="103" t="inlineStr">
+        <is>
+          <t>●  Rot</t>
+        </is>
+      </c>
+      <c r="E15" s="111" t="inlineStr">
+        <is>
+          <t>Vorschlag: Rohail Munir</t>
+        </is>
+      </c>
+      <c r="F15" s="111" t="inlineStr">
+        <is>
+          <t>Vorschlag: Patrik</t>
+        </is>
+      </c>
+      <c r="G15" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H15" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I15" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J15" s="106" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="107" t="inlineStr">
+        <is>
+          <t>Der Termin vom 08.09.2026 ist überschritten; Deutschland ist gelöst, die übrigen Standorte sind offen.</t>
+        </is>
+      </c>
+      <c r="L15" s="107" t="inlineStr">
+        <is>
+          <t>Neues Zieldatum mit Rohail Munir vereinbaren.</t>
+        </is>
+      </c>
+      <c r="M15" s="107" t="inlineStr">
+        <is>
+          <t>Rohail Munir hat eine geprüfte Auswertung mit bestätigten Kundenzuordnungen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="48">
+      <c r="A16" s="92" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="B16" s="93" t="inlineStr">
+        <is>
+          <t>Plattform: Tempo der Webapp und stabiler Nachtlauf</t>
+        </is>
+      </c>
+      <c r="C16" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D16" s="110" t="inlineStr">
+        <is>
+          <t>●  Grün</t>
+        </is>
+      </c>
+      <c r="E16" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F16" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="G16" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H16" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I16" s="97" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J16" s="98" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="99" t="inlineStr">
+        <is>
+          <t>Weitgehend erledigt und produktiv; die Server-Einstellung durch die IT fehlt noch.</t>
+        </is>
+      </c>
+      <c r="L16" s="99" t="inlineStr">
+        <is>
+          <t>IT stellt den Dauerbetrieb des Servers ein.</t>
+        </is>
+      </c>
+      <c r="M16" s="99" t="inlineStr">
+        <is>
+          <t>Seiten laden in wenigen Sekunden, der Nachtlauf läuft täglich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="K18" s="114" t="inlineStr">
+        <is>
+          <t>So wird eingestuft (HERMES zugeschnitten)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="K19" s="115" t="inlineStr">
+        <is>
+          <t>Stufe</t>
+        </is>
+      </c>
+      <c r="L19" s="115" t="inlineStr">
+        <is>
+          <t>Aufwand</t>
+        </is>
+      </c>
+      <c r="M19" s="115" t="inlineStr">
+        <is>
+          <t>Vorgehen</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="K20" s="116" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+      <c r="L20" s="117" t="inlineStr">
+        <is>
+          <t>unter ca. 5 Personentage</t>
+        </is>
+      </c>
+      <c r="M20" s="117" t="inlineStr">
+        <is>
+          <t>Ticket, keine HERMES-Dokumente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="K21" s="118" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="L21" s="117" t="inlineStr">
+        <is>
+          <t>ca. 5 bis 40 Personentage</t>
+        </is>
+      </c>
+      <c r="M21" s="117" t="inlineStr">
+        <is>
+          <t>Auftrag, Abnahme, Statuszeile</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="K22" s="119" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+      <c r="L22" s="117" t="inlineStr">
+        <is>
+          <t>über ca. 40 Personentage</t>
+        </is>
+      </c>
+      <c r="M22" s="117" t="inlineStr">
+        <is>
+          <t>HERMES zugeschnitten, mit Risikoliste, eventuell Ausschuss</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1" s="48">
+      <c r="K24" s="120" t="inlineStr">
+        <is>
+          <t>① Freigabe</t>
+        </is>
+      </c>
+      <c r="L24" s="121" t="inlineStr">
+        <is>
+          <t>Der Auftraggeber hat den Projektauftrag unterschrieben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1" s="48">
+      <c r="K25" s="120" t="inlineStr">
+        <is>
+          <t>② Abnahme</t>
+        </is>
+      </c>
+      <c r="L25" s="121" t="inlineStr">
+        <is>
+          <t>Der Anwendervertreter bestätigt fachlich, das Ergebnis ist produktiv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1" s="48">
+      <c r="K26" s="120" t="inlineStr">
+        <is>
+          <t>③ Abschluss</t>
+        </is>
+      </c>
+      <c r="L26" s="121" t="inlineStr">
+        <is>
+          <t>Übergeben in den Betrieb, mit kurzer Betriebsdokumentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1" s="48">
+      <c r="K27" s="120" t="inlineStr">
+        <is>
+          <t>✔ / ○</t>
+        </is>
+      </c>
+      <c r="L27" s="121" t="inlineStr">
+        <is>
+          <t>Erledigt mit Datum / noch offen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1" s="48">
+      <c r="K28" s="120" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="L28" s="121" t="inlineStr">
+        <is>
+          <t>Die Rolle ist noch niemandem zugeordnet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1" s="48">
+      <c r="K29" s="120" t="inlineStr">
+        <is>
+          <t>● Ampel</t>
+        </is>
+      </c>
+      <c r="L29" s="121" t="inlineStr">
+        <is>
+          <t>Grün im Plan · Gelb wartet auf Entscheid oder Zulieferung · Rot blockiert oder Termin überschritten.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J8:J16">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1366,13 +3073,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -1386,6 +3093,8 @@
     <col width="12" customWidth="1" style="47" min="9" max="9"/>
     <col width="90" customWidth="1" style="47" min="10" max="10"/>
     <col width="13" customWidth="1" style="47" min="11" max="11"/>
+    <col width="10" customWidth="1" style="48" min="12" max="12"/>
+    <col width="14" customWidth="1" style="48" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="48">
@@ -1444,6 +3153,16 @@
           <t>Erledigt am</t>
         </is>
       </c>
+      <c r="L1" s="56" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="M1" s="56" t="inlineStr">
+        <is>
+          <t>HERMES-Stufe</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="57" t="inlineStr">
@@ -1497,6 +3216,16 @@
           <t>02.09.2026</t>
         </is>
       </c>
+      <c r="L2" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M2" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
@@ -1545,7 +3274,17 @@
           <t>Nachtrag und Import am 18.08.2026 bestätigt; keine Aktion</t>
         </is>
       </c>
-      <c r="K3" s="57" t="n"/>
+      <c r="K3" s="57" t="inlineStr"/>
+      <c r="L3" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M3" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="57" t="inlineStr">
@@ -1595,6 +3334,16 @@
         </is>
       </c>
       <c r="K4" s="57" t="inlineStr"/>
+      <c r="L4" s="57" t="inlineStr">
+        <is>
+          <t>PM-02</t>
+        </is>
+      </c>
+      <c r="M4" s="123" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="57" t="inlineStr">
@@ -1643,7 +3392,17 @@
           <t>Eskalieren, seit 30.07.2026 keine Faktura mehr (18 Tage)</t>
         </is>
       </c>
-      <c r="K5" s="57" t="n"/>
+      <c r="K5" s="57" t="inlineStr"/>
+      <c r="L5" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M5" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="57" t="inlineStr">
@@ -1692,7 +3451,17 @@
           <t>Produktiven Schalter in Settings vergleichen; Andreas entscheidet, ob Fremdbezug die Herstellerregel als Ausnahme bricht (Default bleibt bisherige Regel)</t>
         </is>
       </c>
-      <c r="K6" s="57" t="n"/>
+      <c r="K6" s="57" t="inlineStr"/>
+      <c r="L6" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M6" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
@@ -1741,7 +3510,17 @@
           <t>Termin mit Andreas, Punkt 2 von 3</t>
         </is>
       </c>
-      <c r="K7" s="57" t="n"/>
+      <c r="K7" s="57" t="inlineStr"/>
+      <c r="L7" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M7" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="57" t="inlineStr">
@@ -1790,7 +3569,17 @@
           <t>Termin mit Andreas, Punkt 3 von 3</t>
         </is>
       </c>
-      <c r="K8" s="57" t="n"/>
+      <c r="K8" s="57" t="inlineStr"/>
+      <c r="L8" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M8" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="57" t="inlineStr">
@@ -1839,7 +3628,17 @@
           <t>Entschieden am 27.08.2026: steht kein Lieferant, gelten die lokalen Standardkosten der verkaufenden Gesellschaft; keine Aufteilung je Land</t>
         </is>
       </c>
-      <c r="K9" s="57" t="n"/>
+      <c r="K9" s="57" t="inlineStr"/>
+      <c r="L9" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M9" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="57" t="inlineStr">
@@ -1888,7 +3687,17 @@
           <t>Diagnoselauf p_diag und Regressionstest, danach Transport nach B76</t>
         </is>
       </c>
-      <c r="K10" s="57" t="n"/>
+      <c r="K10" s="57" t="inlineStr"/>
+      <c r="L10" s="57" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="M10" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="57" t="inlineStr">
@@ -1937,7 +3746,17 @@
           <t>Ann-Katrin Michel vorwarnen: Spalte Exklusiv liefert künftig auch "?"</t>
         </is>
       </c>
-      <c r="K11" s="57" t="n"/>
+      <c r="K11" s="57" t="inlineStr"/>
+      <c r="L11" s="57" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="M11" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="57" t="inlineStr">
@@ -1991,6 +3810,16 @@
           <t>07.09.2026</t>
         </is>
       </c>
+      <c r="L12" s="57" t="inlineStr">
+        <is>
+          <t>PM-03</t>
+        </is>
+      </c>
+      <c r="M12" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="57" t="inlineStr">
@@ -2040,6 +3869,16 @@
         </is>
       </c>
       <c r="K13" s="57" t="inlineStr"/>
+      <c r="L13" s="57" t="inlineStr">
+        <is>
+          <t>PM-03</t>
+        </is>
+      </c>
+      <c r="M13" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="57" t="inlineStr">
@@ -2088,7 +3927,17 @@
           <t>Zuerst eigene Export-SQL prüfen, erst danach den Standort fragen. Präzedenzfall UK, belegt am 02.09.2026: die Lieferantenspalten waren in der UK-Datei seit jeher gefüllt (1881/1881) und nur nie gemappt</t>
         </is>
       </c>
-      <c r="K14" s="57" t="n"/>
+      <c r="K14" s="57" t="inlineStr"/>
+      <c r="L14" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M14" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="57" t="inlineStr">
@@ -2137,7 +3986,17 @@
           <t>Produktiv seit 27.08.2026 15:28. Beim nächsten Export die Indien-Quote im Excel gegen die App gegenprüfen</t>
         </is>
       </c>
-      <c r="K15" s="57" t="n"/>
+      <c r="K15" s="57" t="inlineStr"/>
+      <c r="L15" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M15" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="57" t="inlineStr">
@@ -2186,7 +4045,17 @@
           <t>FinanzJournalSet auf T76/100 am 11.09.2026 gebaut, aktiviert und geprueft ($metadata und Datenabruf HTTP 200, Werte gegengelesen, bestehende Sets unveraendert). Produktiv erst nach Freigabe und Import des Transports nach P76 wirksam.</t>
         </is>
       </c>
-      <c r="K16" s="57" t="n"/>
+      <c r="K16" s="57" t="inlineStr"/>
+      <c r="L16" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M16" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="57" t="inlineStr">
@@ -2235,7 +4104,17 @@
           <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren. Am 11.09.2026 gegen docs/rag/PURCHASING.md geprueft: beide Punkte stehen unveraendert offen, ohne Betriebsauswirkung. Das Dashboard selbst ist seit 03.09.2026 durch den Filter-Snapshot beschleunigt (Commits 756e931, 2444731).</t>
         </is>
       </c>
-      <c r="K17" s="57" t="n"/>
+      <c r="K17" s="57" t="inlineStr"/>
+      <c r="L17" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M17" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="57" t="inlineStr">
@@ -2284,7 +4163,17 @@
           <t>3 Deploys angemeldet sichtprüfen: Segmente, Umfrage, Jahresfilter</t>
         </is>
       </c>
-      <c r="K18" s="57" t="n"/>
+      <c r="K18" s="57" t="inlineStr"/>
+      <c r="L18" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M18" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="57" t="inlineStr">
@@ -2338,6 +4227,16 @@
           <t>27.08.2026</t>
         </is>
       </c>
+      <c r="L19" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M19" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="57" t="inlineStr">
@@ -2387,6 +4286,16 @@
         </is>
       </c>
       <c r="K20" s="57" t="inlineStr"/>
+      <c r="L20" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M20" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="57" t="inlineStr">
@@ -2435,7 +4344,17 @@
           <t>Komplett erledigt 2026-08-20 laut Ingo: Pilotmaterialien zugeordnet, CL30N-Abnahme gefahren</t>
         </is>
       </c>
-      <c r="K21" s="57" t="n"/>
+      <c r="K21" s="57" t="inlineStr"/>
+      <c r="L21" s="57" t="inlineStr">
+        <is>
+          <t>PM-06</t>
+        </is>
+      </c>
+      <c r="M21" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="57" t="inlineStr">
@@ -2484,7 +4403,17 @@
           <t>6 offene Entscheide bei Finance, nur beobachten</t>
         </is>
       </c>
-      <c r="K22" s="57" t="n"/>
+      <c r="K22" s="57" t="inlineStr"/>
+      <c r="L22" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M22" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="57" t="inlineStr">
@@ -2533,7 +4462,17 @@
           <t>Exporter-Fertigstellung abwarten, danach Anbindung/Auswertung planen</t>
         </is>
       </c>
-      <c r="K23" s="57" t="n"/>
+      <c r="K23" s="57" t="inlineStr"/>
+      <c r="L23" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M23" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="57" t="inlineStr">
@@ -2582,7 +4521,17 @@
           <t>Verlauf je Woche produktiv seit 28.09.2026 (Wunsch Einkauf, von Marco bestätigt). Einkauf-Lauf fiel 10.-28.09. aus (IIS-Leerlauf), per Code abgesichert, IT-Einstellung als ISS-017 offen. Danach Armins Entscheid zu Disponent 004, MB5L-Abgleich und serverseitigen Einkauf-Lauf als Kettennachweis ausführen</t>
         </is>
       </c>
-      <c r="K24" s="57" t="n"/>
+      <c r="K24" s="57" t="inlineStr"/>
+      <c r="L24" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M24" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="57" t="inlineStr">
@@ -2635,7 +4584,17 @@
           <t>Ueberholt den Stand vom 09.09. 07:20. Rohail Munirs Rechnungen_20260909.xlsx loeste den Schluessel: 60'539 Rechnungen mit fachlicher Adressnr._R, die interne RechnungsAdressenID wird nicht mehr gebraucht. Produktiver Nachzug am 09.09.2026 um 14:37, 3'043 Zeilen in einer Transaktion, fachliche Nummern von 4'549 auf 7'592 von 7'622, Segmente von 19 auf 24, quick_check ok, SalesPriceValue unveraendert. Deutscher Bahnumsatz erstmals belegbar: 2025 rund 578'636 EUR, 2026 bis 09.09. rund 432'237 EUR. OFFEN: 30 Gutschriftenzeilen ohne fachliche Nummer, weil Rohails Datei keine Gutschriften enthaelt, und die 40 Zeilen der drei Doppelnummern Sonepar, EMS und Magnetic Sense. Der Termin 08.09.2026 ist ueberschritten, neues Zieldatum offen.</t>
         </is>
       </c>
-      <c r="K25" s="57" t="n"/>
+      <c r="K25" s="57" t="inlineStr"/>
+      <c r="L25" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M25" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="57" t="inlineStr">
@@ -2688,7 +4647,17 @@
           <t>171 offene Vorschlaege der anderen Standorte bleiben fachlich zu pruefen. Rohails DE-Stamm bestaetigt keine auslaendischen Kundenschluessel. DE nur direkte Belegzuordnung und reine Bahnbranche automatisch bestaetigen. Am 10.09.2026 produktiv nachgemessen und unveraendert: von 196 Zuordnungen sind 25 bestaetigt, davon 24 aus TRDE; die 171 uebrigen bleiben Namensabgleich-Vorschlaege.</t>
         </is>
       </c>
-      <c r="K26" s="57" t="n"/>
+      <c r="K26" s="57" t="inlineStr"/>
+      <c r="L26" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M26" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="57" t="inlineStr">
@@ -2741,7 +4710,17 @@
           <t>09.09.: korrigierte DE-Pruefmappe mit Belegnachweisen, historischen Vorschlaegen und Restliste; Bahnmarkt_Rohail_2026-09-09.xlsx aus konsistentem Produktivsnapshot erzeugt und rueckgelesen (19 DE-Kunden bestaetigt). Kein Versand erfolgt.</t>
         </is>
       </c>
-      <c r="K27" s="57" t="n"/>
+      <c r="K27" s="57" t="inlineStr"/>
+      <c r="L27" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M27" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="57" t="inlineStr">
@@ -2795,6 +4774,16 @@
           <t>27.08.2026</t>
         </is>
       </c>
+      <c r="L28" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M28" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="57" t="inlineStr">
@@ -2843,7 +4832,17 @@
           <t>Sales Type in den oberen Block ziehen, Zweig ohne Lieferant und Währungszeile ergänzen, danach Sales_All neu generieren. Als Abgleich dient docs/FINANCE_LIEFERANT_STANDARDKOSTEN_WORKFLOW_2026-09-02.svg</t>
         </is>
       </c>
-      <c r="K29" s="57" t="n"/>
+      <c r="K29" s="57" t="inlineStr"/>
+      <c r="L29" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M29" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="57" t="inlineStr">
@@ -2892,7 +4891,17 @@
           <t>Am 02.09.2026 im Code gefunden: GroupDistributionWithoutGroupCost prüft nur den Sales Type LRD, nicht ob eine liefernde Konzerngesellschaft erkannt wurde. Zeilen mit Lieferant Trafag AG oder Trafag Italia ohne Konzernkostentreffer zeigen still eine Marge auf dem lokalen IC-Preis. Obergrenze 19'221 Zeilen (18,3 %). Zuerst die echte Menge gegen GroupStandardCosts in der Produktiv-DB messen, dann Andreas entscheiden lassen</t>
         </is>
       </c>
-      <c r="K30" s="57" t="n"/>
+      <c r="K30" s="57" t="inlineStr"/>
+      <c r="L30" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M30" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="57" t="inlineStr">
@@ -2941,7 +4950,17 @@
           <t>ShouldUseSwissStprs prüft den SupplierType nicht und setzt die liefernde Gesellschaft bedingungslos auf TR_AG. Im Alternativmodus bekämen auch Extern-, Lokal- und Unklar-Zeilen Schweizer Kosten. Klären, ob die Bedingung im Code fehlt oder die Beschriftung zu eng ist. Produktiv unbetroffen, Default DeliveringEntityCosts</t>
         </is>
       </c>
-      <c r="K31" s="57" t="n"/>
+      <c r="K31" s="57" t="inlineStr"/>
+      <c r="L31" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M31" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="57" t="inlineStr">
@@ -2990,7 +5009,17 @@
           <t>Alle 41 Konfliktzeilen gehen auf einen einzigen Lieferanten zurück. Indien prüfen lassen, ob diese Artikel wirklich Eigenfertigung sind oder der Sales Type falsch steht</t>
         </is>
       </c>
-      <c r="K32" s="57" t="n"/>
+      <c r="K32" s="57" t="inlineStr"/>
+      <c r="L32" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M32" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="57" t="inlineStr">
@@ -3040,6 +5069,16 @@
         </is>
       </c>
       <c r="K33" s="57" t="inlineStr"/>
+      <c r="L33" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M33" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="57" t="inlineStr">
@@ -3089,6 +5128,16 @@
         </is>
       </c>
       <c r="K34" s="57" t="inlineStr"/>
+      <c r="L34" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M34" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="57" t="inlineStr">
@@ -3138,6 +5187,16 @@
         </is>
       </c>
       <c r="K35" s="57" t="inlineStr"/>
+      <c r="L35" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M35" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="57" t="inlineStr">
@@ -3187,6 +5246,16 @@
         </is>
       </c>
       <c r="K36" s="57" t="inlineStr"/>
+      <c r="L36" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M36" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="57" t="inlineStr">
@@ -3236,6 +5305,16 @@
         </is>
       </c>
       <c r="K37" s="57" t="inlineStr"/>
+      <c r="L37" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M37" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="57" t="inlineStr">
@@ -3285,6 +5364,16 @@
         </is>
       </c>
       <c r="K38" s="57" t="inlineStr"/>
+      <c r="L38" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M38" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="57" t="inlineStr">
@@ -3338,6 +5427,16 @@
           <t>28.09.2026</t>
         </is>
       </c>
+      <c r="L39" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M39" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="57" t="inlineStr">
@@ -3391,6 +5490,16 @@
         </is>
       </c>
       <c r="K40" s="57" t="inlineStr"/>
+      <c r="L40" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M40" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="57" t="inlineStr">
@@ -3440,6 +5549,16 @@
         </is>
       </c>
       <c r="K41" s="57" t="inlineStr"/>
+      <c r="L41" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M41" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="57" t="inlineStr">
@@ -3489,6 +5608,16 @@
         </is>
       </c>
       <c r="K42" s="57" t="inlineStr"/>
+      <c r="L42" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M42" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="57" t="inlineStr">
@@ -3538,16 +5667,26 @@
         </is>
       </c>
       <c r="K43" s="57" t="inlineStr"/>
+      <c r="L43" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M43" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K40"/>
+  <autoFilter ref="A1:M43"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3711,7 +5850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5015,4 +7154,685 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="48" min="1" max="1"/>
+    <col width="22" customWidth="1" style="48" min="2" max="2"/>
+    <col width="22" customWidth="1" style="48" min="3" max="3"/>
+    <col width="22" customWidth="1" style="48" min="4" max="4"/>
+    <col width="22" customWidth="1" style="48" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" s="48">
+      <c r="A1" s="125" t="inlineStr">
+        <is>
+          <t>Projektauftrag  ·  eine Seite</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" s="48">
+      <c r="A2" s="126" t="inlineStr">
+        <is>
+          <t>Für Vorhaben und Projekte nach HERMES (ab ca. 5 Personentage). Mit der Unterschrift des Auftraggebers ist der Entscheidungspunkt ① Freigabe erreicht.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="127" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="B4" s="134" t="n"/>
+      <c r="C4" s="134" t="n"/>
+      <c r="D4" s="134" t="n"/>
+      <c r="E4" s="134" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="48">
+      <c r="A5" s="128" t="inlineStr">
+        <is>
+          <t>Bezeichnung und ID</t>
+        </is>
+      </c>
+      <c r="B5" s="129" t="n"/>
+      <c r="C5" s="130" t="n"/>
+      <c r="D5" s="130" t="n"/>
+      <c r="E5" s="130" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="48">
+      <c r="A6" s="128" t="inlineStr">
+        <is>
+          <t>HERMES-Stufe</t>
+        </is>
+      </c>
+      <c r="B6" s="129" t="n"/>
+      <c r="C6" s="130" t="n"/>
+      <c r="D6" s="130" t="n"/>
+      <c r="E6" s="130" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="48">
+      <c r="A7" s="128" t="inlineStr">
+        <is>
+          <t>Grober Aufwand (Personentage)</t>
+        </is>
+      </c>
+      <c r="B7" s="129" t="n"/>
+      <c r="C7" s="130" t="n"/>
+      <c r="D7" s="130" t="n"/>
+      <c r="E7" s="130" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="127" t="inlineStr">
+        <is>
+          <t>Inhalt</t>
+        </is>
+      </c>
+      <c r="B9" s="134" t="n"/>
+      <c r="C9" s="134" t="n"/>
+      <c r="D9" s="134" t="n"/>
+      <c r="E9" s="134" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1" s="48">
+      <c r="A10" s="128" t="inlineStr">
+        <is>
+          <t>Ausgangslage</t>
+        </is>
+      </c>
+      <c r="B10" s="129" t="n"/>
+      <c r="C10" s="130" t="n"/>
+      <c r="D10" s="130" t="n"/>
+      <c r="E10" s="130" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1" s="48">
+      <c r="A11" s="128" t="inlineStr">
+        <is>
+          <t>Ziel</t>
+        </is>
+      </c>
+      <c r="B11" s="129" t="n"/>
+      <c r="C11" s="130" t="n"/>
+      <c r="D11" s="130" t="n"/>
+      <c r="E11" s="130" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="48">
+      <c r="A12" s="128" t="inlineStr">
+        <is>
+          <t>Nutzen (ein Satz genügt)</t>
+        </is>
+      </c>
+      <c r="B12" s="129" t="n"/>
+      <c r="C12" s="130" t="n"/>
+      <c r="D12" s="130" t="n"/>
+      <c r="E12" s="130" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="48">
+      <c r="A13" s="128" t="inlineStr">
+        <is>
+          <t>Nicht im Umfang</t>
+        </is>
+      </c>
+      <c r="B13" s="129" t="n"/>
+      <c r="C13" s="130" t="n"/>
+      <c r="D13" s="130" t="n"/>
+      <c r="E13" s="130" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="127" t="inlineStr">
+        <is>
+          <t>Rollen</t>
+        </is>
+      </c>
+      <c r="B15" s="134" t="n"/>
+      <c r="C15" s="134" t="n"/>
+      <c r="D15" s="134" t="n"/>
+      <c r="E15" s="134" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="48">
+      <c r="A16" s="128" t="inlineStr">
+        <is>
+          <t>Auftraggeber (entscheidet, priorisiert)</t>
+        </is>
+      </c>
+      <c r="B16" s="129" t="n"/>
+      <c r="C16" s="130" t="n"/>
+      <c r="D16" s="130" t="n"/>
+      <c r="E16" s="130" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="48">
+      <c r="A17" s="128" t="inlineStr">
+        <is>
+          <t>Anwendervertreter (definiert fachlich, nimmt ab)</t>
+        </is>
+      </c>
+      <c r="B17" s="129" t="n"/>
+      <c r="C17" s="130" t="n"/>
+      <c r="D17" s="130" t="n"/>
+      <c r="E17" s="130" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="48">
+      <c r="A18" s="128" t="inlineStr">
+        <is>
+          <t>Projektleitung / Umsetzung</t>
+        </is>
+      </c>
+      <c r="B18" s="129" t="n"/>
+      <c r="C18" s="130" t="n"/>
+      <c r="D18" s="130" t="n"/>
+      <c r="E18" s="130" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="127" t="inlineStr">
+        <is>
+          <t>Abnahmekriterien: Das Vorhaben ist fertig, wenn …</t>
+        </is>
+      </c>
+      <c r="B20" s="134" t="n"/>
+      <c r="C20" s="134" t="n"/>
+      <c r="D20" s="134" t="n"/>
+      <c r="E20" s="134" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="131" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B21" s="131" t="inlineStr">
+        <is>
+          <t>Kriterium</t>
+        </is>
+      </c>
+      <c r="C21" s="131" t="inlineStr"/>
+      <c r="D21" s="131" t="inlineStr">
+        <is>
+          <t>Wie geprüft</t>
+        </is>
+      </c>
+      <c r="E21" s="131" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" s="48">
+      <c r="A22" s="130" t="n"/>
+      <c r="B22" s="130" t="n"/>
+      <c r="C22" s="130" t="n"/>
+      <c r="D22" s="130" t="n"/>
+      <c r="E22" s="130" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="48">
+      <c r="A23" s="130" t="n"/>
+      <c r="B23" s="130" t="n"/>
+      <c r="C23" s="130" t="n"/>
+      <c r="D23" s="130" t="n"/>
+      <c r="E23" s="130" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" s="48">
+      <c r="A24" s="130" t="n"/>
+      <c r="B24" s="130" t="n"/>
+      <c r="C24" s="130" t="n"/>
+      <c r="D24" s="130" t="n"/>
+      <c r="E24" s="130" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="48">
+      <c r="A25" s="130" t="n"/>
+      <c r="B25" s="130" t="n"/>
+      <c r="C25" s="130" t="n"/>
+      <c r="D25" s="130" t="n"/>
+      <c r="E25" s="130" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="127" t="inlineStr">
+        <is>
+          <t>Freigabe</t>
+        </is>
+      </c>
+      <c r="B27" s="134" t="n"/>
+      <c r="C27" s="134" t="n"/>
+      <c r="D27" s="134" t="n"/>
+      <c r="E27" s="134" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1" s="48">
+      <c r="A28" s="128" t="inlineStr">
+        <is>
+          <t>Termin Zielabnahme</t>
+        </is>
+      </c>
+      <c r="B28" s="129" t="n"/>
+      <c r="C28" s="130" t="n"/>
+      <c r="D28" s="130" t="n"/>
+      <c r="E28" s="130" t="n"/>
+    </row>
+    <row r="29" ht="34" customHeight="1" s="48">
+      <c r="A29" s="128" t="inlineStr">
+        <is>
+          <t>Datum, Unterschrift Auftraggeber</t>
+        </is>
+      </c>
+      <c r="B29" s="129" t="n"/>
+      <c r="C29" s="130" t="n"/>
+      <c r="D29" s="130" t="n"/>
+      <c r="E29" s="130" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="127" t="inlineStr">
+        <is>
+          <t>Änderungsanträge nach der Freigabe (gehen über den Auftraggeber)</t>
+        </is>
+      </c>
+      <c r="B31" s="134" t="n"/>
+      <c r="C31" s="134" t="n"/>
+      <c r="D31" s="134" t="n"/>
+      <c r="E31" s="134" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="131" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B32" s="131" t="inlineStr">
+        <is>
+          <t>Änderung</t>
+        </is>
+      </c>
+      <c r="C32" s="131" t="inlineStr">
+        <is>
+          <t>Aufwand</t>
+        </is>
+      </c>
+      <c r="D32" s="131" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="E32" s="131" t="inlineStr">
+        <is>
+          <t>Visum</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="48">
+      <c r="A33" s="130" t="n"/>
+      <c r="B33" s="130" t="n"/>
+      <c r="C33" s="130" t="n"/>
+      <c r="D33" s="130" t="n"/>
+      <c r="E33" s="130" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1" s="48">
+      <c r="A34" s="130" t="n"/>
+      <c r="B34" s="130" t="n"/>
+      <c r="C34" s="130" t="n"/>
+      <c r="D34" s="130" t="n"/>
+      <c r="E34" s="130" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1" s="48">
+      <c r="A35" s="130" t="n"/>
+      <c r="B35" s="130" t="n"/>
+      <c r="C35" s="130" t="n"/>
+      <c r="D35" s="130" t="n"/>
+      <c r="E35" s="130" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E8B57"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="48" min="1" max="1"/>
+    <col width="22" customWidth="1" style="48" min="2" max="2"/>
+    <col width="22" customWidth="1" style="48" min="3" max="3"/>
+    <col width="22" customWidth="1" style="48" min="4" max="4"/>
+    <col width="22" customWidth="1" style="48" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" s="48">
+      <c r="A1" s="132" t="inlineStr">
+        <is>
+          <t>Abnahmeprotokoll  ·  eine Seite</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" s="48">
+      <c r="A2" s="126" t="inlineStr">
+        <is>
+          <t>Mit der Unterschrift des Anwendervertreters ist der Entscheidungspunkt ② Abnahme erreicht. Die Übergabe in den Betrieb schliesst das Vorhaben ab (③ Abschluss).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="133" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="B4" s="135" t="n"/>
+      <c r="C4" s="135" t="n"/>
+      <c r="D4" s="135" t="n"/>
+      <c r="E4" s="135" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="48">
+      <c r="A5" s="128" t="inlineStr">
+        <is>
+          <t>Bezeichnung und ID</t>
+        </is>
+      </c>
+      <c r="B5" s="129" t="n"/>
+      <c r="C5" s="130" t="n"/>
+      <c r="D5" s="130" t="n"/>
+      <c r="E5" s="130" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="48">
+      <c r="A6" s="128" t="inlineStr">
+        <is>
+          <t>Abnahmegegenstand und Version</t>
+        </is>
+      </c>
+      <c r="B6" s="129" t="n"/>
+      <c r="C6" s="130" t="n"/>
+      <c r="D6" s="130" t="n"/>
+      <c r="E6" s="130" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="48">
+      <c r="A7" s="128" t="inlineStr">
+        <is>
+          <t>Datum der Abnahme</t>
+        </is>
+      </c>
+      <c r="B7" s="129" t="n"/>
+      <c r="C7" s="130" t="n"/>
+      <c r="D7" s="130" t="n"/>
+      <c r="E7" s="130" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="133" t="inlineStr">
+        <is>
+          <t>Prüfung der Abnahmekriterien aus dem Projektauftrag</t>
+        </is>
+      </c>
+      <c r="B9" s="135" t="n"/>
+      <c r="C9" s="135" t="n"/>
+      <c r="D9" s="135" t="n"/>
+      <c r="E9" s="135" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="131" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B10" s="131" t="inlineStr">
+        <is>
+          <t>Kriterium</t>
+        </is>
+      </c>
+      <c r="C10" s="131" t="inlineStr">
+        <is>
+          <t>✔ erfüllt / ✘ nicht</t>
+        </is>
+      </c>
+      <c r="D10" s="131" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+      <c r="E10" s="131" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1" s="48">
+      <c r="A11" s="130" t="n"/>
+      <c r="B11" s="130" t="n"/>
+      <c r="C11" s="130" t="n"/>
+      <c r="D11" s="130" t="n"/>
+      <c r="E11" s="130" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1" s="48">
+      <c r="A12" s="130" t="n"/>
+      <c r="B12" s="130" t="n"/>
+      <c r="C12" s="130" t="n"/>
+      <c r="D12" s="130" t="n"/>
+      <c r="E12" s="130" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="48">
+      <c r="A13" s="130" t="n"/>
+      <c r="B13" s="130" t="n"/>
+      <c r="C13" s="130" t="n"/>
+      <c r="D13" s="130" t="n"/>
+      <c r="E13" s="130" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="48">
+      <c r="A14" s="130" t="n"/>
+      <c r="B14" s="130" t="n"/>
+      <c r="C14" s="130" t="n"/>
+      <c r="D14" s="130" t="n"/>
+      <c r="E14" s="130" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1" s="48">
+      <c r="A15" s="130" t="n"/>
+      <c r="B15" s="130" t="n"/>
+      <c r="C15" s="130" t="n"/>
+      <c r="D15" s="130" t="n"/>
+      <c r="E15" s="130" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="133" t="inlineStr">
+        <is>
+          <t>Offene Mängel</t>
+        </is>
+      </c>
+      <c r="B17" s="135" t="n"/>
+      <c r="C17" s="135" t="n"/>
+      <c r="D17" s="135" t="n"/>
+      <c r="E17" s="135" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="131" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B18" s="131" t="inlineStr">
+        <is>
+          <t>Mangel</t>
+        </is>
+      </c>
+      <c r="C18" s="131" t="inlineStr">
+        <is>
+          <t>Schwere</t>
+        </is>
+      </c>
+      <c r="D18" s="131" t="inlineStr">
+        <is>
+          <t>Erledigen bis</t>
+        </is>
+      </c>
+      <c r="E18" s="131" t="inlineStr">
+        <is>
+          <t>Wer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" s="48">
+      <c r="A19" s="130" t="n"/>
+      <c r="B19" s="130" t="n"/>
+      <c r="C19" s="130" t="n"/>
+      <c r="D19" s="130" t="n"/>
+      <c r="E19" s="130" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1" s="48">
+      <c r="A20" s="130" t="n"/>
+      <c r="B20" s="130" t="n"/>
+      <c r="C20" s="130" t="n"/>
+      <c r="D20" s="130" t="n"/>
+      <c r="E20" s="130" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="48">
+      <c r="A21" s="130" t="n"/>
+      <c r="B21" s="130" t="n"/>
+      <c r="C21" s="130" t="n"/>
+      <c r="D21" s="130" t="n"/>
+      <c r="E21" s="130" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="133" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="B23" s="135" t="n"/>
+      <c r="C23" s="135" t="n"/>
+      <c r="D23" s="135" t="n"/>
+      <c r="E23" s="135" t="n"/>
+    </row>
+    <row r="24" ht="48" customHeight="1" s="48">
+      <c r="A24" s="128" t="inlineStr">
+        <is>
+          <t>☐ abgenommen
+☐ mit Auflagen
+☐ nicht abgenommen</t>
+        </is>
+      </c>
+      <c r="B24" s="129" t="n"/>
+      <c r="C24" s="130" t="n"/>
+      <c r="D24" s="130" t="n"/>
+      <c r="E24" s="130" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1" s="48">
+      <c r="A25" s="128" t="inlineStr">
+        <is>
+          <t>Auflagen</t>
+        </is>
+      </c>
+      <c r="B25" s="129" t="n"/>
+      <c r="C25" s="130" t="n"/>
+      <c r="D25" s="130" t="n"/>
+      <c r="E25" s="130" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="133" t="inlineStr">
+        <is>
+          <t>Übergabe in den Betrieb</t>
+        </is>
+      </c>
+      <c r="B27" s="135" t="n"/>
+      <c r="C27" s="135" t="n"/>
+      <c r="D27" s="135" t="n"/>
+      <c r="E27" s="135" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="48">
+      <c r="A28" s="128" t="inlineStr">
+        <is>
+          <t>Betriebsdokumentation vorhanden (Ablage)</t>
+        </is>
+      </c>
+      <c r="B28" s="129" t="n"/>
+      <c r="C28" s="130" t="n"/>
+      <c r="D28" s="130" t="n"/>
+      <c r="E28" s="130" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="48">
+      <c r="A29" s="128" t="inlineStr">
+        <is>
+          <t>Zuständig im Betrieb</t>
+        </is>
+      </c>
+      <c r="B29" s="129" t="n"/>
+      <c r="C29" s="130" t="n"/>
+      <c r="D29" s="130" t="n"/>
+      <c r="E29" s="130" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="133" t="inlineStr">
+        <is>
+          <t>Unterschriften</t>
+        </is>
+      </c>
+      <c r="B31" s="135" t="n"/>
+      <c r="C31" s="135" t="n"/>
+      <c r="D31" s="135" t="n"/>
+      <c r="E31" s="135" t="n"/>
+    </row>
+    <row r="32" ht="34" customHeight="1" s="48">
+      <c r="A32" s="128" t="inlineStr">
+        <is>
+          <t>Anwendervertreter, Datum</t>
+        </is>
+      </c>
+      <c r="B32" s="129" t="n"/>
+      <c r="C32" s="130" t="n"/>
+      <c r="D32" s="130" t="n"/>
+      <c r="E32" s="130" t="n"/>
+    </row>
+    <row r="33" ht="34" customHeight="1" s="48">
+      <c r="A33" s="128" t="inlineStr">
+        <is>
+          <t>Auftraggeber (zur Kenntnis), Datum</t>
+        </is>
+      </c>
+      <c r="B33" s="129" t="n"/>
+      <c r="C33" s="130" t="n"/>
+      <c r="D33" s="130" t="n"/>
+      <c r="E33" s="130" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="B32:E32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Smartsheet, data lake and Power BI as HERMES work packages
PM-10 to PM-12 enter the HERMES list, the project status and the weekly
todo. The overview gets a grey "Neu" state, a seventh tile and row
heights derived from the text length.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -31,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=""/>
   </numFmts>
-  <fonts count="47">
+  <fonts count="49">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -354,8 +354,20 @@
       <color rgb="002F5597"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -532,6 +544,11 @@
         <fgColor rgb="002E8B57"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -698,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="141">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1085,6 +1102,19 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1245,14 +1275,28 @@
               </a:ln>
             </spPr>
           </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="7F7F7F"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
-              <f>'HERMES Übersicht'!$P$8:$P$10</f>
+              <f>'HERMES Übersicht'!$P$8:$P$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'HERMES Übersicht'!$Q$8:$Q$10</f>
+              <f>'HERMES Übersicht'!$Q$8:$Q$11</f>
             </numRef>
           </val>
         </ser>
@@ -1314,12 +1358,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'HERMES Übersicht'!$A$8:$A$16</f>
+              <f>'HERMES Übersicht'!$A$8:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'HERMES Übersicht'!$J$8:$J$16</f>
+              <f>'HERMES Übersicht'!$J$8:$J$19</f>
             </numRef>
           </val>
         </ser>
@@ -1369,7 +1413,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3600000" cy="2700000"/>
@@ -1391,7 +1435,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="2700000"/>
@@ -1721,7 +1765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="48" min="1" max="1"/>
@@ -1780,22 +1824,27 @@
         </is>
       </c>
       <c r="H4" s="82" t="n"/>
-      <c r="I4" s="83" t="inlineStr">
+      <c r="I4" s="136" t="inlineStr">
+        <is>
+          <t>● NEU</t>
+        </is>
+      </c>
+      <c r="J4" s="137" t="n"/>
+      <c r="K4" s="83" t="inlineStr">
         <is>
           <t>FREIGABE FEHLT</t>
         </is>
       </c>
-      <c r="J4" s="84" t="n"/>
-      <c r="K4" s="83" t="inlineStr">
+      <c r="L4" s="84" t="n"/>
+      <c r="M4" s="83" t="inlineStr">
         <is>
           <t>ROLLE OFFEN</t>
         </is>
       </c>
-      <c r="L4" s="84" t="n"/>
     </row>
     <row r="5" ht="38" customHeight="1" s="48">
       <c r="A5" s="85" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B5" s="76" t="n"/>
       <c r="C5" s="86" t="n">
@@ -1810,14 +1859,17 @@
         <v>2</v>
       </c>
       <c r="H5" s="82" t="n"/>
-      <c r="I5" s="89" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" s="84" t="n"/>
-      <c r="K5" s="90" t="n">
-        <v>10</v>
+      <c r="I5" s="138" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="137" t="n"/>
+      <c r="K5" s="89" t="n">
+        <v>9</v>
       </c>
       <c r="L5" s="84" t="n"/>
+      <c r="M5" s="90" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="48">
       <c r="A7" s="91" t="inlineStr">
@@ -1896,7 +1948,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" s="48">
+    <row r="8" ht="53" customHeight="1" s="48">
       <c r="A8" s="92" t="inlineStr">
         <is>
           <t>PM-01</t>
@@ -1969,7 +2021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1" s="48">
+    <row r="9" ht="53" customHeight="1" s="48">
       <c r="A9" s="100" t="inlineStr">
         <is>
           <t>PM-02</t>
@@ -2042,7 +2094,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" s="48">
+    <row r="10" ht="53" customHeight="1" s="48">
       <c r="A10" s="92" t="inlineStr">
         <is>
           <t>PM-03</t>
@@ -2115,7 +2167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1" s="48">
+    <row r="11" ht="53" customHeight="1" s="48">
       <c r="A11" s="100" t="inlineStr">
         <is>
           <t>PM-04</t>
@@ -2179,8 +2231,16 @@
           <t>Der Einkauf nutzt das Dashboard ohne Rückfragen, der Lagerwert ist gegen SAP abgestimmt.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="48" customHeight="1" s="48">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Neu</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1" s="48">
       <c r="A12" s="92" t="inlineStr">
         <is>
           <t>PM-05</t>
@@ -2245,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" s="48">
+    <row r="13" ht="53" customHeight="1" s="48">
       <c r="A13" s="100" t="inlineStr">
         <is>
           <t>PM-06</t>
@@ -2310,7 +2370,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1" s="48">
+    <row r="14" ht="38" customHeight="1" s="48">
       <c r="A14" s="92" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -2375,7 +2435,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1" s="48">
+    <row r="15" ht="53" customHeight="1" s="48">
       <c r="A15" s="100" t="inlineStr">
         <is>
           <t>PM-08</t>
@@ -2440,7 +2500,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1" s="48">
+    <row r="16" ht="38" customHeight="1" s="48">
       <c r="A16" s="92" t="inlineStr">
         <is>
           <t>PM-09</t>
@@ -2505,178 +2565,373 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="K18" s="114" t="inlineStr">
+    <row r="17" ht="68" customHeight="1" s="48">
+      <c r="A17" s="100" t="inlineStr">
+        <is>
+          <t>PM-10</t>
+        </is>
+      </c>
+      <c r="B17" s="101" t="inlineStr">
+        <is>
+          <t>Ablösung Smartsheet</t>
+        </is>
+      </c>
+      <c r="C17" s="94" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+      <c r="D17" s="139" t="inlineStr">
+        <is>
+          <t>●  Neu</t>
+        </is>
+      </c>
+      <c r="E17" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F17" s="111" t="inlineStr">
+        <is>
+          <t>Vorschlag: Philip Steiger</t>
+        </is>
+      </c>
+      <c r="G17" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="H17" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="I17" s="112" t="inlineStr">
+        <is>
+          <t>○  offen</t>
+        </is>
+      </c>
+      <c r="J17" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="107" t="inlineStr">
+        <is>
+          <t>Neu aufgenommen am 29.09.2026; es gibt noch keinen Auftrag, keine Anforderungen und keine Aufwandschätzung. Philip Steiger testet das Project Power Pack.</t>
+        </is>
+      </c>
+      <c r="L17" s="107" t="inlineStr">
+        <is>
+          <t>Projektauftrag in der Initialisierung schreiben und dabei die Stufe nach Aufwand festlegen.</t>
+        </is>
+      </c>
+      <c r="M17" s="107" t="inlineStr">
+        <is>
+          <t>Der Projektauftrag ist freigegeben, der Nachfolger von Smartsheet ist bestimmt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="68" customHeight="1" s="48">
+      <c r="A18" s="92" t="inlineStr">
+        <is>
+          <t>PM-11</t>
+        </is>
+      </c>
+      <c r="B18" s="93" t="inlineStr">
+        <is>
+          <t>Data Lake: Leistung analysieren und messen</t>
+        </is>
+      </c>
+      <c r="C18" s="102" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+      <c r="D18" s="139" t="inlineStr">
+        <is>
+          <t>●  Neu</t>
+        </is>
+      </c>
+      <c r="E18" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F18" s="96" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="G18" s="140" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="H18" s="140" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="I18" s="140" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="J18" s="98" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="99" t="inlineStr">
+        <is>
+          <t>Neu aufgenommen am 29.09.2026 als Kleinauftrag «Analyse und Messung»; die Abgrenzung zu PM-09 (Tempo der Webapp, am 28.09.2026 weitgehend erledigt) ist zu klären.</t>
+        </is>
+      </c>
+      <c r="L18" s="99" t="inlineStr">
+        <is>
+          <t>Klären, welche Leistung gemeint ist, und danach messen; je nach Befund ein Vorhaben daraus machen.</t>
+        </is>
+      </c>
+      <c r="M18" s="99" t="inlineStr">
+        <is>
+          <t>Ein Messbericht mit Befund und Empfehlung liegt vor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="68" customHeight="1" s="48">
+      <c r="A19" s="100" t="inlineStr">
+        <is>
+          <t>PM-12</t>
+        </is>
+      </c>
+      <c r="B19" s="101" t="inlineStr">
+        <is>
+          <t>Power BI: je Dashboard ein Anwendervertreter</t>
+        </is>
+      </c>
+      <c r="C19" s="102" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+      <c r="D19" s="139" t="inlineStr">
+        <is>
+          <t>●  Neu</t>
+        </is>
+      </c>
+      <c r="E19" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="F19" s="104" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="G19" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="H19" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="I19" s="105" t="inlineStr">
+        <is>
+          <t>–  nicht nötig</t>
+        </is>
+      </c>
+      <c r="J19" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="107" t="inlineStr">
+        <is>
+          <t>Neu aufgenommen am 29.09.2026; die Liste der Dashboards und ihre Zuordnung zu Fachbereichen fehlt noch.</t>
+        </is>
+      </c>
+      <c r="L19" s="107" t="inlineStr">
+        <is>
+          <t>Dashboards auflisten und je Dashboard einen Anwendervertreter aus dem Fachbereich benennen, der auch für die Datenqualität verantwortlich ist.</t>
+        </is>
+      </c>
+      <c r="M19" s="107" t="inlineStr">
+        <is>
+          <t>Jedes produktive Dashboard hat einen benannten Anwendervertreter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="K21" s="114" t="inlineStr">
         <is>
           <t>So wird eingestuft (HERMES zugeschnitten)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="K19" s="115" t="inlineStr">
+    <row r="22">
+      <c r="K22" s="115" t="inlineStr">
         <is>
           <t>Stufe</t>
         </is>
       </c>
-      <c r="L19" s="115" t="inlineStr">
+      <c r="L22" s="115" t="inlineStr">
         <is>
           <t>Aufwand</t>
         </is>
       </c>
-      <c r="M19" s="115" t="inlineStr">
+      <c r="M22" s="115" t="inlineStr">
         <is>
           <t>Vorgehen</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="K20" s="116" t="inlineStr">
+    <row r="23">
+      <c r="K23" s="116" t="inlineStr">
         <is>
           <t>Kleinauftrag</t>
         </is>
       </c>
-      <c r="L20" s="117" t="inlineStr">
+      <c r="L23" s="117" t="inlineStr">
         <is>
           <t>unter ca. 5 Personentage</t>
         </is>
       </c>
-      <c r="M20" s="117" t="inlineStr">
+      <c r="M23" s="117" t="inlineStr">
         <is>
           <t>Ticket, keine HERMES-Dokumente</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="K21" s="118" t="inlineStr">
+    <row r="24">
+      <c r="K24" s="118" t="inlineStr">
         <is>
           <t>Vorhaben</t>
         </is>
       </c>
-      <c r="L21" s="117" t="inlineStr">
+      <c r="L24" s="117" t="inlineStr">
         <is>
           <t>ca. 5 bis 40 Personentage</t>
         </is>
       </c>
-      <c r="M21" s="117" t="inlineStr">
+      <c r="M24" s="117" t="inlineStr">
         <is>
           <t>Auftrag, Abnahme, Statuszeile</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="K22" s="119" t="inlineStr">
+    <row r="25">
+      <c r="K25" s="119" t="inlineStr">
         <is>
           <t>Projekt</t>
         </is>
       </c>
-      <c r="L22" s="117" t="inlineStr">
+      <c r="L25" s="117" t="inlineStr">
         <is>
           <t>über ca. 40 Personentage</t>
         </is>
       </c>
-      <c r="M22" s="117" t="inlineStr">
+      <c r="M25" s="117" t="inlineStr">
         <is>
           <t>HERMES zugeschnitten, mit Risikoliste, eventuell Ausschuss</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1" s="48">
-      <c r="K24" s="120" t="inlineStr">
-        <is>
-          <t>① Freigabe</t>
-        </is>
-      </c>
-      <c r="L24" s="121" t="inlineStr">
-        <is>
-          <t>Der Auftraggeber hat den Projektauftrag unterschrieben.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1" s="48">
-      <c r="K25" s="120" t="inlineStr">
-        <is>
-          <t>② Abnahme</t>
-        </is>
-      </c>
-      <c r="L25" s="121" t="inlineStr">
-        <is>
-          <t>Der Anwendervertreter bestätigt fachlich, das Ergebnis ist produktiv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1" s="48">
-      <c r="K26" s="120" t="inlineStr">
-        <is>
-          <t>③ Abschluss</t>
-        </is>
-      </c>
-      <c r="L26" s="121" t="inlineStr">
-        <is>
-          <t>Übergeben in den Betrieb, mit kurzer Betriebsdokumentation.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1" s="48">
       <c r="K27" s="120" t="inlineStr">
         <is>
-          <t>✔ / ○</t>
+          <t>① Freigabe</t>
         </is>
       </c>
       <c r="L27" s="121" t="inlineStr">
         <is>
-          <t>Erledigt mit Datum / noch offen.</t>
+          <t>Der Auftraggeber hat den Projektauftrag unterschrieben.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1" s="48">
       <c r="K28" s="120" t="inlineStr">
         <is>
-          <t>⚠ festlegen</t>
+          <t>② Abnahme</t>
         </is>
       </c>
       <c r="L28" s="121" t="inlineStr">
         <is>
-          <t>Die Rolle ist noch niemandem zugeordnet.</t>
+          <t>Der Anwendervertreter bestätigt fachlich, das Ergebnis ist produktiv.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1" s="48">
       <c r="K29" s="120" t="inlineStr">
         <is>
+          <t>③ Abschluss</t>
+        </is>
+      </c>
+      <c r="L29" s="121" t="inlineStr">
+        <is>
+          <t>Übergeben in den Betrieb, mit kurzer Betriebsdokumentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1" s="48">
+      <c r="K30" s="120" t="inlineStr">
+        <is>
+          <t>✔ / ○</t>
+        </is>
+      </c>
+      <c r="L30" s="121" t="inlineStr">
+        <is>
+          <t>Erledigt mit Datum / noch offen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1" s="48">
+      <c r="K31" s="120" t="inlineStr">
+        <is>
+          <t>⚠ festlegen</t>
+        </is>
+      </c>
+      <c r="L31" s="121" t="inlineStr">
+        <is>
+          <t>Die Rolle ist noch niemandem zugeordnet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1" s="48">
+      <c r="K32" s="120" t="inlineStr">
+        <is>
           <t>● Ampel</t>
         </is>
       </c>
-      <c r="L29" s="121" t="inlineStr">
-        <is>
-          <t>Grün im Plan · Gelb wartet auf Entscheid oder Zulieferung · Rot blockiert oder Termin überschritten.</t>
+      <c r="L32" s="121" t="inlineStr">
+        <is>
+          <t>Grün im Plan · Gelb wartet auf Entscheid oder Zulieferung · Rot blockiert oder Termin überschritten · Grau neu, noch ohne Stand.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="L32:M32"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="L28:M28"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L30:M30"/>
     <mergeCell ref="L29:M29"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="L25:M25"/>
     <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="L31:M31"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K21:M21"/>
     <mergeCell ref="L27:M27"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J8:J16">
+  <conditionalFormatting sqref="J8:J19">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -3079,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -5678,8 +5933,185 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="57" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B44" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C44" s="57" t="inlineStr">
+        <is>
+          <t>Projektmanagement</t>
+        </is>
+      </c>
+      <c r="D44" s="57" t="inlineStr">
+        <is>
+          <t>PM-10</t>
+        </is>
+      </c>
+      <c r="E44" s="57" t="inlineStr">
+        <is>
+          <t>Ablösung Smartsheet: Projektauftrag schreiben</t>
+        </is>
+      </c>
+      <c r="F44" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Philip Steiger</t>
+        </is>
+      </c>
+      <c r="G44" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H44" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I44" s="57" t="inlineStr"/>
+      <c r="J44" s="57" t="inlineStr">
+        <is>
+          <t>Projektauftrag in der Initialisierung schreiben (Vorlage im Blatt Vorlage Projektauftrag), Stufe nach Aufwandschätzung festlegen, Abgleich mit dem Project-Power-Pack-Test von Philip Steiger.</t>
+        </is>
+      </c>
+      <c r="K44" s="57" t="inlineStr"/>
+      <c r="L44" s="57" t="inlineStr">
+        <is>
+          <t>PM-10</t>
+        </is>
+      </c>
+      <c r="M44" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="57" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C45" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D45" s="57" t="inlineStr">
+        <is>
+          <t>PM-11</t>
+        </is>
+      </c>
+      <c r="E45" s="57" t="inlineStr">
+        <is>
+          <t>Data Lake: Leistung analysieren und messen</t>
+        </is>
+      </c>
+      <c r="F45" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G45" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H45" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I45" s="57" t="inlineStr"/>
+      <c r="J45" s="57" t="inlineStr">
+        <is>
+          <t>Klären, welche Leistung gemeint ist und wie sie sich von PM-09 abgrenzt; danach messen und einen kurzen Befund schreiben.</t>
+        </is>
+      </c>
+      <c r="K45" s="57" t="inlineStr"/>
+      <c r="L45" s="57" t="inlineStr">
+        <is>
+          <t>PM-11</t>
+        </is>
+      </c>
+      <c r="M45" s="123" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="57" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C46" s="57" t="inlineStr">
+        <is>
+          <t>Projektmanagement</t>
+        </is>
+      </c>
+      <c r="D46" s="57" t="inlineStr">
+        <is>
+          <t>PM-12</t>
+        </is>
+      </c>
+      <c r="E46" s="57" t="inlineStr">
+        <is>
+          <t>Power BI: Anwendervertreter je Dashboard</t>
+        </is>
+      </c>
+      <c r="F46" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G46" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H46" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I46" s="57" t="inlineStr"/>
+      <c r="J46" s="57" t="inlineStr">
+        <is>
+          <t>Produktive Dashboards auflisten und je Dashboard einen Anwendervertreter aus dem Fachbereich benennen lassen.</t>
+        </is>
+      </c>
+      <c r="K46" s="57" t="inlineStr"/>
+      <c r="L46" s="57" t="inlineStr">
+        <is>
+          <t>PM-12</t>
+        </is>
+      </c>
+      <c r="M46" s="123" t="inlineStr">
+        <is>
+          <t>Kleinauftrag</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M43"/>
+  <autoFilter ref="A1:M46"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Bring the docs up to date for 29.09.
The formula summary no longer recommends the capped cockpit export for
full recalculation, marks Mask/Convert as set in production, adds the
Spain period rule and flags the July supplier conflict as superseded.
The review findings enter the issue log as ISS-018 with a weekly todo
row. RAG summaries, lastchange.md and the router carry today's state:
HERMES view, PM-10 to PM-12, the finance review and Paola's mail.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -6110,8 +6110,67 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="57" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C47" s="57" t="inlineStr">
+        <is>
+          <t>Finance Gruppenmarge</t>
+        </is>
+      </c>
+      <c r="D47" s="57" t="inlineStr">
+        <is>
+          <t>ISS-018</t>
+        </is>
+      </c>
+      <c r="E47" s="57" t="inlineStr">
+        <is>
+          <t>Konsistenzbefunde vom 29.09.: Rechen- und Anzeigefehler beheben</t>
+        </is>
+      </c>
+      <c r="F47" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Andreas</t>
+        </is>
+      </c>
+      <c r="G47" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H47" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I47" s="57" t="inlineStr"/>
+      <c r="J47" s="57" t="inlineStr">
+        <is>
+          <t>Codex-Befunde gegen den Code bestätigt. Reparatur von A1 (CHF-Schalter gegen Prüfbuch), A3/A4 (falsche Währungslabels) und A5 (Cockpit-Export nur 1'000 Zeilen) beauftragen lassen; B1 bis B3 fachlich mit Andreas entscheiden. Bericht docs/FINANCE_REVIEW_2026-09-29.md.</t>
+        </is>
+      </c>
+      <c r="K47" s="57" t="inlineStr"/>
+      <c r="L47" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M47" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M46"/>
+  <autoFilter ref="A1:M47"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Split the review findings into individual issues
ISS-018.1 to .4 cover the visible calculation and label errors (A1, A3,
A4, A5), ISS-018.5 to .7 the business decisions for Andreas (B1, B2,
B3.1). The latent findings stay under the umbrella ISS-018. The weekly
todo gets one repair row and one decision row.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -6118,7 +6118,7 @@
       </c>
       <c r="B47" s="57" t="inlineStr">
         <is>
-          <t>Entscheid</t>
+          <t>Umsetzung</t>
         </is>
       </c>
       <c r="C47" s="57" t="inlineStr">
@@ -6133,12 +6133,12 @@
       </c>
       <c r="E47" s="57" t="inlineStr">
         <is>
-          <t>Konsistenzbefunde vom 29.09.: Rechen- und Anzeigefehler beheben</t>
+          <t>Konsistenz: Reparatur A1, A3, A4, A5 (ISS-018.1 bis .4)</t>
         </is>
       </c>
       <c r="F47" s="57" t="inlineStr">
         <is>
-          <t>Ingo / Andreas</t>
+          <t>Ingo</t>
         </is>
       </c>
       <c r="G47" s="57" t="inlineStr">
@@ -6154,7 +6154,7 @@
       <c r="I47" s="57" t="inlineStr"/>
       <c r="J47" s="57" t="inlineStr">
         <is>
-          <t>Codex-Befunde gegen den Code bestätigt. Reparatur von A1 (CHF-Schalter gegen Prüfbuch), A3/A4 (falsche Währungslabels) und A5 (Cockpit-Export nur 1'000 Zeilen) beauftragen lassen; B1 bis B3 fachlich mit Andreas entscheiden. Bericht docs/FINANCE_REVIEW_2026-09-29.md.</t>
+          <t>Sichtbare Rechen- und Anzeigefehler beheben: CHF-Schalter gegen Prüfbuch, zwei falsche Währungslabels, Cockpit-Export nur 1'000 Zeilen. Braucht einen Reparaturauftrag mit Deploy. Bericht docs/FINANCE_REVIEW_2026-09-29.md.</t>
         </is>
       </c>
       <c r="K47" s="57" t="inlineStr"/>
@@ -6169,8 +6169,67 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="57" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C48" s="57" t="inlineStr">
+        <is>
+          <t>Finance Gruppenmarge</t>
+        </is>
+      </c>
+      <c r="D48" s="57" t="inlineStr">
+        <is>
+          <t>ISS-018</t>
+        </is>
+      </c>
+      <c r="E48" s="57" t="inlineStr">
+        <is>
+          <t>Konsistenz: Fachentscheide B1 bis B3 (ISS-018.5 bis .7)</t>
+        </is>
+      </c>
+      <c r="F48" s="57" t="inlineStr">
+        <is>
+          <t>Andreas / Ingo</t>
+        </is>
+      </c>
+      <c r="G48" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H48" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I48" s="57" t="inlineStr"/>
+      <c r="J48" s="57" t="inlineStr">
+        <is>
+          <t>Andreas entscheidet: Wertgutschriften mit Menge 0, Kosten kostenloser Ware, interner Lieferant ohne Konzernkosten soll offen bleiben statt OK. Vorher Fallzahlen in den Daten messen.</t>
+        </is>
+      </c>
+      <c r="K48" s="57" t="inlineStr"/>
+      <c r="L48" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M48" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M47"/>
+  <autoFilter ref="A1:M48"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Resolve the markdown consistency findings and record the Spain import stop
All 15 finding groups from Codex's markdown review are fixed, using
Ingo's decisions and read-only checks against code and copies of the
production database: Spain is Sage (PrecioCoste, not the German
EinstandsPreis mapping the review cited), UK has a cost column, IT/IN
group costs are live since 25.08., Convert is the code default, the
three separate rate rules are written down, the HR review file marks
what changed on 28.09., and baum.md lists every file again.

ISS-004.2 is closed: the 7-day export is active and was decided on
02.09. Checking it revealed ISS-020: no new Spanish rows have reached
production since mid-July; the folder listing reads only the first
page from Graph. ISS-019 tracks the group-wide railway view and DB4.
Heiko and Patrick are added to the people list.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$50</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="J15" s="106" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" s="107" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -6228,8 +6228,126 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="57" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C49" s="57" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="D49" s="57" t="inlineStr">
+        <is>
+          <t>ISS-019</t>
+        </is>
+      </c>
+      <c r="E49" s="57" t="inlineStr">
+        <is>
+          <t>Railway-Gesamtsicht für Heiko und Patrick, DB4 klären</t>
+        </is>
+      </c>
+      <c r="F49" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Patrik / Andreas</t>
+        </is>
+      </c>
+      <c r="G49" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H49" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I49" s="57" t="inlineStr"/>
+      <c r="J49" s="57" t="inlineStr">
+        <is>
+          <t>Antwort per Teams geben (Umsatz technisch für alle Standorte da, belastbar nur DE); Patrik die 171 Vorschläge außerhalb DE bestätigen lassen; mit Andreas und Rohail festlegen, was DB4 enthält, danach Export-SQL um vorhandene Quellfelder erweitern.</t>
+        </is>
+      </c>
+      <c r="K49" s="57" t="inlineStr"/>
+      <c r="L49" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M49" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="57" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C50" s="57" t="inlineStr">
+        <is>
+          <t>Finance ES</t>
+        </is>
+      </c>
+      <c r="D50" s="57" t="inlineStr">
+        <is>
+          <t>ISS-020</t>
+        </is>
+      </c>
+      <c r="E50" s="57" t="inlineStr">
+        <is>
+          <t>Spanien: seit Mitte Juli keine neuen Zeilen im Import</t>
+        </is>
+      </c>
+      <c r="F50" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G50" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H50" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I50" s="57" t="inlineStr"/>
+      <c r="J50" s="57" t="inlineStr">
+        <is>
+          <t>Dateien im SharePoint-Ordner Import/Finance/Spanien zählen. Liegen dort mehr als 200 Einträge, liest der Import die neuesten nicht (Ordnerliste ohne Folgeseiten); dann Reparatur mit Deploy und Spanien neu importieren.</t>
+        </is>
+      </c>
+      <c r="K50" s="57" t="inlineStr"/>
+      <c r="L50" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M50" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M48"/>
+  <autoFilter ref="A1:M50"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Record the 09:25 deploy of the SharePoint paging fix
ISS-020 cause is confirmed from the production event log and the fix
is live; the Spain re-import shows with the next run. Deployment
protocol, issue log, weekly todo and the Spain notes carry the state.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -6323,15 +6323,15 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H50" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H50" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="I50" s="57" t="inlineStr"/>
       <c r="J50" s="57" t="inlineStr">
         <is>
-          <t>Dateien im SharePoint-Ordner Import/Finance/Spanien zählen. Liegen dort mehr als 200 Einträge, liest der Import die neuesten nicht (Ordnerliste ohne Folgeseiten); dann Reparatur mit Deploy und Spanien neu importieren.</t>
+          <t>Ursache bestätigt und Korrektur seit 29.09. 09:25 produktiv. Offen: nächster Spanien-Import muss die Dateien ab 16.07. einlesen, danach Sales_All neu erzeugen und Spanien-Zahlen prüfen.</t>
         </is>
       </c>
       <c r="K50" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Document Codex's HR and purchasing repairs and the sent reply to Paola
Codex fixed the HR period/YTD logic, person quota, year filter and
table caps, and the purchasing year total, category and exchange-rate
warning. The code is local only: not committed, not deployed; the RAG
summaries, project status and weekly todo say so and carry the commit
and deploy steps. Codex's own report and doc updates are committed here.

Ingo sent the reply to Paola today; ISS-007.1 needs nothing more and
ISS-007.2 waits for her confirmation of the balance-sheet stock value.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$52</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -4537,7 +4537,7 @@
       <c r="I20" s="57" t="inlineStr"/>
       <c r="J20" s="57" t="inlineStr">
         <is>
-          <t>Andreas hat am 09.09.2026 entschieden: keine Priorität, erneute Betrachtung 2027. Paola am 29.09.2026: laut ihren SAP-Beratern doch umstellbar, aber nur mit Bestand null, Belegabschluss, Betriebsunterbruch und Inventur. Offen ist nur die Rückmeldung an Paola, zusammen mit ISS-007.2.</t>
+          <t>Andreas hat am 09.09.2026 entschieden: keine Priorität, erneute Betrachtung 2027. Rückmeldung an Paola am 29.09.2026 versendet. Keine weitere Aktion.</t>
         </is>
       </c>
       <c r="K20" s="57" t="inlineStr"/>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B41" s="57" t="inlineStr">
         <is>
-          <t>Heute</t>
+          <t>Hoch, haengt an anderen</t>
         </is>
       </c>
       <c r="C41" s="57" t="inlineStr">
@@ -5794,13 +5794,13 @@
       </c>
       <c r="H41" s="57" t="inlineStr">
         <is>
-          <t>Gemessen, Fachentscheid offen</t>
+          <t>Wartet auf andere</t>
         </is>
       </c>
       <c r="I41" s="57" t="inlineStr"/>
       <c r="J41" s="57" t="inlineStr">
         <is>
-          <t>Paola baut laut Mail vom 29.09.2026 mit ihren SAP-Beratern eine Abfrage für einen Moving-Average-Wert je Artikel. Das ist seit 09.09. zentral gemessen (OITM.StockValue / OnHand). Paola zurückmelden, bevor Beraterstunden anfallen; danach Fachentscheid Andreas: führende Kostenbasis oder Plausibilisierung.</t>
+          <t>Antwort an Paola am 29.09.2026 versendet. Jetzt auf ihre Bestätigung warten, ob StockValue dem bilanziellen Bestandswert entspricht; danach Fachentscheid Andreas.</t>
         </is>
       </c>
       <c r="K41" s="57" t="inlineStr"/>
@@ -6346,8 +6346,126 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="57" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C51" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D51" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E51" s="57" t="inlineStr">
+        <is>
+          <t>HR-Review-Reparaturen von Codex committen, deployen, sichtprüfen</t>
+        </is>
+      </c>
+      <c r="F51" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G51" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H51" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I51" s="57" t="inlineStr"/>
+      <c r="J51" s="57" t="inlineStr">
+        <is>
+          <t>H1 bis H5 (Zeitraum/YTD, Personenquote, Jahresfilter, Tabellenkappung) sind lokal umgesetzt, 138/138 gezielte Tests laut Codex, aber nicht committet und nicht deployed. Vor dem Deploy Gesamtsuite im sauberen Worktree; Finance_All nicht mitnehmen. Bericht docs/HR_EINKAUF_REVIEW_2026-09-29.md.</t>
+        </is>
+      </c>
+      <c r="K51" s="57" t="inlineStr"/>
+      <c r="L51" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M51" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="57" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C52" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D52" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E52" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf-Review-Reparaturen von Codex committen, deployen, sichtprüfen</t>
+        </is>
+      </c>
+      <c r="F52" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G52" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H52" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I52" s="57" t="inlineStr"/>
+      <c r="J52" s="57" t="inlineStr">
+        <is>
+          <t>E1 Jahres-Spend ungekappt, E2 Warengruppe einheitlich, C1 keine Live-Stichproben-KPIs, C2 Warnung bei fehlenden Kursen sind lokal umgesetzt, nicht committet und nicht deployed. Offen bleibt der Fachentscheid zur Ersatzkursregel.</t>
+        </is>
+      </c>
+      <c r="K52" s="57" t="inlineStr"/>
+      <c r="L52" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M52" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M50"/>
+  <autoFilter ref="A1:M52"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Record the 10:07 deploy, the Spain re-import and Paola's scope question
HR and purchasing repairs are live (eafd1c5, c1fdfa2). Sales_All of
29.09. holds 8,109 Spanish rows up to 28.09., so ISS-020 is closed.
Paola asked whether our stock value uses the same source and scope as
her Inventory Audit Report; a read-only per-warehouse breakdown and a
reply draft are in section 7c of the reference cost note.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B41" s="57" t="inlineStr">
         <is>
-          <t>Hoch, haengt an anderen</t>
+          <t>Heute</t>
         </is>
       </c>
       <c r="C41" s="57" t="inlineStr">
@@ -5792,15 +5792,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H41" s="57" t="inlineStr">
-        <is>
-          <t>Wartet auf andere</t>
+      <c r="H41" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
         </is>
       </c>
       <c r="I41" s="57" t="inlineStr"/>
       <c r="J41" s="57" t="inlineStr">
         <is>
-          <t>Antwort an Paola am 29.09.2026 versendet. Jetzt auf ihre Bestätigung warten, ob StockValue dem bilanziellen Bestandswert entspricht; danach Fachentscheid Andreas.</t>
+          <t>Paola hat am 29.09. nach Quelle und Lagerumfang gefragt. Antwortentwurf mit Aufteilung je Lager liegt vor (Referenzkosten-Doku 7c): sie soll die physischen Lager nennen, dann Abgleich zum Monatsende.</t>
         </is>
       </c>
       <c r="K41" s="57" t="inlineStr"/>
@@ -6323,18 +6323,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H50" s="59" t="inlineStr">
-        <is>
-          <t>Läuft</t>
+      <c r="H50" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I50" s="57" t="inlineStr"/>
       <c r="J50" s="57" t="inlineStr">
         <is>
-          <t>Ursache bestätigt und Korrektur seit 29.09. 09:25 produktiv. Offen: nächster Spanien-Import muss die Dateien ab 16.07. einlesen, danach Sales_All neu erzeugen und Spanien-Zahlen prüfen.</t>
-        </is>
-      </c>
-      <c r="K50" s="57" t="inlineStr"/>
+          <t>Ursache SharePoint-Ordnerliste (200 Einträge) behoben, deployed 09:25; Sales_All_2026-09-29 enthält Spanien bis 28.09.2026 (8'109 Zeilen).</t>
+        </is>
+      </c>
+      <c r="K50" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L50" s="57" t="inlineStr">
         <is>
           <t>PM-05</t>
@@ -6382,18 +6386,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H51" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H51" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I51" s="57" t="inlineStr"/>
       <c r="J51" s="57" t="inlineStr">
         <is>
-          <t>H1 bis H5 (Zeitraum/YTD, Personenquote, Jahresfilter, Tabellenkappung) sind lokal umgesetzt, 138/138 gezielte Tests laut Codex, aber nicht committet und nicht deployed. Vor dem Deploy Gesamtsuite im sauberen Worktree; Finance_All nicht mitnehmen. Bericht docs/HR_EINKAUF_REVIEW_2026-09-29.md.</t>
-        </is>
-      </c>
-      <c r="K51" s="57" t="inlineStr"/>
+          <t>H1 bis H5 (Zeitraum/YTD, Personenquote, Jahresfilter, Tabellenkappung) sind committet (eafd1c5, c1fdfa2) und seit 29.09.2026 10:07 produktiv. Offen bleibt nur die angemeldete Sichtprüfung.</t>
+        </is>
+      </c>
+      <c r="K51" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L51" s="57" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -6441,18 +6449,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H52" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H52" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I52" s="57" t="inlineStr"/>
       <c r="J52" s="57" t="inlineStr">
         <is>
-          <t>E1 Jahres-Spend ungekappt, E2 Warengruppe einheitlich, C1 keine Live-Stichproben-KPIs, C2 Warnung bei fehlenden Kursen sind lokal umgesetzt, nicht committet und nicht deployed. Offen bleibt der Fachentscheid zur Ersatzkursregel.</t>
-        </is>
-      </c>
-      <c r="K52" s="57" t="inlineStr"/>
+          <t>E1 Jahres-Spend ungekappt, E2 Warengruppe einheitlich, C1 keine Live-Stichproben-KPIs, C2 Warnung bei fehlenden Kursen sind committet (eafd1c5, c1fdfa2) und seit 29.09.2026 10:07 produktiv. Offen bleibt nur die angemeldete Sichtprüfung.</t>
+        </is>
+      </c>
+      <c r="K52" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L52" s="57" t="inlineStr">
         <is>
           <t>PM-04</t>

</xml_diff>

<commit_message>
Record the 10:22 cockpit deploy and the refreshed weekly todo
ISS-018.2 and .3 are fixed, .4 is flagged in the export, .1 waits for
Andreas. France delivers again (ISS-001.2 closed), the speed item is
done, the duplicate of ISS-018.7 is merged, and the purchasing label
change is held for a decision because it contradicts the Marco review.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -2547,7 +2547,7 @@
         </is>
       </c>
       <c r="J16" s="98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" s="99" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="B5" s="57" t="inlineStr">
         <is>
-          <t>Hoch, haengt an anderen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="C5" s="57" t="inlineStr">
@@ -3636,18 +3636,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H5" s="57" t="inlineStr">
-        <is>
-          <t>Wartet auf andere</t>
+      <c r="H5" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I5" s="57" t="inlineStr"/>
       <c r="J5" s="57" t="inlineStr">
         <is>
-          <t>Eskalieren, seit 30.07.2026 keine Faktura mehr (18 Tage)</t>
-        </is>
-      </c>
-      <c r="K5" s="57" t="inlineStr"/>
+          <t>Gemessen am 29.09.2026 in Sales_All_2026-09-29.xlsx: Frankreich liefert wieder, Rechnungen bis 28.09.2026, 140 Zeilen seit 01.08. Keine Eskalation mehr nötig.</t>
+        </is>
+      </c>
+      <c r="K5" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L5" s="57" t="inlineStr">
         <is>
           <t>PM-05</t>
@@ -5107,7 +5111,7 @@
       </c>
       <c r="B30" s="57" t="inlineStr">
         <is>
-          <t>Heute</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="C30" s="57" t="inlineStr">
@@ -5135,18 +5139,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H30" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H30" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I30" s="57" t="inlineStr"/>
       <c r="J30" s="57" t="inlineStr">
         <is>
-          <t>Am 02.09.2026 im Code gefunden: GroupDistributionWithoutGroupCost prüft nur den Sales Type LRD, nicht ob eine liefernde Konzerngesellschaft erkannt wurde. Zeilen mit Lieferant Trafag AG oder Trafag Italia ohne Konzernkostentreffer zeigen still eine Marge auf dem lokalen IC-Preis. Obergrenze 19'221 Zeilen (18,3 %). Zuerst die echte Menge gegen GroupStandardCosts in der Produktiv-DB messen, dann Andreas entscheiden lassen</t>
-        </is>
-      </c>
-      <c r="K30" s="57" t="inlineStr"/>
+          <t>Zusammengeführt mit ISS-018.7 (Zeile 47): derselbe Befund, dort mit Fachentscheid Andreas geführt.</t>
+        </is>
+      </c>
+      <c r="K30" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L30" s="57" t="inlineStr">
         <is>
           <t>PM-05</t>
@@ -5343,7 +5351,7 @@
       </c>
       <c r="B34" s="57" t="inlineStr">
         <is>
-          <t>Umsetzung</t>
+          <t>Entscheid</t>
         </is>
       </c>
       <c r="C34" s="57" t="inlineStr">
@@ -5371,15 +5379,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H34" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H34" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf Entscheid</t>
         </is>
       </c>
       <c r="I34" s="57" t="inlineStr"/>
       <c r="J34" s="57" t="inlineStr">
         <is>
-          <t>Beim Deploy vom 10.09.2026 um 09:40 wurde Commit d5bc321 ausgeliefert. Die zuletzt geaenderten drei Statusbeschriftungen waren NICHT committet und sind damit nicht produktiv: "Gebuchter Spend" statt "Bestellwert im Zeitraum" und "Einteilungen" statt "Einteilungen im Zeitraum". Der alte Text steht weiter an vier Stellen in PurchasingDashboard.razor und sechs in PurchasingUiTextCatalog.cs. Nachziehen und ausliefern. Ausserdem steht die produktive Sichtpruefung der neuen Kacheln und der Quellenhilfe noch aus.</t>
+          <t>Nicht nachgezogen, weil es einem dokumentierten Entscheid widerspricht: „Bestellwert im Zeitraum“ wurde nach dem Abgleich mit Marco gewählt, weil er „gebucht“ als „schon Wareneingang“ las (PURCHASING_DASHBOARD_2026-06-05.md). Codex’ späteres „Gebuchter Spend“ brächte das Missverständnis zurück. Ingo entscheidet, ob es beim heutigen Text bleibt; dann Zeile schliessen.</t>
         </is>
       </c>
       <c r="K34" s="57" t="inlineStr"/>
@@ -5579,7 +5587,7 @@
       </c>
       <c r="B38" s="57" t="inlineStr">
         <is>
-          <t>Umsetzung</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="C38" s="57" t="inlineStr">
@@ -5607,18 +5615,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H38" s="59" t="inlineStr">
-        <is>
-          <t>Läuft</t>
+      <c r="H38" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I38" s="57" t="inlineStr"/>
       <c r="J38" s="57" t="inlineStr">
         <is>
-          <t>Erledigt am 28.09.: Oberfläche erscheint sofort (4f2c62f), Einkauf-Standardansicht vorgewärmt (d32a6aa), Management-Cockpit lokal 41 s -&gt; 3,3 s (5a26596), Export-Dashboard 2,3 s -&gt; 0,07 s und SQLite-Cache (c35d3fa), Alles produktiv seit 28.09. 13:32; Server-Einkaufsberechnung 104,7 s -&gt; 24,4 s durch den SQLite-Cache. Offen: Finanzvergleich ohne CSV-Cache (2,4 s lokal), Rest-Faktor 2 der VM. Details docs/PLATTFORM_TEMPO_2026-09-28.md.</t>
-        </is>
-      </c>
-      <c r="K38" s="57" t="inlineStr"/>
+          <t>Am 28.09. produktiv umgesetzt (Oberfläche sofort, Cockpit 41 s -&gt; 3,3 s, Export-Dashboard 0,07 s, SQLite-Cache). Offen ist nur noch die IT-Einstellung, geführt als ISS-017 (Zeile 36).</t>
+        </is>
+      </c>
+      <c r="K38" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L38" s="57" t="inlineStr">
         <is>
           <t>PM-09</t>
@@ -6118,7 +6130,7 @@
       </c>
       <c r="B47" s="57" t="inlineStr">
         <is>
-          <t>Umsetzung</t>
+          <t>Entscheid</t>
         </is>
       </c>
       <c r="C47" s="57" t="inlineStr">
@@ -6133,12 +6145,12 @@
       </c>
       <c r="E47" s="57" t="inlineStr">
         <is>
-          <t>Konsistenz: Reparatur A1, A3, A4, A5 (ISS-018.1 bis .4)</t>
+          <t>Konsistenz: A1 offen, A3/A4 behoben, A5 ausgewiesen (ISS-018.1 bis .4)</t>
         </is>
       </c>
       <c r="F47" s="57" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Andreas / Ingo</t>
         </is>
       </c>
       <c r="G47" s="57" t="inlineStr">
@@ -6146,15 +6158,15 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H47" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H47" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf Entscheid</t>
         </is>
       </c>
       <c r="I47" s="57" t="inlineStr"/>
       <c r="J47" s="57" t="inlineStr">
         <is>
-          <t>Sichtbare Rechen- und Anzeigefehler beheben: CHF-Schalter gegen Prüfbuch, zwei falsche Währungslabels, Cockpit-Export nur 1'000 Zeilen. Braucht einen Reparaturauftrag mit Deploy. Bericht docs/FINANCE_REVIEW_2026-09-29.md.</t>
+          <t>A3 und A4 behoben, A5 im Export ausgewiesen, produktiv seit 29.09.2026 10:22 (91fd9dc). Offen: A1, mit welchem Kurs der CHF-Schalter rechnen soll (Kursprofil oder 31.12.) – Andreas.</t>
         </is>
       </c>
       <c r="K47" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Record the supplier-field check for Germany and Spain
Neither export query reads a supplier column. Alphaplan keeps suppliers
(the old manual Excel carried them), so the gap came with the switch to
the invoice CSVs; for Spain no article supplier shows in our schema
extracts. The next step is a read-only schema extract from the local IT,
not a data-maintenance request. The weekly todo refresh is closed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -4147,7 +4147,7 @@
       </c>
       <c r="B14" s="57" t="inlineStr">
         <is>
-          <t>Umsetzung</t>
+          <t>Hoch, haengt an anderen</t>
         </is>
       </c>
       <c r="C14" s="57" t="inlineStr">
@@ -4175,15 +4175,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H14" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H14" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf andere</t>
         </is>
       </c>
       <c r="I14" s="57" t="inlineStr"/>
       <c r="J14" s="57" t="inlineStr">
         <is>
-          <t>Zuerst eigene Export-SQL prüfen, erst danach den Standort fragen. Präzedenzfall UK, belegt am 02.09.2026: die Lieferantenspalten waren in der UK-Datei seit jeher gefüllt (1881/1881) und nur nie gemappt</t>
+          <t>Eigene Export-SQL am 29.09. geprüft: DE und ES lesen keine Lieferantenspalte, Alphaplan führt die Lieferanten nachweislich. Nächster Schritt: read-only Spaltenauszug des Schemas bei Rohail (DE) und Santi (ES) anfordern, danach Query und Import erweitern. Kein Pflegeauftrag an die Standorte.</t>
         </is>
       </c>
       <c r="K14" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Record the railway overview for Rohail and what mail and Teams revealed
The group-wide railway revenue overview is plausibility-checked: German
railway customers match Rohail's invoice list, the site totals match
his list and the journal within about one percent, the top 15
proposals cover 70 % and are clearly railway, ITEC is a false positive
and the Spanish 2026 share stands out.

Searching mail and Teams for the first time surfaced items the docs did
not hold: Sonja's February wish list, the Rexx Hub order of 29.07.,
Andreas' journal scope of 10.09., the ZZPRDAT test of 17.09. and open
requests from Upgreat and Armin. Weekly todo rows 52 to 57 track them.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$58</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="L5" s="84" t="n"/>
       <c r="M5" s="90" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="48">
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="J10" s="98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="99" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -2482,16 +2482,16 @@
         </is>
       </c>
       <c r="J15" s="106" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K15" s="107" t="inlineStr">
         <is>
-          <t>Der Termin vom 08.09.2026 ist überschritten; Deutschland ist gelöst, die übrigen Standorte sind offen.</t>
+          <t>Umsatz-Gesamtsicht über alle Standorte am 29.09.2026 geliefert und plausibilisiert; bestätigt sind erst DE und ein Kunde in Indien.</t>
         </is>
       </c>
       <c r="L15" s="107" t="inlineStr">
         <is>
-          <t>Neues Zieldatum mit Rohail Munir vereinbaren.</t>
+          <t>Top 15 Vorschläge und Schweiz mit Andreas und Patrik bestätigen.</t>
         </is>
       </c>
       <c r="M15" s="107" t="inlineStr">
@@ -2547,7 +2547,7 @@
         </is>
       </c>
       <c r="J16" s="98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="99" t="inlineStr">
         <is>
@@ -2630,7 +2630,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="68" customHeight="1" s="48">
+    <row r="18" ht="53" customHeight="1" s="48">
       <c r="A18" s="92" t="inlineStr">
         <is>
           <t>PM-11</t>
@@ -2651,9 +2651,9 @@
           <t>●  Neu</t>
         </is>
       </c>
-      <c r="E18" s="96" t="inlineStr">
-        <is>
-          <t>⚠ festlegen</t>
+      <c r="E18" s="108" t="inlineStr">
+        <is>
+          <t>Vorschlag: Andreas Stoller</t>
         </is>
       </c>
       <c r="F18" s="96" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="K18" s="99" t="inlineStr">
         <is>
-          <t>Neu aufgenommen am 29.09.2026 als Kleinauftrag «Analyse und Messung»; die Abgrenzung zu PM-09 (Tempo der Webapp, am 28.09.2026 weitgehend erledigt) ist zu klären.</t>
+          <t>Andreas hat am 28.09.2026 um eine Abstimmung zum Data Lake gebeten; Abgrenzung zu PM-09 (Tempo der Webapp) klären.</t>
         </is>
       </c>
       <c r="L18" s="99" t="inlineStr">
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -6276,15 +6276,15 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H49" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H49" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="I49" s="57" t="inlineStr"/>
       <c r="J49" s="57" t="inlineStr">
         <is>
-          <t>Antwort per Teams geben (Umsatz technisch für alle Standorte da, belastbar nur DE); Patrik die 171 Vorschläge außerhalb DE bestätigen lassen; mit Andreas und Rohail festlegen, was DB4 enthält, danach Export-SQL um vorhandene Quellfelder erweitern.</t>
+          <t>Umsatz-Gesamtsicht am 29.09. erstellt und plausibilisiert (Railway_Umsatz_Gesamtsicht_2026-09-29.xlsx), Teams-Text an Rohail liegt vor. Offen: Top 15 bestätigen, Schweiz über Andreas’ AG-Sicht, DB4-Definition.</t>
         </is>
       </c>
       <c r="K49" s="57" t="inlineStr"/>
@@ -6488,8 +6488,362 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="57" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C53" s="57" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="D53" s="57" t="inlineStr">
+        <is>
+          <t>ISS-019</t>
+        </is>
+      </c>
+      <c r="E53" s="57" t="inlineStr">
+        <is>
+          <t>Railway: Top 15 Vorschläge und Schweiz mit Andreas bestätigen, ITEC verwerfen</t>
+        </is>
+      </c>
+      <c r="F53" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Andreas / Patrik</t>
+        </is>
+      </c>
+      <c r="G53" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H53" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I53" s="57" t="inlineStr"/>
+      <c r="J53" s="57" t="inlineStr">
+        <is>
+          <t>Top 15 = 70 % des vorgeschlagenen Umsatzes; Schweiz über Andreas’ AG-Railway-Sicht; ITEC S.R.L. (Lohnfertiger TR IT) in /marktsegmente verwerfen; danach bereinigte Übersicht an Rohail.</t>
+        </is>
+      </c>
+      <c r="K53" s="57" t="inlineStr"/>
+      <c r="L53" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M53" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="57" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C54" s="57" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="D54" s="57" t="inlineStr">
+        <is>
+          <t>ISS-019</t>
+        </is>
+      </c>
+      <c r="E54" s="57" t="inlineStr">
+        <is>
+          <t>Spanien 2026: Railway-Anteil 30 % (CAF, Barat) beim Standort plausibilisieren</t>
+        </is>
+      </c>
+      <c r="F54" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Santi</t>
+        </is>
+      </c>
+      <c r="G54" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H54" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I54" s="57" t="inlineStr"/>
+      <c r="J54" s="57" t="inlineStr">
+        <is>
+          <t>913 TEUR 2026 gegen 387 TEUR 2025, fast alles CAF und Barat; kurz nachfragen, ob Projektgeschäft.</t>
+        </is>
+      </c>
+      <c r="K54" s="57" t="inlineStr"/>
+      <c r="L54" s="57" t="inlineStr">
+        <is>
+          <t>PM-08</t>
+        </is>
+      </c>
+      <c r="M54" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="57" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C55" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D55" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E55" s="57" t="inlineStr">
+        <is>
+          <t>Mail an Sonja ergänzen (Punkt 2 fehlt) und senden, offene Wünsche ansprechen</t>
+        </is>
+      </c>
+      <c r="F55" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G55" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H55" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I55" s="57" t="inlineStr"/>
+      <c r="J55" s="57" t="inlineStr">
+        <is>
+          <t>Entwurf liegt in Outlook; Punkt 2 (aktuelle Exporte) fehlt. Dabei die offenen Wünsche vom 03.02. (Ferien am Stück, Fit-&amp;-Wohl, Übertrag Restferien) und die Reihenfolge klären.</t>
+        </is>
+      </c>
+      <c r="K55" s="57" t="inlineStr"/>
+      <c r="L55" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M55" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="57" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B56" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C56" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D56" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E56" s="57" t="inlineStr">
+        <is>
+          <t>Rexx-Hub: Stand bei Rexx nachfragen</t>
+        </is>
+      </c>
+      <c r="F56" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Nadja</t>
+        </is>
+      </c>
+      <c r="G56" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H56" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf externe Firma</t>
+        </is>
+      </c>
+      <c r="I56" s="57" t="inlineStr"/>
+      <c r="J56" s="57" t="inlineStr">
+        <is>
+          <t>Nadja hat am 29.07.2026 den Rexx-Hub beauftragt (4’800 EUR p. a., Angebot Artjom Yahno). Stand der Einrichtung erfragen.</t>
+        </is>
+      </c>
+      <c r="K56" s="57" t="inlineStr"/>
+      <c r="L56" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M56" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C57" s="57" t="inlineStr">
+        <is>
+          <t>SAP ZZPRDAT</t>
+        </is>
+      </c>
+      <c r="D57" s="57" t="inlineStr">
+        <is>
+          <t>PM-03</t>
+        </is>
+      </c>
+      <c r="E57" s="57" t="inlineStr">
+        <is>
+          <t>ZZPRDAT: Ergebnis des Tests vom 17.09. mit Lucas festhalten</t>
+        </is>
+      </c>
+      <c r="F57" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G57" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H57" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I57" s="57" t="inlineStr"/>
+      <c r="J57" s="57" t="inlineStr">
+        <is>
+          <t>Lucas Castro hatte den Termin „Tests Produktionsdatum (Ingos Anpassung)“ angesetzt; Ergebnis ist nicht dokumentiert.</t>
+        </is>
+      </c>
+      <c r="K57" s="57" t="inlineStr"/>
+      <c r="L57" s="57" t="inlineStr">
+        <is>
+          <t>PM-03</t>
+        </is>
+      </c>
+      <c r="M57" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="57" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C58" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D58" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E58" s="57" t="inlineStr">
+        <is>
+          <t>Upgreat antworten: Webapp schneller?</t>
+        </is>
+      </c>
+      <c r="F58" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G58" s="57" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H58" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I58" s="57" t="inlineStr"/>
+      <c r="J58" s="57" t="inlineStr">
+        <is>
+          <t>Dardan (Upgreat) fragte am 23.09., ob die Datenabfrage schneller ist. Seit 28.09. deutlich schneller (Tempo-Deploys).</t>
+        </is>
+      </c>
+      <c r="K58" s="57" t="inlineStr"/>
+      <c r="L58" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M58" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M52"/>
+  <autoFilter ref="A1:M58"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Regenerate Wochen_Todo.xlsx with rows 65 to 70
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -1795,7 +1795,7 @@
     <row r="2" ht="20" customHeight="1" s="48">
       <c r="A2" s="74" t="inlineStr">
         <is>
-          <t>Stand 29.09.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
+          <t>Stand 30.09.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="J12" s="98" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K12" s="99" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="38" customHeight="1" s="48">
+    <row r="14" ht="53" customHeight="1" s="48">
       <c r="A14" s="92" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -2417,16 +2417,16 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
-          <t>Die fachlichen Wünsche sind umgesetzt; es fehlt die Exportschnittstelle der externen Firma.</t>
+          <t>Die fachlichen Wünsche sind umgesetzt; es fehlt der automatische Rexx-Export. Kein Rexx-Hub (30.09.), Umsetzung über Upgreat angefragt.</t>
         </is>
       </c>
       <c r="L14" s="99" t="inlineStr">
         <is>
-          <t>Termin der externen Firma einfordern.</t>
+          <t>Antwort Ueli Kunzmann (Upgreat) einholen, Pfad und Berechtigung klären.</t>
         </is>
       </c>
       <c r="M14" s="99" t="inlineStr">
@@ -3334,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -6688,12 +6688,12 @@
       </c>
       <c r="E56" s="57" t="inlineStr">
         <is>
-          <t>Rexx-Hub: Stand bei Rexx nachfragen</t>
+          <t>Rexx-Export ohne Hub über Upgreat</t>
         </is>
       </c>
       <c r="F56" s="57" t="inlineStr">
         <is>
-          <t>Ingo / Nadja</t>
+          <t>Ingo</t>
         </is>
       </c>
       <c r="G56" s="57" t="inlineStr">
@@ -6709,7 +6709,7 @@
       <c r="I56" s="57" t="inlineStr"/>
       <c r="J56" s="57" t="inlineStr">
         <is>
-          <t>Nadja hat am 29.07.2026 den Rexx-Hub beauftragt (4’800 EUR p. a., Angebot Artjom Yahno). Stand der Einrichtung erfragen.</t>
+          <t>Kein Rexx-Hub (Ingo 30.09.). Mail an Ueli Kunzmann (Upgreat) am 30.09. versendet: vier Rexx-Berichte täglich in den HR-Datenordner. Antwort abwarten, Pfad und Berechtigung klären; mit Nadja klären, ob der Hub-Auftrag bei Rexx zurückgenommen wird.</t>
         </is>
       </c>
       <c r="K56" s="57" t="inlineStr"/>
@@ -6842,8 +6842,783 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="57" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C59" s="57" t="inlineStr">
+        <is>
+          <t>Finance IT</t>
+        </is>
+      </c>
+      <c r="D59" s="57" t="inlineStr">
+        <is>
+          <t>ISS-021</t>
+        </is>
+      </c>
+      <c r="E59" s="57" t="inlineStr">
+        <is>
+          <t>Italien: Doppelzeilen (Lieferantenadresse) und provisorischer Kundenausschluss hoben sich auf; beides behoben</t>
+        </is>
+      </c>
+      <c r="F59" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Andreas</t>
+        </is>
+      </c>
+      <c r="G59" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H59" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I59" s="57" t="inlineStr"/>
+      <c r="J59" s="57" t="inlineStr">
+        <is>
+          <t>Nachgewiesen 30.09.: Italien 2025 7,70 Mio. EUR, 0,36 % über Rhino; keine Doppelzeilen mehr. Andreas informieren.</t>
+        </is>
+      </c>
+      <c r="K59" s="57" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="L59" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M59" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="57" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C60" s="57" t="inlineStr">
+        <is>
+          <t>Finance CH</t>
+        </is>
+      </c>
+      <c r="D60" s="57" t="inlineStr">
+        <is>
+          <t>ISS-022</t>
+        </is>
+      </c>
+      <c r="E60" s="57" t="inlineStr">
+        <is>
+          <t>Proforma F5/F8 im Schweizer Umsatz: 2025 1,91 Mio., 2026 5,97 Mio. CHF</t>
+        </is>
+      </c>
+      <c r="F60" s="57" t="inlineStr">
+        <is>
+          <t>Andreas / Ingo</t>
+        </is>
+      </c>
+      <c r="G60" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H60" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf Entscheid</t>
+        </is>
+      </c>
+      <c r="I60" s="57" t="inlineStr"/>
+      <c r="J60" s="57" t="inlineStr">
+        <is>
+          <t>Andreas entscheiden lassen, ob F5/F8 in Net Sales gehören; danach Regel je Belegart.</t>
+        </is>
+      </c>
+      <c r="K60" s="57" t="inlineStr"/>
+      <c r="L60" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M60" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="57" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid</t>
+        </is>
+      </c>
+      <c r="C61" s="57" t="inlineStr">
+        <is>
+          <t>Finance Sollwerte</t>
+        </is>
+      </c>
+      <c r="D61" s="57" t="inlineStr">
+        <is>
+          <t>ISS-024</t>
+        </is>
+      </c>
+      <c r="E61" s="57" t="inlineStr">
+        <is>
+          <t>Kein Sollwert für CH (auch CN, RU), dazu fehlen alle Sollwerte 2026 (ISS-023)</t>
+        </is>
+      </c>
+      <c r="F61" s="57" t="inlineStr">
+        <is>
+          <t>Andreas</t>
+        </is>
+      </c>
+      <c r="G61" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H61" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf Daten</t>
+        </is>
+      </c>
+      <c r="I61" s="57" t="inlineStr"/>
+      <c r="J61" s="57" t="inlineStr">
+        <is>
+          <t>Sollwerte CH und 2026 bei Andreas anfordern.</t>
+        </is>
+      </c>
+      <c r="K61" s="57" t="inlineStr"/>
+      <c r="L61" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M61" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="57" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C62" s="57" t="inlineStr">
+        <is>
+          <t>Standortdaten DE</t>
+        </is>
+      </c>
+      <c r="D62" s="57" t="inlineStr">
+        <is>
+          <t>ISS-029</t>
+        </is>
+      </c>
+      <c r="E62" s="57" t="inlineStr">
+        <is>
+          <t>Deutschland endet am 23.09.2026, September erst 125 Zeilen</t>
+        </is>
+      </c>
+      <c r="F62" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G62" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H62" s="57" t="inlineStr">
+        <is>
+          <t>Wartet auf DE</t>
+        </is>
+      </c>
+      <c r="I62" s="57" t="inlineStr"/>
+      <c r="J62" s="57" t="inlineStr">
+        <is>
+          <t>Import in Ordnung; Alphaplan-Delta seit 24.09. fast leer (2-3 KB statt 12-15 KB). Rohail/IT DE fragen.</t>
+        </is>
+      </c>
+      <c r="K62" s="57" t="inlineStr"/>
+      <c r="L62" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M62" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="57" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C63" s="57" t="inlineStr">
+        <is>
+          <t>Standortdaten IN</t>
+        </is>
+      </c>
+      <c r="D63" s="57" t="inlineStr">
+        <is>
+          <t>ISS-030</t>
+        </is>
+      </c>
+      <c r="E63" s="57" t="inlineStr">
+        <is>
+          <t>Indien liefert 17 Positionen mehrfach (andere Ursache als Italien)</t>
+        </is>
+      </c>
+      <c r="F63" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G63" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H63" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I63" s="57" t="inlineStr"/>
+      <c r="J63" s="57" t="inlineStr">
+        <is>
+          <t>Gleiche Ursache wie ISS-021 (zwei IN-Adressen je Lieferant), mit 15:02 behoben; nach Export 30.09. nachmessen.</t>
+        </is>
+      </c>
+      <c r="K63" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+      <c r="L63" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M63" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="57" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C64" s="57" t="inlineStr">
+        <is>
+          <t>Finance Technik</t>
+        </is>
+      </c>
+      <c r="D64" s="57" t="inlineStr">
+        <is>
+          <t>ISS-026/027</t>
+        </is>
+      </c>
+      <c r="E64" s="57" t="inlineStr">
+        <is>
+          <t>Kleinfixes: Gutschriften nach Belegart erkennen, OK-Text in der Excel-Formel als Konstante</t>
+        </is>
+      </c>
+      <c r="F64" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G64" s="57" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H64" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I64" s="57" t="inlineStr"/>
+      <c r="J64" s="57" t="inlineStr">
+        <is>
+          <t>Produktiv 29.09.2026 15:58 (b699fa5).</t>
+        </is>
+      </c>
+      <c r="K64" s="57" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+      <c r="L64" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M64" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="57" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C65" s="57" t="inlineStr">
+        <is>
+          <t>Finance Abnahme</t>
+        </is>
+      </c>
+      <c r="D65" s="57" t="inlineStr">
+        <is>
+          <t>ISS-028</t>
+        </is>
+      </c>
+      <c r="E65" s="57" t="inlineStr">
+        <is>
+          <t>Sichtprüfung Cockpit angemeldet, auch Dunkelmodus</t>
+        </is>
+      </c>
+      <c r="F65" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G65" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H65" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I65" s="57" t="inlineStr"/>
+      <c r="J65" s="57" t="inlineStr">
+        <is>
+          <t>Management-Cockpit und Finance-Vergleich durchsehen.</t>
+        </is>
+      </c>
+      <c r="K65" s="57" t="inlineStr"/>
+      <c r="L65" s="57" t="inlineStr">
+        <is>
+          <t>PM-05</t>
+        </is>
+      </c>
+      <c r="M65" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="57" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C66" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D66" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E66" s="57" t="inlineStr">
+        <is>
+          <t>SAP-HR-Datei automatisch über HrKpiSet produktiv setzen</t>
+        </is>
+      </c>
+      <c r="F66" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G66" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H66" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I66" s="57" t="inlineStr"/>
+      <c r="J66" s="57" t="inlineStr">
+        <is>
+          <t>In T76 gebaut und geprüft (4051506, HR_KPI.md 8.6). Offen: Wertestichprobe per Screenshot Gateway Client, Transport T76K912530 nach P76 (gemeinsam mit dem Journal), Deploy Cockpit (zusammen mit Ampel-Fix 81140fa).</t>
+        </is>
+      </c>
+      <c r="K66" s="57" t="inlineStr"/>
+      <c r="L66" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M66" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="57" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C67" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D67" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E67" s="57" t="inlineStr">
+        <is>
+          <t>Kaderkennzeichen für 8,1-h-Arbeitstag klären</t>
+        </is>
+      </c>
+      <c r="F67" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Sonja</t>
+        </is>
+      </c>
+      <c r="G67" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H67" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I67" s="57" t="inlineStr"/>
+      <c r="J67" s="57" t="inlineStr">
+        <is>
+          <t>HR 30.09.: Kader 8,1 h, normale 8,0 h. Kein Kaderfeld in den Dateien; Kandidaten SAP-Mitarbeiterkreis oder Rexx Leitung j/n (HR_KPI.md 8.5).</t>
+        </is>
+      </c>
+      <c r="K67" s="57" t="inlineStr"/>
+      <c r="L67" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M67" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="57" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B68" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C68" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D68" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E68" s="57" t="inlineStr">
+        <is>
+          <t>Abwesenheitsliste je Fall (Von/Bis/Status) aus Rexx</t>
+        </is>
+      </c>
+      <c r="F68" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Sonja</t>
+        </is>
+      </c>
+      <c r="G68" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H68" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I68" s="57" t="inlineStr"/>
+      <c r="J68" s="57" t="inlineStr">
+        <is>
+          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau.</t>
+        </is>
+      </c>
+      <c r="K68" s="57" t="inlineStr"/>
+      <c r="L68" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M68" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="57" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B69" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C69" s="57" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D69" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="E69" s="57" t="inlineStr">
+        <is>
+          <t>Arbeitstag 8,0 h statt 8,4 h</t>
+        </is>
+      </c>
+      <c r="F69" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G69" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H69" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I69" s="57" t="inlineStr"/>
+      <c r="J69" s="57" t="inlineStr">
+        <is>
+          <t>Produktiv 30.09.2026 09:36 (e3545c4). Mail an Sonja als .eml vorbereitet.</t>
+        </is>
+      </c>
+      <c r="K69" s="57" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="L69" s="57" t="inlineStr">
+        <is>
+          <t>PM-07</t>
+        </is>
+      </c>
+      <c r="M69" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="57" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B70" s="57" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C70" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D70" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E70" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf beim Auffrischen schneller (Rückmeldung Armin)</t>
+        </is>
+      </c>
+      <c r="F70" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G70" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H70" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I70" s="57" t="inlineStr"/>
+      <c r="J70" s="57" t="inlineStr">
+        <is>
+          <t>Entscheid: nach Delta alten Stand weiter zeigen oder 55 Abfragen bündeln (PLATTFORM_TEMPO 10).</t>
+        </is>
+      </c>
+      <c r="K70" s="57" t="inlineStr"/>
+      <c r="L70" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M70" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="57" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B71" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C71" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D71" s="57" t="inlineStr"/>
+      <c r="E71" s="57" t="inlineStr">
+        <is>
+          <t>Konditionsart ZRL2 Mengenrabatt EkOrg 1200 nach P76</t>
+        </is>
+      </c>
+      <c r="F71" s="57" t="inlineStr">
+        <is>
+          <t>Ingo / Fabio</t>
+        </is>
+      </c>
+      <c r="G71" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H71" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I71" s="57" t="inlineStr"/>
+      <c r="J71" s="57" t="inlineStr">
+        <is>
+          <t>T76K912628 importiert 30.09. nach Freigabe Lucas; Stammdaten pflegt Fabio im Live (SAP_ZRL2_MENGENRABATT_AT_2026-09-30.md).</t>
+        </is>
+      </c>
+      <c r="K71" s="57" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="L71" s="57" t="inlineStr"/>
+      <c r="M71" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M58"/>
+  <autoFilter ref="A1:M71"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Record Kader 8.1 h via Rexx Leitung j/n and close Wochen_Todo 66
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -1795,7 +1795,7 @@
     <row r="2" ht="20" customHeight="1" s="48">
       <c r="A2" s="74" t="inlineStr">
         <is>
-          <t>Stand 30.09.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
+          <t>Stand 01.10.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -7362,18 +7362,22 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H67" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H67" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I67" s="57" t="inlineStr"/>
       <c r="J67" s="57" t="inlineStr">
         <is>
-          <t>HR 30.09.: Kader 8,1 h, normale 8,0 h. Kein Kaderfeld in den Dateien; Kandidaten SAP-Mitarbeiterkreis oder Rexx Leitung j/n (HR_KPI.md 8.5).</t>
-        </is>
-      </c>
-      <c r="K67" s="57" t="inlineStr"/>
+          <t>Kader = Rexx Leitung j/n = ja (Ingo 01.10.). c51445c: 8,1 h statt 8,0 h für Krankheitstage, Langzeitgrenze, FTE. Deploy offen, zusammen mit 4051506/81140fa.</t>
+        </is>
+      </c>
+      <c r="K67" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="L67" s="57" t="inlineStr">
         <is>
           <t>PM-07</t>

</xml_diff>

<commit_message>
Record DB4 timing question, Rexx Zeitraum measurement and Kader deploy scope
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -6284,7 +6284,7 @@
       <c r="I49" s="57" t="inlineStr"/>
       <c r="J49" s="57" t="inlineStr">
         <is>
-          <t>Umsatz-Gesamtsicht am 29.09. erstellt und plausibilisiert (Railway_Umsatz_Gesamtsicht_2026-09-29.xlsx), Teams-Text an Rohail liegt vor. Offen: Top 15 bestätigen, Schweiz über Andreas’ AG-Sicht, DB4-Definition.</t>
+          <t>Umsatz-Gesamtsicht am 29.09. erstellt und plausibilisiert (Railway_Umsatz_Gesamtsicht_2026-09-29.xlsx), Teams-Text an Rohail liegt vor. Offen: Top 15 bestätigen, Schweiz über Andreas’ AG-Sicht, DB4-Definition. NACHTRAG 01.10.: Rückfrage, bis wann DB4 kommt (für Heiko), und Korrekturanfrage Patrick „Account designation Marketsegment SAP.xlsx“ (Datei noch nicht gesehen, Zusammenhang offen). Ingos Schätzung ca. 2 Wochen gilt nur für die Zusatzfelder an den Standorten; vorher DB4-Definition mit Andreas und Rohail, erst dann Termin.</t>
         </is>
       </c>
       <c r="K49" s="57" t="inlineStr"/>
@@ -7311,7 +7311,7 @@
       <c r="I66" s="57" t="inlineStr"/>
       <c r="J66" s="57" t="inlineStr">
         <is>
-          <t>In T76 gebaut und geprüft (4051506, HR_KPI.md 8.6). Offen: Wertestichprobe per Screenshot Gateway Client, Transport T76K912530 nach P76 (gemeinsam mit dem Journal), Deploy Cockpit (zusammen mit Ampel-Fix 81140fa).</t>
+          <t>In T76 gebaut und geprüft (4051506, HR_KPI.md 8.6). Offen: Wertestichprobe per Screenshot Gateway Client, Transport T76K912530 nach P76 (gemeinsam mit dem Journal), Deploy Cockpit (zusammen mit Ampel-Fix 81140fa und Kader 8,1 h c51445c).</t>
         </is>
       </c>
       <c r="K66" s="57" t="inlineStr"/>
@@ -7433,7 +7433,7 @@
       <c r="I68" s="57" t="inlineStr"/>
       <c r="J68" s="57" t="inlineStr">
         <is>
-          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau.</t>
+          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau. Gemessen 01.10. an #744 (Stand 26.05.): (Zeitraum)-Spalten nennen je Person nur den letzten Fall, bei 63 von 113 Personen mit Stunden gibt es mehr Stunden als der Zeitraum; #744 hat keine Ferienspalte. Weitere Spalten im Personenbericht lösen das nicht, nötig ist die Liste je Fall (HR_KPI.md 8.5).</t>
         </is>
       </c>
       <c r="K68" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Record the 09:12 deploy of HrKpiSet import, absence traffic light and Kader hours
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -7311,7 +7311,7 @@
       <c r="I66" s="57" t="inlineStr"/>
       <c r="J66" s="57" t="inlineStr">
         <is>
-          <t>In T76 gebaut und geprüft (4051506, HR_KPI.md 8.6). Offen: Wertestichprobe per Screenshot Gateway Client, Transport T76K912530 nach P76 (gemeinsam mit dem Journal), Deploy Cockpit (zusammen mit Ampel-Fix 81140fa und Kader 8,1 h c51445c).</t>
+          <t>Cockpit produktiv seit 01.10. 09:12 (ba9cf5c, mit Ampel 81140fa und Kader c51445c). Offen: Wertestichprobe per Screenshot Gateway Client, Transport T76K912530 nach P76 (gemeinsam mit dem Journal); bis dahin lässt der Tagesabruf die Handdatei stehen.</t>
         </is>
       </c>
       <c r="K66" s="57" t="inlineStr"/>
@@ -7370,7 +7370,7 @@
       <c r="I67" s="57" t="inlineStr"/>
       <c r="J67" s="57" t="inlineStr">
         <is>
-          <t>Kader = Rexx Leitung j/n = ja (Ingo 01.10.). c51445c: 8,1 h statt 8,0 h für Krankheitstage, Langzeitgrenze, FTE. Deploy offen, zusammen mit 4051506/81140fa.</t>
+          <t>Kader = Rexx Leitung j/n = ja (Ingo 01.10.). c51445c: 8,1 h statt 8,0 h für Krankheitstage, Langzeitgrenze, FTE. Produktiv seit 01.10. 09:12.</t>
         </is>
       </c>
       <c r="K67" s="57" t="inlineStr">

</xml_diff>

<commit_message>
Record the 09:44 deploy, the first HrKpiSet import and absences per case in PA2001
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -7303,18 +7303,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H66" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H66" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I66" s="57" t="inlineStr"/>
       <c r="J66" s="57" t="inlineStr">
         <is>
-          <t>Cockpit produktiv seit 01.10. 09:12, Transport T76K912530 am 01.10. in P76, HrKpiSet dort 200 (Gateway Client). Erster echter Abruf am 02.10. ab 05:00. Wertestichprobe 01.10. bestanden (3 Personen, alle Felder gleich wie Handdatei). Offen: Kontrolle der Datei am 02.10.. Entschieden 01.10.: laufender Monat bleibt (Stammdaten zum Stichtag); Unfalltage-Kachel beschriften oder BU/NBU ab Jahresbeginn liefern ist Vorschlag.</t>
-        </is>
-      </c>
-      <c r="K66" s="57" t="inlineStr"/>
+          <t>Produktiv: Transport T76K912530 in P76, Wertestichprobe bestanden, erster Abruf 01.10. 09:46 mit 1'168 Personen, danach täglich ab 05:00. Laufender Monat bleibt (Entscheid 01.10.), Unfalltage-Kacheln entsprechend beschriftet (931f151).</t>
+        </is>
+      </c>
+      <c r="K66" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="L66" s="57" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -7433,7 +7437,7 @@
       <c r="I68" s="57" t="inlineStr"/>
       <c r="J68" s="57" t="inlineStr">
         <is>
-          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau. Gemessen 01.10. an #744 (Stand 26.05.): (Zeitraum)-Spalten nennen je Person nur den letzten Fall, bei 63 von 113 Personen mit Stunden gibt es mehr Stunden als der Zeitraum; #744 hat keine Ferienspalte. Weitere Spalten im Personenbericht lösen das nicht, nötig ist die Liste je Fall (HR_KPI.md 8.5).</t>
+          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau. Gemessen 01.10. an #744 (Stand 26.05.): (Zeitraum)-Spalten nennen je Person nur den letzten Fall, bei 63 von 113 Personen mit Stunden gibt es mehr Stunden als der Zeitraum; #744 hat keine Ferienspalte. Weitere Spalten im Personenbericht lösen das nicht, nötig ist die Liste je Fall (HR_KPI.md 8.5). NEU 01.10.: SAP PA2001 hat Absenzen je Fall (Krankheit 0260/0270, Ferien 0100, Kompensation, Unfall) mit Von/Bis (T76 gemessen, HR_KPI.md 8.7). Erst in P76 Aktualität prüfen; dann HrAbsenzSet statt Rexx-Liste.</t>
         </is>
       </c>
       <c r="K68" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Record HrAbsenzSet in T76, transport T76K912644 and the cockpit switch to SAP absences
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -7416,12 +7416,12 @@
       </c>
       <c r="E68" s="57" t="inlineStr">
         <is>
-          <t>Abwesenheitsliste je Fall (Von/Bis/Status) aus Rexx</t>
+          <t>Abwesenheiten je Fall aus SAP PA2001 (HrAbsenzSet) statt Rexx-Liste</t>
         </is>
       </c>
       <c r="F68" s="57" t="inlineStr">
         <is>
-          <t>Ingo / Sonja</t>
+          <t>Ingo</t>
         </is>
       </c>
       <c r="G68" s="57" t="inlineStr">
@@ -7429,15 +7429,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H68" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H68" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="I68" s="57" t="inlineStr"/>
       <c r="J68" s="57" t="inlineStr">
         <is>
-          <t>Beispieldatei von Sonja holen, dann Leser bauen und als fünfte Datei bei Ueli (Upgreat) anfragen. Macht die Krankenquote periodengenau. Gemessen 01.10. an #744 (Stand 26.05.): (Zeitraum)-Spalten nennen je Person nur den letzten Fall, bei 63 von 113 Personen mit Stunden gibt es mehr Stunden als der Zeitraum; #744 hat keine Ferienspalte. Weitere Spalten im Personenbericht lösen das nicht, nötig ist die Liste je Fall (HR_KPI.md 8.5). NEU 01.10.: SAP PA2001 hat Absenzen je Fall (Krankheit 0260/0270, Ferien 0100, Kompensation, Unfall) mit Von/Bis (T76 gemessen, HR_KPI.md 8.7). Erst in P76 Aktualität prüfen; dann HrAbsenzSet statt Rexx-Liste.</t>
+          <t>Gebaut 01.10.: HrAbsenzSet in T76 (Transport T76K912644), Cockpit c749d32 nimmt Krankheit je Fall und Ferien/Kompensation/Militär aus SAP, sonst Rexx. Offen: Transport nach P76, Deploy, HR bestätigt Krankheitsarten (0210 Arzt? 0220–0270).</t>
         </is>
       </c>
       <c r="K68" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Record the HrAbsenzSet import in P76, the 10:50 deploy and the first SAP absence fetch
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -7429,18 +7429,22 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H68" s="59" t="inlineStr">
-        <is>
-          <t>Läuft</t>
+      <c r="H68" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I68" s="57" t="inlineStr"/>
       <c r="J68" s="57" t="inlineStr">
         <is>
-          <t>Gebaut 01.10.: HrAbsenzSet in T76 (Transport T76K912644), Cockpit c749d32 nimmt Krankheit je Fall und Ferien/Kompensation/Militär aus SAP, sonst Rexx. Offen: Transport nach P76, Deploy, HR bestätigt Krankheitsarten (0210 Arzt? 0220–0270).</t>
-        </is>
-      </c>
-      <c r="K68" s="57" t="inlineStr"/>
+          <t>Produktiv seit 01.10. 10:50: HrAbsenzSet in P76 (T76K912644), erster Abruf 4'948 Fälle 2025/2026. Krankenquote je Fall auf den Zeitraum zugeschnitten (2025 ca. 3,1 %, 2026 ca. 2,8 %), Ferien/Kompensation/Militär im Zeitraum. Rest: HR bestätigt Krankheitsarten; Personenbasis wartet auf tägliche Rexx-Exporte (Zeile 55).</t>
+        </is>
+      </c>
+      <c r="K68" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="L68" s="57" t="inlineStr">
         <is>
           <t>PM-07</t>

</xml_diff>

<commit_message>
Close or update open items that needed no input and add the timestamp rule
Measured read-only: journal set in P76, stock value history running,
Germany still thin, B1/B2 case counts, ZZPRDAT test moved to 12.10.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J14" s="98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
@@ -4295,13 +4295,13 @@
       </c>
       <c r="H16" s="57" t="inlineStr">
         <is>
-          <t>Auf T76 erledigt, Transport offen</t>
+          <t>In P76, Ladelauf offen</t>
         </is>
       </c>
       <c r="I16" s="57" t="inlineStr"/>
       <c r="J16" s="57" t="inlineStr">
         <is>
-          <t>FinanzJournalSet auf T76/100 am 11.09.2026 gebaut, aktiviert und geprueft ($metadata und Datenabruf HTTP 200, Werte gegengelesen, bestehende Sets unveraendert). Produktiv erst nach Freigabe und Import des Transports nach P76 wirksam.</t>
+          <t>T76K912530 am 01.10. nach P76 importiert (mit HrKpiSet). P76: FinanzJournalSet mit Filter 200 in 0,9 s. Letzter Journal-Import vom 10.09. war am fehlenden Set gescheitert. Offen: Journal-Ladelauf CH/AT im Admin auslösen (Ingo), danach Werte prüfen.</t>
         </is>
       </c>
       <c r="K16" s="57" t="inlineStr"/>
@@ -4769,18 +4769,22 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H24" s="57" t="inlineStr">
-        <is>
-          <t>Teil umgesetzt, Nachweis offen</t>
+      <c r="H24" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I24" s="57" t="inlineStr"/>
       <c r="J24" s="57" t="inlineStr">
         <is>
-          <t>Verlauf je Woche produktiv seit 28.09.2026 (Wunsch Einkauf, von Marco bestätigt). Einkauf-Lauf fiel 10.-28.09. aus (IIS-Leerlauf), per Code abgesichert, IT-Einstellung als ISS-017 offen. Danach Armins Entscheid zu Disponent 004, MB5L-Abgleich und serverseitigen Einkauf-Lauf als Kettennachweis ausführen</t>
-        </is>
-      </c>
-      <c r="K24" s="57" t="inlineStr"/>
+          <t>Wochenverlauf läuft: Tagesstände 28., 29., 30.09. je 87 Disponenten, Bewertungskreis 1100 (11,30 / 11,21 / 11,23 Mio.), gemessen 01.10. in der Produktiv-DB.</t>
+        </is>
+      </c>
+      <c r="K24" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:34</t>
+        </is>
+      </c>
       <c r="L24" s="57" t="inlineStr">
         <is>
           <t>PM-04</t>
@@ -5741,9 +5745,9 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H40" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H40" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I40" s="57" t="inlineStr">
@@ -5753,10 +5757,14 @@
       </c>
       <c r="J40" s="57" t="inlineStr">
         <is>
-          <t>Mail-Entwurf an Sonja mit dem Umsetzungsstand liegt vor (28.09.), Versand durch Ingo. Rexx-Absenzdatei hat pro Person nur Summen, periodengenau nur mit auf den Zeitraum eingegrenztem Export. Dateien auf dem Server sind vom 08.07. (Rexx) und 26.05. (SAP), neue Exporte anfordern.</t>
-        </is>
-      </c>
-      <c r="K40" s="57" t="inlineStr"/>
+          <t>Periodengenau gelöst über SAP PA2001 (HrAbsenzSet, produktiv 01.10. 10:50, HR_KPI.md 8.7). Aktuelle Rexx-Exporte: Zeile 55 (Upgreat), Mail an Sonja: Zeile 54.</t>
+        </is>
+      </c>
+      <c r="K40" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:34</t>
+        </is>
+      </c>
       <c r="L40" s="57" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -6225,7 +6233,7 @@
       <c r="I48" s="57" t="inlineStr"/>
       <c r="J48" s="57" t="inlineStr">
         <is>
-          <t>Andreas entscheidet: Wertgutschriften mit Menge 0, Kosten kostenloser Ware, interner Lieferant ohne Konzernkosten soll offen bleiben statt OK. Vorher Fallzahlen in den Daten messen.</t>
+          <t>Fallzahlen 01.10. (Produktiv-DB, CentralSalesRecords ab 2025): B1 Menge 0 mit Wertgutschrift: 57 Zeilen, keine mit Stückkosten, derzeit ohne Wirkung. B2 kostenlose Ware (Umsatz 0, Menge und Kosten ≠ 0): an allen Standorten, grösster Teil CH 2025 1'843 Zeilen (297 TEUR + 225 TCHF Kosten), 2026 753 Zeilen; Details ISS-018.6. B3 nicht per SQL zählbar (Klassifizierung im Code). Andreas entscheidet.</t>
         </is>
       </c>
       <c r="K48" s="57" t="inlineStr"/>
@@ -6760,15 +6768,19 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H57" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="I57" s="57" t="inlineStr"/>
+      <c r="H57" s="57" t="inlineStr">
+        <is>
+          <t>Terminiert</t>
+        </is>
+      </c>
+      <c r="I57" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
       <c r="J57" s="57" t="inlineStr">
         <is>
-          <t>Lucas Castro hatte den Termin „Tests Produktionsdatum (Ingos Anpassung)“ angesetzt; Ergebnis ist nicht dokumentiert.</t>
+          <t>Test hat noch nicht stattgefunden: Lucas hat ihn auf 12.10.2026 16:00 gelegt (Marco, Adil, Ingo; Ingo hat am 01.10. zugesagt). Danach Ergebnis festhalten.</t>
         </is>
       </c>
       <c r="K57" s="57" t="inlineStr"/>
@@ -6819,15 +6831,15 @@
           <t>Niedrig</t>
         </is>
       </c>
-      <c r="H58" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H58" s="57" t="inlineStr">
+        <is>
+          <t>Entwurf liegt vor</t>
         </is>
       </c>
       <c r="I58" s="57" t="inlineStr"/>
       <c r="J58" s="57" t="inlineStr">
         <is>
-          <t>Dardan (Upgreat) fragte am 23.09., ob die Datenabfrage schneller ist. Seit 28.09. deutlich schneller (Tempo-Deploys).</t>
+          <t>Antwort als .eml in Downloads (Mail_Dardan_Upgreat_Tempo_Webapp_2026-10-01.eml), Empfänger eintragen und senden (Ingo).</t>
         </is>
       </c>
       <c r="K58" s="57" t="inlineStr"/>
@@ -7067,7 +7079,7 @@
       <c r="I62" s="57" t="inlineStr"/>
       <c r="J62" s="57" t="inlineStr">
         <is>
-          <t>Import in Ordnung; Alphaplan-Delta seit 24.09. fast leer (2-3 KB statt 12-15 KB). Rohail/IT DE fragen.</t>
+          <t>Import in Ordnung; Alphaplan-Delta seit 24.09. fast leer (2-3 KB statt 12-15 KB). Rohail/IT DE fragen. Nachgemessen 01.10.: weiter dünn, September 131 Zeilen, seit 24.09. nur 6, letzte Rechnung 29.09., Extraktion 30.09.</t>
         </is>
       </c>
       <c r="K62" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Bring the Wochen_Todo summary sheet up to date and fix rows 3 and 12
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -550,7 +550,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left>
         <color rgb="FF000000"/>
@@ -711,11 +711,27 @@
         <color rgb="FF000000"/>
       </diagonal>
     </border>
+    <border>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="002F5597"/>
+      </bottom>
+    </border>
+    <border>
+      <right>
+        <color rgb="FF000000"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="002E8B57"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="144">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1115,6 +1131,9 @@
     <xf numFmtId="0" fontId="39" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3015,12 +3034,12 @@
       </c>
       <c r="E2" s="51" t="inlineStr">
         <is>
-          <t>Fixes 10-18 fertig, aber Transaktion startet Z_ZLO03_TURBO2 statt der gepatchten Version.</t>
+          <t>Fixes 10-18 fertig; Diagnoselauf p_diag und Regressionstest stehen aus.</t>
         </is>
       </c>
       <c r="F2" s="51" t="inlineStr">
         <is>
-          <t>Diagnoselauf p_diag, danach Transport nach B76.</t>
+          <t>Diagnoselauf p_diag und Regressionstest, danach Transport nach B76; Ann-Katrin Michel vorwarnen (Spalte Exklusiv liefert auch "?").</t>
         </is>
       </c>
     </row>
@@ -3041,16 +3060,16 @@
         </is>
       </c>
       <c r="D3" s="53" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="E3" s="51" t="inlineStr">
         <is>
-          <t>Blockiert, Tracing ist tot (p_debug deaktiviert).</t>
+          <t>ZC12 = ZM_ABGLEICH_KTSCH geklaert; Entscheid 07.09.: Tracing scharf schalten. Geaenderte Fassung (p_debug aktiv) liegt bereit, in T76 noch nicht gesichert (Stand 01.10.).</t>
         </is>
       </c>
       <c r="F3" s="51" t="inlineStr">
         <is>
-          <t>Vorfrage in SE93: ist ZC12 = Z_ABGLEICH_KTSCH?</t>
+          <t>Fassung in T76 sichern und aktivieren (Ingo), dann Nullmengenfall mit p_debug tracen.</t>
         </is>
       </c>
     </row>
@@ -3071,16 +3090,16 @@
         </is>
       </c>
       <c r="D4" s="53" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="E4" s="51" t="inlineStr">
         <is>
-          <t>Root Cause geklaert, Umsetzung fachlich blockiert durch drei offene Klaerungen.</t>
+          <t>In T76 umgesetzt und getestet, Pruefbericht Z_ZZPRDAT_CHECK am 07.09. korrigiert; Abnahme offen.</t>
         </is>
       </c>
       <c r="F4" s="51" t="inlineStr">
         <is>
-          <t>Aenderungsbelege zu Auftrag 1214608 lesen.</t>
+          <t>Test mit Lucas, Marco und Adil am 12.10.2026 16:00; danach Abnahme und Transport nach P76.</t>
         </is>
       </c>
     </row>
@@ -3101,16 +3120,16 @@
         </is>
       </c>
       <c r="D5" s="53" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
-          <t>SAP-Direktanbindung produktiv seit 12.08.2026, Materialtext MAKTX seit 18.08.2026.</t>
+          <t>Produktiv. Seit 01.10.: Texte D1/D5 im Dashboard; nach "Delta aktualisieren" sofort alter Stand mit Hinweis.</t>
         </is>
       </c>
       <c r="F5" s="51" t="inlineStr">
         <is>
-          <t>D1/D5-Texte pflegen, SEGW-Key auf DISPO_KZ + DISPO korrigieren.</t>
+          <t>Entscheid SEGW-Key (Empfehlung: nicht umsetzen); spaeter Abfragen buendeln (Tempo, Variante b).</t>
         </is>
       </c>
     </row>
@@ -3135,12 +3154,12 @@
       </c>
       <c r="E6" s="51" t="inlineStr">
         <is>
-          <t>Produktiv; Detailarbeit laeuft im Finance-Issue-Log. ISS-003.4 ist als Option produktiv, Andreas entscheidet die Ausnahme.</t>
+          <t>Produktiv; Journal CH/AT seit 01.10. in P76, Ladelauf offen. Mehrere Fachentscheide liegen bei Andreas (ISS-018, ISS-022, ISS-024).</t>
         </is>
       </c>
       <c r="F6" s="51" t="inlineStr">
         <is>
-          <t>Ueber das Finance-Issue-Log weiterfuehren; CH/AT-Option mit Andreas entscheiden.</t>
+          <t>Journal-Ladelauf CH/AT ausloesen; Entscheide mit Andreas.</t>
         </is>
       </c>
     </row>
@@ -3191,16 +3210,16 @@
         </is>
       </c>
       <c r="D8" s="53" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E8" s="51" t="inlineStr">
         <is>
-          <t>Wartet auf die externe Firma; Schnittstelle und Zeitplan sind unbekannt.</t>
+          <t>HR-Cockpit produktiv; seit 01.10. taeglich aus SAP: HR-Felder (HrKpiSet) und Absenzen je Fall (HrAbsenzSet, Krankenquote periodengenau). Rexx-Dateien noch vom 08.07.</t>
         </is>
       </c>
       <c r="F8" s="51" t="inlineStr">
         <is>
-          <t>Fertigstellung des automatischen Exporters abwarten, danach Anbindung planen.</t>
+          <t>Upgreat: taegliche Rexx-Exporte; Sonja: Krankheitsarten bestaetigen, Mail senden.</t>
         </is>
       </c>
     </row>
@@ -3225,12 +3244,12 @@
       </c>
       <c r="E9" s="51" t="inlineStr">
         <is>
-          <t>99 gepflegte Bahnbranchen liegen vor; der App-Leser fuer die fachlichen Kundenfelder ist getestet. Der produktive Rohkopf liefert noch nur die interne Adress-ID.</t>
+          <t>DE-Bahnumsatz belegt (2025 rund 579 TEUR); Gesamtsicht aller Standorte am 29.09. erstellt; 171 Vorschlaege anderer Standorte offen.</t>
         </is>
       </c>
       <c r="F9" s="51" t="inlineStr">
         <is>
-          <t>Alphaplan-Kopfexport um AdressNummer-Kunde, Name, Land und Branche ergaenzen; danach TRDE neu laden und die 99 Nummern bestaetigt uebernehmen.</t>
+          <t>Top 15 mit Andreas und Patrik bestaetigen; DB4-Definition mit Andreas und Rohail, erst dann Termin.</t>
         </is>
       </c>
     </row>
@@ -3251,16 +3270,16 @@
         </is>
       </c>
       <c r="D10" s="53" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E10" s="51" t="inlineStr">
         <is>
-          <t>Produktiv persistent gespeichert; Kachel zeigt CHF 9'205'959 (Stand 24.08.2026).</t>
+          <t>Erledigt: Wochenverlauf produktiv, Tagesstaende seit 28.09. (rund 11,2 Mio. CHF, Bewertungskreis 1100).</t>
         </is>
       </c>
       <c r="F10" s="51" t="inlineStr">
         <is>
-          <t>MB5L-Abgleich und serverseitigen Einkauf-Lauf als Kettennachweis ausfuehren.</t>
+          <t>Keiner.</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3323,7 @@
     <row r="14">
       <c r="A14" s="55" t="inlineStr">
         <is>
-          <t>Quellen: projektmanagement/PROJEKTSTATUS.md (PM-01 bis PM-07), docs/AGENT_COORDINATION.md (aktuellerer Stand) und docs/Issue_Log_Konsolidiert_2026-08-12.tsv (Finance).</t>
+          <t>Quellen: projektmanagement/PROJEKTSTATUS.md, projektmanagement/Wochen_Todo.tsv, docs/Issue_Log_Konsolidiert_2026-08-12.tsv. Von Hand nachgefuehrt am 01.10.2026.</t>
         </is>
       </c>
     </row>
@@ -3585,7 +3604,7 @@
       <c r="I4" s="57" t="inlineStr"/>
       <c r="J4" s="57" t="inlineStr">
         <is>
-          <t>Vorfrage am 04.09.2026 beantwortet: ZC12 ist eine Reporttransaktion auf ZM_ABGLEICH_KTSCH; der Quelltext nennt sich selbst falsch Z_ABGLEICH_KTSCH. Version 3 vom 18.05.2026 ist der komplette Neuaufbau, laut eigener Kopfhistorie vom 28.-30.04.2026 durch I.Kohler; fmt_quan gehört dazu, also Testlücke statt Regression. Die Trace-Infrastruktur samt auskommentiertem p_debug hat KOI am 27.05.2026 eingebaut. Entscheid vom 07.09.2026: scharf schalten. Die geänderte Fassung liegt als saptasks/zc12/ZM_ABGLEICH_KTSCH_nachher.abap, ist aber NOCH NICHT im System - das Zurückschreiben hat der Berechtigungsfilter abgelehnt und muss von Hand abgesetzt werden. Danach den Nullmengenfall tracen; das Trace-Log landet auf dem Applikationsserver unter /tmp, nicht auf dem Arbeitsplatz.</t>
+          <t>Vorfrage am 04.09.2026 beantwortet: ZC12 ist eine Reporttransaktion auf ZM_ABGLEICH_KTSCH; der Quelltext nennt sich selbst falsch Z_ABGLEICH_KTSCH. Version 3 vom 18.05.2026 ist der komplette Neuaufbau, laut eigener Kopfhistorie vom 28.-30.04.2026 durch I.Kohler; fmt_quan gehört dazu, also Testlücke statt Regression. Die Trace-Infrastruktur samt auskommentiertem p_debug hat KOI am 27.05.2026 eingebaut. Entscheid vom 07.09.2026: scharf schalten. Die geänderte Fassung liegt als saptasks/zc12/ZM_ABGLEICH_KTSCH_nachher.abap, ist aber NOCH NICHT im System - das Zurückschreiben hat der Berechtigungsfilter abgelehnt und muss von Hand abgesetzt werden. Danach den Nullmengenfall tracen; das Trace-Log landet auf dem Applikationsserver unter /tmp, nicht auf dem Arbeitsplatz. Stand 01.10.: T76 hat weiter den vorher-Stand; der Versuch, die Fassung per Skript zu sichern, wurde erneut von der Freigabe-Sperre abgelehnt. Ingo sichert und aktiviert in SE38.</t>
         </is>
       </c>
       <c r="K4" s="57" t="inlineStr"/>
@@ -4124,7 +4143,7 @@
       <c r="I13" s="57" t="inlineStr"/>
       <c r="J13" s="57" t="inlineStr">
         <is>
-          <t>Anschreiben liegt als Outlook-Entwurf mit Betreff und angehängtem Lösungsdokument; vor dem Versand die Empfängeradressen eintragen und den Text aus docs/ZZPRDAT_Mail_Abnahme_2026-09-04.html hineinkopieren. Das Dokument hat seit 07.09.2026 die Kapitel 'So testen Sie es selbst' und 'Nachmessung vom 7. September'. Marco prüft Etikett und Typenschild und dabei neu auch den Zeitpunkt: der Verbuchungsbaustein läuft als V2 nach der Standardverbuchung, ein unmittelbarer Druck könnte das Feld noch leer sehen. Nicht behoben ist ausserdem, dass Z_ZZPRDAT_CHECK jeden abweichenden Wert als 'Write-once nachgewiesen' meldet.</t>
+          <t>Anschreiben liegt als Outlook-Entwurf mit Betreff und angehängtem Lösungsdokument; vor dem Versand die Empfängeradressen eintragen und den Text aus docs/ZZPRDAT_Mail_Abnahme_2026-09-04.html hineinkopieren. Das Dokument hat seit 07.09.2026 die Kapitel 'So testen Sie es selbst' und 'Nachmessung vom 7. September'. Marco prüft Etikett und Typenschild und dabei neu auch den Zeitpunkt: der Verbuchungsbaustein läuft als V2 nach der Standardverbuchung, ein unmittelbarer Druck könnte das Feld noch leer sehen. Z_ZZPRDAT_CHECK ist seit 07.09. korrigiert (nur Momentaufnahme, kein Write-once-Anspruch; zzprdat-kontext.md). Testtermin mit Lucas, Marco, Adil: 12.10.2026 16:00.</t>
         </is>
       </c>
       <c r="K13" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Update HERMES status for PM-03, PM-04, PM-07 and PM-09
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2164,12 +2164,12 @@
       </c>
       <c r="K10" s="99" t="inlineStr">
         <is>
-          <t>Die Lösung ist gebaut und im Testsystem vollständig geprüft; die Abnahmeanfrage ist vorbereitet, aber noch nicht versendet.</t>
+          <t>Die Lösung ist gebaut und im Testsystem vollständig geprüft; der gemeinsame Test mit Lucas, Marco und Adil ist auf den 12.10.2026 gelegt.</t>
         </is>
       </c>
       <c r="L10" s="99" t="inlineStr">
         <is>
-          <t>Abnahmeanfrage versenden.</t>
+          <t>Test am 12.10.2026 durchführen, danach Abnahme und Übernahme ins Produktivsystem.</t>
         </is>
       </c>
       <c r="M10" s="99" t="inlineStr">
@@ -2186,7 +2186,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="53" customHeight="1" s="48">
+    <row r="11" ht="68" customHeight="1" s="48">
       <c r="A11" s="100" t="inlineStr">
         <is>
           <t>PM-04</t>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
-          <t>Produktiv; zwei Nacharbeiten im SAP und drei Beschriftungen sind offen.</t>
+          <t>Produktiv; seit 01.10.2026 Texte D1/D5 im Dashboard und sofortige Anzeige nach dem Auffrischen. Offen sind nur ein SAP-Schlüssel (Empfehlung: nicht umsetzen) und drei Beschriftungen.</t>
         </is>
       </c>
       <c r="L11" s="107" t="inlineStr">
         <is>
-          <t>Nacharbeiten im SAP anstossen.</t>
+          <t>Entscheid zu SAP-Schlüssel und Beschriftungen, dann abschliessen.</t>
         </is>
       </c>
       <c r="M11" s="107" t="inlineStr">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="53" customHeight="1" s="48">
+    <row r="14" ht="68" customHeight="1" s="48">
       <c r="A14" s="92" t="inlineStr">
         <is>
           <t>PM-07</t>
@@ -2440,12 +2440,12 @@
       </c>
       <c r="K14" s="99" t="inlineStr">
         <is>
-          <t>Die fachlichen Wünsche sind umgesetzt; es fehlt der automatische Rexx-Export. Kein Rexx-Hub (30.09.), Umsetzung über Upgreat angefragt.</t>
+          <t>Seit 01.10.2026 holt das HR-Cockpit SAP-Daten und Abwesenheiten je Fall täglich selbst; die Krankenquote ist damit periodengenau. Es fehlt der tägliche Rexx-Export (Upgreat).</t>
         </is>
       </c>
       <c r="L14" s="99" t="inlineStr">
         <is>
-          <t>Antwort Ueli Kunzmann (Upgreat) einholen, Pfad und Berechtigung klären.</t>
+          <t>Antwort Ueli Kunzmann (Upgreat) einholen; HR bestätigt die Krankheitsarten.</t>
         </is>
       </c>
       <c r="M14" s="99" t="inlineStr">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1" s="48">
+    <row r="16" ht="68" customHeight="1" s="48">
       <c r="A16" s="92" t="inlineStr">
         <is>
           <t>PM-09</t>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="K16" s="99" t="inlineStr">
         <is>
-          <t>Weitgehend erledigt und produktiv; die Server-Einstellung durch die IT fehlt noch.</t>
+          <t>Weitgehend erledigt und produktiv; seit 01.10.2026 zeigt der Einkauf nach dem Auffrischen sofort den bisherigen Stand. Die Server-Einstellung durch die IT fehlt noch.</t>
         </is>
       </c>
       <c r="L16" s="99" t="inlineStr">

</xml_diff>

<commit_message>
Record Ingo's check of Logistik live and the decisions on ZC12 and the journal run
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -3604,7 +3604,7 @@
       <c r="I4" s="57" t="inlineStr"/>
       <c r="J4" s="57" t="inlineStr">
         <is>
-          <t>Vorfrage am 04.09.2026 beantwortet: ZC12 ist eine Reporttransaktion auf ZM_ABGLEICH_KTSCH; der Quelltext nennt sich selbst falsch Z_ABGLEICH_KTSCH. Version 3 vom 18.05.2026 ist der komplette Neuaufbau, laut eigener Kopfhistorie vom 28.-30.04.2026 durch I.Kohler; fmt_quan gehört dazu, also Testlücke statt Regression. Die Trace-Infrastruktur samt auskommentiertem p_debug hat KOI am 27.05.2026 eingebaut. Entscheid vom 07.09.2026: scharf schalten. Die geänderte Fassung liegt als saptasks/zc12/ZM_ABGLEICH_KTSCH_nachher.abap, ist aber NOCH NICHT im System - das Zurückschreiben hat der Berechtigungsfilter abgelehnt und muss von Hand abgesetzt werden. Danach den Nullmengenfall tracen; das Trace-Log landet auf dem Applikationsserver unter /tmp, nicht auf dem Arbeitsplatz. Stand 01.10.: T76 hat weiter den vorher-Stand; der Versuch, die Fassung per Skript zu sichern, wurde erneut von der Freigabe-Sperre abgelehnt. Ingo sichert und aktiviert in SE38.</t>
+          <t>Vorfrage am 04.09.2026 beantwortet: ZC12 ist eine Reporttransaktion auf ZM_ABGLEICH_KTSCH; der Quelltext nennt sich selbst falsch Z_ABGLEICH_KTSCH. Version 3 vom 18.05.2026 ist der komplette Neuaufbau, laut eigener Kopfhistorie vom 28.-30.04.2026 durch I.Kohler; fmt_quan gehört dazu, also Testlücke statt Regression. Die Trace-Infrastruktur samt auskommentiertem p_debug hat KOI am 27.05.2026 eingebaut. Entscheid vom 07.09.2026: scharf schalten. Die geänderte Fassung liegt als saptasks/zc12/ZM_ABGLEICH_KTSCH_nachher.abap, ist aber NOCH NICHT im System - das Zurückschreiben hat der Berechtigungsfilter abgelehnt und muss von Hand abgesetzt werden. Danach den Nullmengenfall tracen; das Trace-Log landet auf dem Applikationsserver unter /tmp, nicht auf dem Arbeitsplatz. Stand 01.10.: T76 hat weiter den vorher-Stand; der Versuch, die Fassung per Skript zu sichern, wurde erneut von der Freigabe-Sperre abgelehnt. Ingo sichert und aktiviert in SE38. Entscheid Ingo 2026-10-01 15:13: Editor in T76 so lassen, nichts tun.</t>
         </is>
       </c>
       <c r="K4" s="57" t="inlineStr"/>
@@ -4320,7 +4320,7 @@
       <c r="I16" s="57" t="inlineStr"/>
       <c r="J16" s="57" t="inlineStr">
         <is>
-          <t>T76K912530 am 01.10. nach P76 importiert (mit HrKpiSet). P76: FinanzJournalSet mit Filter 200 in 0,9 s. Letzter Journal-Import vom 10.09. war am fehlenden Set gescheitert. Offen: Journal-Ladelauf CH/AT im Admin auslösen (Ingo), danach Werte prüfen.</t>
+          <t>T76K912530 am 01.10. nach P76 importiert (mit HrKpiSet). P76: FinanzJournalSet mit Filter 200 in 0,9 s. Letzter Journal-Import vom 10.09. war am fehlenden Set gescheitert. Offen: Journal-Ladelauf CH/AT im Admin auslösen (Ingo), danach Werte prüfen. 2026-10-01 15:13: Ingo will den Lauf ausloesen lassen; geht nur ueber die Schaltflaeche auf /finance-journal-import (Chrome-Erweiterung nicht verbunden), Ingo klickt.</t>
         </is>
       </c>
       <c r="K16" s="57" t="inlineStr"/>
@@ -7708,7 +7708,7 @@
       <c r="I72" s="57" t="inlineStr"/>
       <c r="J72" s="57" t="inlineStr">
         <is>
-          <t>Produktiv seit 01.10. 15:01 (Transport T76K912650 in P76, Gateway Client P76 0,7 bis 2,0 s, Deploy 6b4bf21). Offen: Sichtprüfung Ingo, Werte gegen SAP prüfen.</t>
+          <t>Produktiv seit 01.10. 15:01, von Ingo gesichtet (2026-10-01 15:13: „sieht super aus“). Offen nur: einzelne Werte gegen SAP abgleichen.</t>
         </is>
       </c>
       <c r="K72" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Weltlage tab: radar per department, countries, commodities and currencies, events from GDELT, FRED, Eurostat and IMF with firewall state per source
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$77</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="J16" s="98" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K16" s="99" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M76"/>
+  <dimension ref="A1:M77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -7963,8 +7963,67 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="57" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B77" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C77" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D77" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E77" s="57" t="inlineStr">
+        <is>
+          <t>Reiter Weltlage (Radar je Abteilung, Länder, Rohstoffe und Währungen, Ereignisse) – erster Wurf</t>
+        </is>
+      </c>
+      <c r="F77" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G77" s="57" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H77" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I77" s="57" t="inlineStr"/>
+      <c r="J77" s="57" t="inlineStr">
+        <is>
+          <t>DEPLOYSTAND. Externe Quellen GDELT, FRED, Eurostat, IMF ohne Anmeldung, verknüpft mit Verkauf, Einkauf, Kursen; offen für alle. Offen: Firewall-Freigaben für die blockierten Quellen beantragen, Rechenregeln mit Ingo schärfen.</t>
+        </is>
+      </c>
+      <c r="K77" s="57" t="inlineStr"/>
+      <c r="L77" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M77" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M76"/>
+  <autoFilter ref="A1:M77"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Weltlage: currency change from the ECB 90-day reference rates instead of the sparse rate table, document production source states
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -7708,7 +7708,7 @@
       <c r="I72" s="57" t="inlineStr"/>
       <c r="J72" s="57" t="inlineStr">
         <is>
-          <t>Produktiv seit 01.10. 15:01, von Ingo gesichtet (2026-10-01 15:13: „sieht super aus“). Offen nur: einzelne Werte gegen SAP abgleichen. 05.10.: Umschalter 3D-Lagerplatzansicht (Paletten je Platz), DEPLOYSTAND.</t>
+          <t>Produktiv seit 01.10. 15:01, von Ingo gesichtet (2026-10-01 15:13: „sieht super aus“). Offen nur: einzelne Werte gegen SAP abgleichen. 05.10.: Umschalter 3D-Lagerplatzansicht (Paletten je Platz), produktiv 09:21 (98146c6).</t>
         </is>
       </c>
       <c r="K72" s="57" t="inlineStr"/>
@@ -8007,7 +8007,7 @@
       <c r="I77" s="57" t="inlineStr"/>
       <c r="J77" s="57" t="inlineStr">
         <is>
-          <t>DEPLOYSTAND. Externe Quellen GDELT, FRED, Eurostat, IMF ohne Anmeldung, verknüpft mit Verkauf, Einkauf, Kursen; offen für alle. Offen: Firewall-Freigaben für die blockierten Quellen beantragen, Rechenregeln mit Ingo schärfen.</t>
+          <t>Produktiv seit 05.10. 09:21 (e54190a). Vom Server: GDELT und Eurostat verbunden, FRED und IMF Firewall blockiert. Externe Quellen ohne Anmeldung, verknüpft mit Verkauf, Einkauf, Kursen; offen für alle. Offen: Firewall-Freigabe fred.stlouisfed.org und www.imf.org beantragen, Rechenregeln mit Ingo schärfen.</t>
         </is>
       </c>
       <c r="K77" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Sales_All Finance Details: standard cost, cost basis and margin in CHF with cost source, status and cost timing; meeting follow-ups in Wochen_Todo
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$83</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="J16" s="98" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K16" s="99" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -8144,8 +8144,244 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="57" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B80" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C80" s="57" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D80" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E80" s="57" t="inlineStr">
+        <is>
+          <t>Standardkosten, Kostenbasis und Marge in CHF im Blatt Finance Details (Sales_All)</t>
+        </is>
+      </c>
+      <c r="F80" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G80" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H80" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I80" s="57" t="inlineStr"/>
+      <c r="J80" s="57" t="inlineStr">
+        <is>
+          <t>Gebaut 06.10., Deploy offen; danach Andreas Bescheid geben (Spalten AH-AP, Cost Timing historisch/aktuell).</t>
+        </is>
+      </c>
+      <c r="K80" s="57" t="inlineStr"/>
+      <c r="L80" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M80" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="57" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B81" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C81" s="57" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D81" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E81" s="57" t="inlineStr">
+        <is>
+          <t>Prüfung Andreas: Umsatz gegen Konsolidierungstool, Standardkosten gegen Standortmargen, Abweichungen mit Rino und Kendra</t>
+        </is>
+      </c>
+      <c r="F81" s="57" t="inlineStr">
+        <is>
+          <t>Andreas</t>
+        </is>
+      </c>
+      <c r="G81" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H81" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I81" s="57" t="inlineStr"/>
+      <c r="J81" s="57" t="inlineStr">
+        <is>
+          <t>Nach Deploy der CHF-Spalten; Thermostat-Fall Indien→Italien→Deutschland (eine Stufe) mit Beispielen prüfen.</t>
+        </is>
+      </c>
+      <c r="K81" s="57" t="inlineStr"/>
+      <c r="L81" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M81" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="57" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B82" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C82" s="57" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D82" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E82" s="57" t="inlineStr">
+        <is>
+          <t>Vier-Augen-Prüfung der Summen durch Rino (unabhängig)</t>
+        </is>
+      </c>
+      <c r="F82" s="57" t="inlineStr">
+        <is>
+          <t>Rino</t>
+        </is>
+      </c>
+      <c r="G82" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H82" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I82" s="57" t="inlineStr"/>
+      <c r="J82" s="57" t="inlineStr">
+        <is>
+          <t>Andreas regelt das mit Rino (Gespräch 06.10.).</t>
+        </is>
+      </c>
+      <c r="K82" s="57" t="inlineStr"/>
+      <c r="L82" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M82" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="57" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B83" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C83" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D83" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="E83" s="57" t="inlineStr">
+        <is>
+          <t>Statement Weltlage-Radar an Andreas (Eigeninitiative, Ziel, Stand), er leitet ans Management weiter</t>
+        </is>
+      </c>
+      <c r="F83" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G83" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H83" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I83" s="57" t="inlineStr"/>
+      <c r="J83" s="57" t="inlineStr">
+        <is>
+          <t>Entwurf liegt im Chat vom 06.10.; Ingo sendet selbst.</t>
+        </is>
+      </c>
+      <c r="K83" s="57" t="inlineStr"/>
+      <c r="L83" s="57" t="inlineStr">
+        <is>
+          <t>PM-09</t>
+        </is>
+      </c>
+      <c r="M83" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M79"/>
+  <autoFilter ref="A1:M83"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
SAP T76: ZM_OFFENE_FAUF shows pegged requirements (MD_PEGGING_NODIALOG) as hideable fields, transport T76K912714; docs and SAP tooling
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$87</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -8557,8 +8557,67 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="57" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B87" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C87" s="57" t="inlineStr">
+        <is>
+          <t>Logistik</t>
+        </is>
+      </c>
+      <c r="D87" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E87" s="57" t="inlineStr">
+        <is>
+          <t>ZM_OFFENE_FAUF: Bedarfsverursacher (Dispoelement, Nummer, Daten zum Dispoelement) als einblendbare Felder</t>
+        </is>
+      </c>
+      <c r="F87" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G87" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H87" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I87" s="57" t="inlineStr"/>
+      <c r="J87" s="57" t="inlineStr">
+        <is>
+          <t>In T76 fertig und getestet (07.10.), Transport T76K912714. Ingo: in T76 ansehen, freigeben, nach P76 importieren; Bestellabruf klären; Z_PEG_TEST ($TMP) löschen?</t>
+        </is>
+      </c>
+      <c r="K87" s="57" t="inlineStr"/>
+      <c r="L87" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M87" s="122" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M86"/>
+  <autoFilter ref="A1:M87"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Deploy log 2026-10-08 06:39 Operations (Shopfloor)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -1814,7 +1814,7 @@
     <row r="2" ht="20" customHeight="1" s="48">
       <c r="A2" s="74" t="inlineStr">
         <is>
-          <t>Stand 07.10.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
+          <t>Stand 08.10.2026  ·  eine Zeile je Vorhaben  ·  Rollen mit «Vorschlag» sind aus der Dokumentation abgeleitet und noch nicht bestätigt</t>
         </is>
       </c>
     </row>
@@ -8660,7 +8660,7 @@
       <c r="I88" s="57" t="inlineStr"/>
       <c r="J88" s="57" t="inlineStr">
         <is>
-          <t>Committet 07.10., nur Ingo sichtbar. Deploy; T76K912718 freigeben/importieren, dann Caches leeren und Shopfloor:SapSyncEnabled=true; Freigabe durch Leitung Produktion/Operations einholen (vorher keine Ankündigung).</t>
+          <t>Produktiv 08.10. 06:39, nur Ingo sichtbar. T76K912718 freigeben/importieren, dann Caches leeren und Shopfloor:SapSyncEnabled=true; Freigabe durch Leitung Produktion/Operations einholen (vorher keine Ankündigung).</t>
         </is>
       </c>
       <c r="K88" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Einkauf (Armin 2026-10-08): open quantity-contract value like ME3L (EinkKontraktSet with EKAB call-offs, incl. expired) on Kontrakte and dashboard tile; Spend-Aufriss by lifecycle and assortment code (EinkMatLzSet); SAP T76 transports T76K912724 + T76K912718
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$91</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="J11" s="106" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M88"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -8675,8 +8675,173 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="57" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B89" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C89" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D89" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E89" s="57" t="inlineStr">
+        <is>
+          <t>Armin: offener Mengenkontraktwert (ME3L) auf Kontrakte und Dashboard; LZ-/Sortiments-Code im Spend-Aufriss</t>
+        </is>
+      </c>
+      <c r="F89" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G89" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H89" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I89" s="57" t="inlineStr"/>
+      <c r="J89" s="57" t="inlineStr">
+        <is>
+          <t>Cockpit committet 08.10.; T76K912724 dann T76K912718 nach P76, Caches leeren, Einkauf-Lauf, Wert gegen ME3L (16–17 Mio) mit Armin prüfen. Offen mit Armin: nur Bsart MK?</t>
+        </is>
+      </c>
+      <c r="K89" s="57" t="inlineStr"/>
+      <c r="L89" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M89" s="57" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="57" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="B90" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C90" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D90" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E90" s="57" t="inlineStr">
+        <is>
+          <t>Armin: Produktgruppe aus ZC23 im Spend-Aufriss (Disponent → Produktgruppe, Vererbung über ZLO03 auf Einkaufsteile)</t>
+        </is>
+      </c>
+      <c r="F90" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G90" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H90" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I90" s="57" t="inlineStr"/>
+      <c r="J90" s="57" t="inlineStr">
+        <is>
+          <t>Konzept: ZC23-Zuordnung Disponent→Produktgruppe, ZLO03-Auflösung verkürzte Nummern, Mehrfachnennung.</t>
+        </is>
+      </c>
+      <c r="K90" s="57" t="inlineStr"/>
+      <c r="L90" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M90" s="57" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="57" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B91" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C91" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D91" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="E91" s="57" t="inlineStr">
+        <is>
+          <t>Armin: Performance Report ZC23</t>
+        </is>
+      </c>
+      <c r="F91" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G91" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H91" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I91" s="57" t="inlineStr"/>
+      <c r="J91" s="57" t="inlineStr">
+        <is>
+          <t>Quelltext lesen, Laufzeit messen (T76), Engpass benennen.</t>
+        </is>
+      </c>
+      <c r="K91" s="57" t="inlineStr"/>
+      <c r="L91" s="57" t="inlineStr">
+        <is>
+          <t>PM-04</t>
+        </is>
+      </c>
+      <c r="M91" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M88"/>
+  <autoFilter ref="A1:M91"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Einkauf (Armin 2026-10-08, Punkt 4): product group in Spend-Aufriss via ZLO03 per purchased component
The product-group perspective only read MaterialUsageCache (86 rows, filled by hand
from the BOM page), so almost all spend showed "ohne Produktgruppe". The purchasing
run now asks ZSTR_LZCODE_USAGESet bottom-up per purchased material (short number and
its Disponent), 8 min budget per run, weekly recheck, 404-tolerant; new caches
PurchasingComponentDispoCache/State. No SAP change. Ceiling per ZPOWERBI_VC_TXT 72-77 % of spend.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -8766,15 +8766,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H90" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H90" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="I90" s="57" t="inlineStr"/>
       <c r="J90" s="57" t="inlineStr">
         <is>
-          <t>Konzept: ZC23-Zuordnung Disponent→Produktgruppe, ZLO03-Auflösung verkürzte Nummern, Mehrfachnennung.</t>
+          <t>Cockpit committet 08.10.: Einkauf-Lauf fragt je bestellter Komponente ZLO03 Bottom-Up (ZSTR_LZCODE_USAGESet) ab, Disponent der verkürzten Nummer → ZC23, 1/n bei Mehrfachnennung; ohne SAP-Änderung. Ursache „fehlt“: Verwendungs-Cache hatte nur 86 Zeilen. Obergrenze laut VC_TXT rund 72–77 % des Spends. Offen: Deploy, nach 1–2 Läufen Anteil messen und mit Armin prüfen; Umlaut-Fehler ZDISPO_SPART-Texte (P76) und doppelte Regeln DS1/DS2/016 klären.</t>
         </is>
       </c>
       <c r="K90" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: deploy 2026-10-08 15:03 (Einkauf contracts/LZ, product group ZLO03, Shopfloor no-cache)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -8719,7 +8719,7 @@
       <c r="I89" s="57" t="inlineStr"/>
       <c r="J89" s="57" t="inlineStr">
         <is>
-          <t>Cockpit committet 08.10.; T76K912724 dann T76K912718 nach P76, Caches leeren, Einkauf-Lauf, Wert gegen ME3L (16–17 Mio) mit Armin prüfen. Offen mit Armin: nur Bsart MK?</t>
+          <t>Cockpit produktiv 08.10. 15:03; T76K912724 dann T76K912718 nach P76, Caches leeren, Einkauf-Lauf, Wert gegen ME3L (16–17 Mio) mit Armin prüfen. Offen mit Armin: nur Bsart MK?</t>
         </is>
       </c>
       <c r="K89" s="57" t="inlineStr"/>
@@ -8774,7 +8774,7 @@
       <c r="I90" s="57" t="inlineStr"/>
       <c r="J90" s="57" t="inlineStr">
         <is>
-          <t>Cockpit committet 08.10.: Einkauf-Lauf fragt je bestellter Komponente ZLO03 Bottom-Up (ZSTR_LZCODE_USAGESet) ab, Disponent der verkürzten Nummer → ZC23, 1/n bei Mehrfachnennung; ohne SAP-Änderung. Ursache „fehlt“: Verwendungs-Cache hatte nur 86 Zeilen. Obergrenze laut VC_TXT rund 72–77 % des Spends. Offen: Deploy, nach 1–2 Läufen Anteil messen und mit Armin prüfen; Umlaut-Fehler ZDISPO_SPART-Texte (P76) und doppelte Regeln DS1/DS2/016 klären.</t>
+          <t>Cockpit produktiv 08.10. 15:03: Einkauf-Lauf fragt je bestellter Komponente ZLO03 Bottom-Up (ZSTR_LZCODE_USAGESet) ab, Disponent der verkürzten Nummer → ZC23, 1/n bei Mehrfachnennung; ohne SAP-Änderung. Ursache „fehlt“: Verwendungs-Cache hatte nur 86 Zeilen. Obergrenze laut VC_TXT rund 72–77 % des Spends. Offen: Deploy, nach 1–2 Läufen Anteil messen und mit Armin prüfen; Umlaut-Fehler ZDISPO_SPART-Texte (P76) und doppelte Regeln DS1/DS2/016 klären.</t>
         </is>
       </c>
       <c r="K90" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: ZM_OFFENE_FAUF columns visible incl. plant, layout learning; ZLO03 meaning of Exklusiv (B63491), TSTC ZLO03 -> Z_ZLO03_TURBO2
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -4021,7 +4021,7 @@
       <c r="I11" s="57" t="inlineStr"/>
       <c r="J11" s="57" t="inlineStr">
         <is>
-          <t>Ann-Katrin Michel vorwarnen: Spalte Exklusiv liefert künftig auch "?"</t>
+          <t>Ann-Katrin Michel vorwarnen: Spalte Exklusiv liefert künftig auch "?" | 08.10.: Bedeutung „Exklusiv“ für Ann-Katrin erklärt (B63491, zlo03/EXKLUSIV_LOGIK_2026-10-08.md), Antwort als .eml bei Ingo.</t>
         </is>
       </c>
       <c r="K11" s="57" t="inlineStr"/>
@@ -8580,7 +8580,7 @@
       </c>
       <c r="E87" s="57" t="inlineStr">
         <is>
-          <t>ZM_OFFENE_FAUF: Bedarfsverursacher (Dispoelement, Nummer, Daten zum Dispoelement) als einblendbare Felder</t>
+          <t>ZM_OFFENE_FAUF: Bedarfsverursacher (Dispoelement, Nummer, Daten zum Dispoelement, Werk), standardmässig sichtbar</t>
         </is>
       </c>
       <c r="F87" s="57" t="inlineStr">
@@ -8601,7 +8601,7 @@
       <c r="I87" s="57" t="inlineStr"/>
       <c r="J87" s="57" t="inlineStr">
         <is>
-          <t>In T76 fertig und getestet (07.10.), Transport T76K912714. Ingo: in T76 ansehen, freigeben, nach P76 importieren; Bestellabruf klären; Z_PEG_TEST ($TMP) löschen?</t>
+          <t>T76 fertig 08.10.: Spalten sichtbar, Feld Werk (MDRQ-WERKS) neu, Standardlayout / P00 TX in T76 ergänzt; alles in T76K912714. Ingo: freigeben und nach P76 importieren, danach Layout in P76 (Fabio). Offen: Fall BANF in 1200 prüfen (zeigt Werk 1200 oder den Umlagerungsbedarf in 1100?).</t>
         </is>
       </c>
       <c r="K87" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: ZZPRDAT acceptance test postponed two weeks (from 12.10.), Marco's polling load concern noted for logistics live sets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -6774,7 +6774,7 @@
       </c>
       <c r="E57" s="57" t="inlineStr">
         <is>
-          <t>ZZPRDAT: Ergebnis des Tests vom 17.09. mit Lucas festhalten</t>
+          <t>ZZPRDAT: Ergebnis des Abnahmetests mit Lucas festhalten</t>
         </is>
       </c>
       <c r="F57" s="57" t="inlineStr">
@@ -6794,12 +6794,12 @@
       </c>
       <c r="I57" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J57" s="57" t="inlineStr">
         <is>
-          <t>Test hat noch nicht stattgefunden: Lucas hat ihn auf 12.10.2026 16:00 gelegt (Marco, Adil, Ingo; Ingo hat am 01.10. zugesagt). Danach Ergebnis festhalten.</t>
+          <t>12.10.: Test (geplant 12.10. 16:00, Lucas, Marco, Adil, Ingo) um zwei Wochen verschoben, voraussichtlich Woche ab 26.10.2026, genauer Termin offen. Technik in T76 unverändert seit 07.09. (T76K912490 offen). Danach Ergebnis festhalten. saptasks/ZZPRDAT_TRANSPORTPLAN.md</t>
         </is>
       </c>
       <c r="K57" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs ZLO03: record time-of-day dependency reported by Ann-Katrin, todo row 94
Batch jobs end around 06:32 (SM37 13.10.), so they do not explain the
afternoon differences. Candidates and read-only next steps documented.
LEARNINGS: reindex must not be wrapped with *>&1 in PowerShell 5.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$95</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="J8" s="98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="99" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -8993,8 +8993,71 @@
       <c r="L94" s="57" t="inlineStr"/>
       <c r="M94" s="57" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="57" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="B95" s="57" t="inlineStr">
+        <is>
+          <t>Heute</t>
+        </is>
+      </c>
+      <c r="C95" s="57" t="inlineStr">
+        <is>
+          <t>SAP ZLO03</t>
+        </is>
+      </c>
+      <c r="D95" s="57" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="E95" s="57" t="inlineStr">
+        <is>
+          <t>ZLO03 liefert je nach Tageszeit verschieden viele VKNR (Meldung Ann-Katrin, für „5 to X“)</t>
+        </is>
+      </c>
+      <c r="F95" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G95" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H95" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I95" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="J95" s="57" t="inlineStr">
+        <is>
+          <t>13.10.: Batch-Jobs enden laut SM37 um etwa 06:32 und erklären die Unterschiede am Nachmittag nicht. Nur lesend prüfen: ZM_LZCODES20_BG/ZM_LZCODE20_BG (ZLO03N/NN), Z_ZLO03_TURBO2, Job-Schritte (TBTCP), SM37 ohne Benutzerfilter; Ann-Katrin fragen, ob der Effekt noch auftritt. zlo03/TAGESZEIT_ABHAENGIGKEIT_2026-10-13.md</t>
+        </is>
+      </c>
+      <c r="K95" s="57" t="inlineStr"/>
+      <c r="L95" s="57" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="M95" s="124" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M94"/>
+  <autoFilter ref="A1:M95"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Wochen_Todo: Data Lake performance (row 44, PM-11) done per Ingo; HERMES note on row 92, lastchange, LEARNINGS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -731,7 +731,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="145">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1134,6 +1134,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="33" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1867,7 +1870,7 @@
       </c>
       <c r="B5" s="76" t="n"/>
       <c r="C5" s="86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="78" t="n"/>
       <c r="E5" s="87" t="n">
@@ -1879,7 +1882,7 @@
       </c>
       <c r="H5" s="82" t="n"/>
       <c r="I5" s="138" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" s="137" t="n"/>
       <c r="K5" s="89" t="n">
@@ -2037,7 +2040,7 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" ht="53" customHeight="1" s="48">
@@ -2256,7 +2259,7 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" s="48">
@@ -2649,7 +2652,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="53" customHeight="1" s="48">
+    <row r="18" ht="38" customHeight="1" s="48">
       <c r="A18" s="92" t="inlineStr">
         <is>
           <t>PM-11</t>
@@ -2665,9 +2668,9 @@
           <t>Kleinauftrag</t>
         </is>
       </c>
-      <c r="D18" s="139" t="inlineStr">
-        <is>
-          <t>●  Neu</t>
+      <c r="D18" s="110" t="inlineStr">
+        <is>
+          <t>●  Grün</t>
         </is>
       </c>
       <c r="E18" s="108" t="inlineStr">
@@ -2690,22 +2693,22 @@
           <t>–  nicht nötig</t>
         </is>
       </c>
-      <c r="I18" s="140" t="inlineStr">
-        <is>
-          <t>–  nicht nötig</t>
+      <c r="I18" s="144" t="inlineStr">
+        <is>
+          <t>✔  13.10.2026</t>
         </is>
       </c>
       <c r="J18" s="98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="99" t="inlineStr">
         <is>
-          <t>Andreas hat am 28.09.2026 um eine Abstimmung zum Data Lake gebeten; Abgrenzung zu PM-09 (Tempo der Webapp) klären.</t>
+          <t>Erledigt laut Ingo am 13.10.2026 (Sitzung).</t>
         </is>
       </c>
       <c r="L18" s="99" t="inlineStr">
         <is>
-          <t>Klären, welche Leistung gemeint ist, und danach messen; je nach Befund ein Vorhaben daraus machen.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M18" s="99" t="inlineStr">
@@ -6075,18 +6078,22 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H45" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H45" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I45" s="57" t="inlineStr"/>
       <c r="J45" s="57" t="inlineStr">
         <is>
-          <t>Klären, welche Leistung gemeint ist und wie sie sich von PM-09 abgrenzt; danach messen und einen kurzen Befund schreiben.</t>
-        </is>
-      </c>
-      <c r="K45" s="57" t="inlineStr"/>
+          <t>Klären, welche Leistung gemeint ist und wie sie sich von PM-09 abgrenzt; danach messen und einen kurzen Befund schreiben. | 13.10.: Laut Ingo erledigt (Sitzung 13.10.2026).</t>
+        </is>
+      </c>
+      <c r="K45" s="57" t="inlineStr">
+        <is>
+          <t>2026-10-13 09:26</t>
+        </is>
+      </c>
       <c r="L45" s="57" t="inlineStr">
         <is>
           <t>PM-11</t>
@@ -8939,7 +8946,7 @@
       <c r="I93" s="57" t="inlineStr"/>
       <c r="J93" s="57" t="inlineStr">
         <is>
-          <t>Produktiv 09.10. 10:18, Sichtprüfung mit Testprojekt bestanden (danach archiviert). CSS-Korrektur produktiv 11:07. Offen: erstes echtes Projekt anlegen. Abgleich mit Philip Steiger bleibt sinnvoll.</t>
+          <t>Produktiv 09.10. 10:18, Sichtprüfung mit Testprojekt bestanden (danach archiviert). CSS-Korrektur produktiv 11:07. Offen: erstes echtes Projekt anlegen. Abgleich mit Philip Steiger bleibt sinnvoll. | 13.10.: HERMES-Angaben je Projekt, Reiter Portfolio (HERMES) und Demoprojekt HDEMO gebaut (7e20f93); Vorhaben der Wochen-Todo bewusst nicht übernommen.</t>
         </is>
       </c>
       <c r="K93" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: SAP authorization case Wolfurt (contract 46010612, M_RAHM_EKO EKORG 1200), strategy for authorization cases, read-only P76 GUI tools, LEARNINGS, Wochen_Todo 95
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$96</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M95"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9063,8 +9063,55 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="57" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="B96" s="57" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C96" s="57" t="inlineStr">
+        <is>
+          <t>SAP Berechtigung</t>
+        </is>
+      </c>
+      <c r="D96" s="57" t="inlineStr"/>
+      <c r="E96" s="57" t="inlineStr">
+        <is>
+          <t>Wolfurt: Abruf gegen Rahmenvertrag 46010612 (BLS Sarah, GAL Alexandra) scheitert an M_RAHM_EKO EKORG 1200</t>
+        </is>
+      </c>
+      <c r="F96" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G96" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H96" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I96" s="57" t="inlineStr"/>
+      <c r="J96" s="57" t="inlineStr">
+        <is>
+          <t>13.10.: Ursache lesend in P76 gefunden (AT-Rolle ZD_SD_SUPAUS_ADMIN_RW_AT erlaubt M_RAHM_EKO nur EKORG 1100). Uebergang: Z_MM_BESTAND_RW mit Enddatum an BLS/GAL, Sarah testet, sonst SU53. Hauptadmin: M_RAHM_EKO 1200 in AT-Rolle ergaenzen, Z_MM_BESTAND_RW entfernen. Doku saptasks/BERECHTIGUNG_RAHMENVERTRAG_AT_2026-10-13.md</t>
+        </is>
+      </c>
+      <c r="K96" s="57" t="inlineStr"/>
+      <c r="L96" s="57" t="inlineStr"/>
+      <c r="M96" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M95"/>
+  <autoFilter ref="A1:M96"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Docs: Operations KPI and Shopfloor mapping deployed 10:04/10:11, live pull needs role ZF_BR_SALES_MANAGER for ZPOWERBI, LEARNINGS (3), Wochen_Todo 87/96
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$97</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -8675,7 +8675,7 @@
       <c r="I88" s="57" t="inlineStr"/>
       <c r="J88" s="57" t="inlineStr">
         <is>
-          <t>Produktiv 08.10.; T76K912718 am 09.10. von Ingo nach P76 importiert, Caches geleert, SAP-Abgleich seit 09.10. 11:32 eingeschaltet (werktags 05:45 und 12:45). Erster Lauf 11:33: ZD05 58 Positionen, 6'449 Aufträge, 3'858 im Forecast bis 06.11. 14.10.: Feld-Mapping-Excel übernommen (b613f7c): Abteilung über Disponent (SEH S*, TR5 EK*, TX EL*, DW D*, CZ 017–028), nur FPY aus MES, Mapping je Feld auf der Seite Schnittstelle. Offen: 134 Felder Status offen (Spalten J–N Ingo), Disponenten auf „prüfen“ (012, 013, PKA, TL1, TPT u. a.), Übergabe 04:00 als Abruf oder Push entscheiden; Freigabe durch Leitung Produktion/Operations (vorher keine Ankündigung).</t>
+          <t>Produktiv 08.10.; T76K912718 am 09.10. von Ingo nach P76 importiert, Caches geleert, SAP-Abgleich seit 09.10. 11:32 eingeschaltet (werktags 05:45 und 12:45). Erster Lauf 11:33: ZD05 58 Positionen, 6'449 Aufträge, 3'858 im Forecast bis 06.11. 14.10.: Feld-Mapping-Excel übernommen (b613f7c, produktiv 10:04, danach nur noch 294 statt 1'912 Aufträge ohne Abteilung): Abteilung über Disponent (SEH S*, TR5 EK*, TX EL*, DW D*, CZ 017–028), nur FPY aus MES, Mapping je Feld auf der Seite Schnittstelle. Offen: 134 Felder Status offen (Spalten J–N Ingo), Disponenten auf „prüfen“ (012, 013, PKA, TL1, TPT u. a.), Übergabe 04:00 als Abruf oder Push entscheiden; Freigabe durch Leitung Produktion/Operations (vorher keine Ankündigung).</t>
         </is>
       </c>
       <c r="K88" s="57" t="inlineStr"/>
@@ -9110,8 +9110,55 @@
       <c r="L96" s="57" t="inlineStr"/>
       <c r="M96" s="57" t="inlineStr"/>
     </row>
+    <row r="97">
+      <c r="A97" s="57" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="B97" s="57" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C97" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D97" s="57" t="inlineStr"/>
+      <c r="E97" s="57" t="inlineStr">
+        <is>
+          <t>Operations &gt; KPI: Liefertreue OTD / OTIF / OTP (Spezifikation Fabio Palma)</t>
+        </is>
+      </c>
+      <c r="F97" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G97" s="57" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H97" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I97" s="57" t="inlineStr"/>
+      <c r="J97" s="57" t="inlineStr">
+        <is>
+          <t>14.10.: gebaut und produktiv 10:04 (89e9c7c, 982e193), Menü Operations &gt; KPI und Shopfloor, Abnahmewerte aus Fabios Daten exakt. Live-Abruf scheitert: technischer Cockpit-Benutzer ZPOWERBI braucht Rolle ZF_BR_SALES_MANAGER (Query 2CCSDSLSORDDLVPRFQ), KOI hat sie schon; danach Abruf 202609 gegen Abnahme prüfen, Antwort an Fabio (Feiertage?).</t>
+        </is>
+      </c>
+      <c r="K97" s="57" t="inlineStr"/>
+      <c r="L97" s="57" t="inlineStr"/>
+      <c r="M97" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M96"/>
+  <autoFilter ref="A1:M97"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Docs: low dashboard usage (findings, causes, measures), usage measurement deployed, Wochen_Todo 97
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$98</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9157,8 +9157,59 @@
       <c r="L97" s="57" t="inlineStr"/>
       <c r="M97" s="57" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" s="57" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="B98" s="57" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C98" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D98" s="57" t="inlineStr"/>
+      <c r="E98" s="57" t="inlineStr">
+        <is>
+          <t>Geringe Nutzung des Dashboards: messen und Massnahmen (Ersetzen statt ergänzen, Besitzer je Bereich, ins Meeting holen)</t>
+        </is>
+      </c>
+      <c r="F98" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G98" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H98" s="59" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I98" s="57" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="J98" s="57" t="inlineStr">
+        <is>
+          <t>14.10.: anonyme Nutzungsmessung produktiv (4615268, Admin &gt; Nutzung). Zwei bis vier Wochen messen, dann Seiten mit Besitzern besprechen; Massnahmen in docs/NUTZUNG_2026-10-14.md.</t>
+        </is>
+      </c>
+      <c r="K98" s="57" t="inlineStr"/>
+      <c r="L98" s="57" t="inlineStr"/>
+      <c r="M98" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M97"/>
+  <autoFilter ref="A1:M98"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Docs: Operations login switch (8bfe424, deploy pending); ZC23 material share analysis (ZM03 source from T76, proposal, open questions); Wochen_Todo 103/104, xlsx regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$105</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M102"/>
+  <dimension ref="A1:M105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9338,15 +9338,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H101" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H101" s="57" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
         </is>
       </c>
       <c r="I101" s="57" t="inlineStr"/>
       <c r="J101" s="57" t="inlineStr">
         <is>
-          <t>15.10. beim Prüfen der Weitergabe an Fabio gefunden: appsettings.json im Git enthält die Hashes. In eine Server-Einstellung auslagern, die nicht eingecheckt wird; Deploy darf sie nicht überschreiben.</t>
+          <t>15.10.: Teilschritt umgesetzt (e1afd49, produktiv 15.10. 10:56): Passwörter liegen deploy-fest in der Cockpit-DB und werden unter Admin &gt; Passwörter gesetzt; appsettings ist nur noch Rückfall. Nach dem Deploy setzt Ingo alle Bereiche dort neu, danach die alten Hashes in appsettings.json leeren oder ersetzen. 15.10. beim Prüfen der Weitergabe an Fabio gefunden: appsettings.json im Git enthält die Hashes. In eine Server-Einstellung auslagern, die nicht eingecheckt wird; Deploy darf sie nicht überschreiben.</t>
         </is>
       </c>
       <c r="K101" s="57" t="inlineStr"/>
@@ -9404,8 +9404,149 @@
       <c r="L102" s="57" t="inlineStr"/>
       <c r="M102" s="57" t="inlineStr"/>
     </row>
+    <row r="103">
+      <c r="A103" s="57" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="B103" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C103" s="57" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="D103" s="57" t="inlineStr"/>
+      <c r="E103" s="57" t="inlineStr">
+        <is>
+          <t>Passwörter aller Bereiche (Admin, Finance, HR, Operations, Logistik) im Admin setzbar, gespeichert in der DB</t>
+        </is>
+      </c>
+      <c r="F103" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G103" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H103" s="57" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="I103" s="57" t="inlineStr"/>
+      <c r="J103" s="57" t="inlineStr">
+        <is>
+          <t>15.10.: Seite Admin &gt; Passwörter produktiv (e1afd49, Deploy 10:56, 1232/1232). Ingo setzt dort das Admin-Passwort und bei Bedarf die übrigen.</t>
+        </is>
+      </c>
+      <c r="K103" s="57" t="inlineStr"/>
+      <c r="L103" s="57" t="inlineStr"/>
+      <c r="M103" s="57" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="57" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="B104" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C104" s="57" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D104" s="57" t="inlineStr"/>
+      <c r="E104" s="57" t="inlineStr">
+        <is>
+          <t>Operations-Login per Admin-Schalter abschaltbar (alle sehen dasselbe, Wunsch Fabio)</t>
+        </is>
+      </c>
+      <c r="F104" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G104" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H104" s="57" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="I104" s="57" t="inlineStr"/>
+      <c r="J104" s="57" t="inlineStr">
+        <is>
+          <t>15.10.: gebaut und getestet (8bfe424, 1234/1234), Schalter unter Admin &gt; Passwörter, Standard Login nötig. Deploy offen.</t>
+        </is>
+      </c>
+      <c r="K104" s="57" t="inlineStr"/>
+      <c r="L104" s="57" t="inlineStr"/>
+      <c r="M104" s="57" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="57" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="B105" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C105" s="57" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D105" s="57" t="inlineStr"/>
+      <c r="E105" s="57" t="inlineStr">
+        <is>
+          <t>ZC23: neue Spalte Materialanteil (Material aus der Standardkalkulation wie ZM03)</t>
+        </is>
+      </c>
+      <c r="F105" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G105" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H105" s="60" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I105" s="57" t="inlineStr"/>
+      <c r="J105" s="57" t="inlineStr">
+        <is>
+          <t>15.10.: Analyse ZM03 fertig (saptasks/zc23_materialanteil/NOTES.md). Offen: welche Kalkulation (jüngste oder freigegebene), Fremdleistung zu Material oder Arbeit, auch ins Dashboard? Einbau in ZM_OFFENE_KDAUF_OPT, zusammen mit Transport T76K912728.</t>
+        </is>
+      </c>
+      <c r="K105" s="57" t="inlineStr"/>
+      <c r="L105" s="57" t="inlineStr"/>
+      <c r="M105" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M102"/>
+  <autoFilter ref="A1:M105"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
ZC23 material share: ABAP prepared (selection, calculation like ZM03, ALV columns, ZPOWERBI_KDAUF fields), SAP scripts find the T76 connection, learnings
Decisions Ingo 2026-10-15: costing (released or latest) and external processing
selectable on the selection screen; standard value and material share also in
ZPOWERBI_KDAUF (Power BI). Built via bauen.js parts, REF unchanged, calculation runs
after vergleich_export so the CMP comparison stays clean. Nothing changed in T76 yet:
the SE11 step was denied by auto mode and waits for Ingo's go-ahead.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9530,15 +9530,15 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H105" s="60" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H105" s="57" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
         </is>
       </c>
       <c r="I105" s="57" t="inlineStr"/>
       <c r="J105" s="57" t="inlineStr">
         <is>
-          <t>15.10.: Analyse ZM03 fertig (saptasks/zc23_materialanteil/NOTES.md). Offen: welche Kalkulation (jüngste oder freigegebene), Fremdleistung zu Material oder Arbeit, auch ins Dashboard? Einbau in ZM_OFFENE_KDAUF_OPT, zusammen mit Transport T76K912728.</t>
+          <t>15.10.: Entscheide Ingo: Kalkulation und Fremdleistung im Selektionsbild wählbar, Standardwert + Materialanteil auch in ZPOWERBI_KDAUF (Power BI). ABAP im Repository fertig (bauen.js, teile/opt_mata_*). Einbau in T76 offen: SE11-Änderung vom Auto-Modus abgelehnt, braucht Freigabe Ingo. Schritte in saptasks/zc23_materialanteil/NOTES.md.</t>
         </is>
       </c>
       <c r="K105" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
ZC23 material share: fast level-wise loading and on/off switch, copied into ZM_OFFENE_KDAUF (T76K912736 complete); NA fix deployed 12:48; docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9532,13 +9532,13 @@
       </c>
       <c r="H105" s="57" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Wartet</t>
         </is>
       </c>
       <c r="I105" s="57" t="inlineStr"/>
       <c r="J105" s="57" t="inlineStr">
         <is>
-          <t>15.10.: in T76 eingebaut (Transport T76K912736: ZMM_UEB_KDAUF, ZPOWERBI_KDAUF, OData), OPT geprüft: Vergleich identisch, Werte = ZM03 und Nachrechnung. Offen: Laufzeit Q2 48 s statt 5 s (Entscheid Ingo), danach Übernahme in ZM_OFFENE_KDAUF, Freigabe und Import P76.</t>
+          <t>15.10.: in T76 fertig: Transport T76K912736 (ZMM_UEB_KDAUF, ZPOWERBI_KDAUF, OData, ZM_OFFENE_KDAUF), schnelle Fassung mit Schalter, Q2 13,5 s, Werte = ZM03. Offen: Ingo gibt T76K912736 frei, Import P76, Gateway-Caches leeren, ZC23 ansehen.</t>
         </is>
       </c>
       <c r="K105" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Fiori: first test app ZFI_ERSTE_APP (read-only, ZPOWERBI_EINKAUF_SRV) with harness notes, T76 prerequisites, upload paths; learnings, router, Wochen_Todo 105
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$106</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M105"/>
+  <dimension ref="A1:M106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9545,8 +9545,55 @@
       <c r="L105" s="57" t="inlineStr"/>
       <c r="M105" s="57" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" s="57" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="B106" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C106" s="57" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D106" s="57" t="inlineStr"/>
+      <c r="E106" s="57" t="inlineStr">
+        <is>
+          <t>Erste Fiori-App (Harness fuer kuenftige Erfassungs-Apps), nur lesen, T76 $TMP</t>
+        </is>
+      </c>
+      <c r="F106" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G106" s="57" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H106" s="57" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="I106" s="57" t="inlineStr"/>
+      <c r="J106" s="57" t="inlineStr">
+        <is>
+          <t>15.10.: App ZFI_ERSTE_APP gebaut (saptasks/fiori_erste_app), T76-Voraussetzungen geprueft (S/4 2023, UI5 758, Port 8000). Offen: Upload in T76 (Weg A von Hand per /UI5/UI5_REPOSITORY_LOAD oder Freigabe fuer RFC-Weg B), dann Link oeffnen.</t>
+        </is>
+      </c>
+      <c r="K106" s="57" t="inlineStr"/>
+      <c r="L106" s="57" t="inlineStr"/>
+      <c r="M106" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M105"/>
+  <autoFilter ref="A1:M106"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Fiori: ZFI_ERSTE_APP runs in browser (App wrapper and full height, client-side $top because service ignores it); cache and height learnings; coordination closed, Wochen_Todo 105 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9577,18 +9577,22 @@
           <t>Niedrig</t>
         </is>
       </c>
-      <c r="H106" s="57" t="inlineStr">
-        <is>
-          <t>Wartet</t>
+      <c r="H106" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I106" s="57" t="inlineStr"/>
       <c r="J106" s="57" t="inlineStr">
         <is>
-          <t>15.10.: App ZFI_ERSTE_APP gebaut (saptasks/fiori_erste_app), T76-Voraussetzungen geprueft (S/4 2023, UI5 758, Port 8000). In T76 hochgeladen per RFC /UI5/REPO_LOAD_FROM_ZIP, ICF-Knoten aktiv. Offen: Ingo oeffnet http://travt762.sap.trafag.com:8000/sap/bc/ui5_ui5/sap/zfi_erste_app/index.html?sap-client=100.</t>
-        </is>
-      </c>
-      <c r="K106" s="57" t="inlineStr"/>
+          <t>15.10.: Schritt 1 erledigt: ZFI_ERSTE_APP in T76, laeuft im Browser (50 Zeilen ProductDivisionRefSet). Link http://travt762.sap.trafag.com:8000/sap/bc/ui5_ui5/sap/zfi_erste_app/index.html?sap-client=100. Naechster Schritt bei Bedarf: Erfassung (CREATE) oder Launchpad-Kachel.</t>
+        </is>
+      </c>
+      <c r="K106" s="57" t="inlineStr">
+        <is>
+          <t>15.10.2026</t>
+        </is>
+      </c>
       <c r="L106" s="57" t="inlineStr"/>
       <c r="M106" s="57" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Docs: ZC23 Fiori app done in T76 (T76K912738), verified against ZPOWERBI_KDAUF; notes, router, baum, lastchange, Wochen_Todo 106, learnings, OData user POWERBI; coordination closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$107</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9596,8 +9596,55 @@
       <c r="L106" s="57" t="inlineStr"/>
       <c r="M106" s="57" t="inlineStr"/>
     </row>
+    <row r="107">
+      <c r="A107" s="57" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="B107" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C107" s="57" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D107" s="57" t="inlineStr"/>
+      <c r="E107" s="57" t="inlineStr">
+        <is>
+          <t>Fiori-App ZC23 live mit Selektion, Kacheln und Trafag-Logo (Zc23Set)</t>
+        </is>
+      </c>
+      <c r="F107" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G107" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H107" s="57" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="I107" s="57" t="inlineStr"/>
+      <c r="J107" s="57" t="inlineStr">
+        <is>
+          <t>15.10.: in T76 fertig und geprueft (Q2 gleich ZPOWERBI_KDAUF). Transport T76K912738 (ZM_OFFENE_KDAUF P_APP, ZSTR_ZC23_APP, MPC/DPC). App ZFI_ZC23 in $TMP. Offen: Ingo/Armin sehen an; T76 ist eine alte Kopie, live erst nach Import P76 (App dafuer mit Paket/Transport neu hochladen).</t>
+        </is>
+      </c>
+      <c r="K107" s="57" t="inlineStr"/>
+      <c r="L107" s="57" t="inlineStr"/>
+      <c r="M107" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M106"/>
+  <autoFilter ref="A1:M107"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Docs: operations open for all deployed 07:48 (70a02b1); Wochen_Todo 103 done; learning; coordination closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9483,18 +9483,22 @@
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H104" s="57" t="inlineStr">
-        <is>
-          <t>In Arbeit</t>
+      <c r="H104" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I104" s="57" t="inlineStr"/>
       <c r="J104" s="57" t="inlineStr">
         <is>
-          <t>15.10.: produktiv 12:15 (8bfe424), Freigabe Produktionsleitung erteilt. Offen: Ingo legt unter Admin &gt; Passwörter „Operations: Login nötig“ auf aus.</t>
-        </is>
-      </c>
-      <c r="K104" s="57" t="inlineStr"/>
+          <t>15.10.: produktiv 12:15 (8bfe424), Freigabe Produktionsleitung erteilt. 16.10.: Login aus über Shopfloor:OpenForAll = true (70a02b1, produktiv 07:48); der Admin-Schalter hat weiter Vorrang, falls er gesetzt wird.</t>
+        </is>
+      </c>
+      <c r="K104" s="57" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
       <c r="L104" s="57" t="inlineStr"/>
       <c r="M104" s="57" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Handbook: operations chapter extended (business process, every shopfloor page with interpretation, glossary); Word regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$109</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M108"/>
+  <dimension ref="A1:M109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9694,8 +9694,59 @@
       <c r="L108" s="57" t="inlineStr"/>
       <c r="M108" s="57" t="inlineStr"/>
     </row>
+    <row r="109">
+      <c r="A109" s="57" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="B109" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C109" s="57" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D109" s="57" t="inlineStr"/>
+      <c r="E109" s="57" t="inlineStr">
+        <is>
+          <t>Benutzerhandbuch Kapitel Operations erweitern (alle Seiten, Interpretation, Geschaeftsprozess)</t>
+        </is>
+      </c>
+      <c r="F109" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G109" s="57" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H109" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I109" s="57" t="inlineStr"/>
+      <c r="J109" s="57" t="inlineStr">
+        <is>
+          <t>16.10.: Kapitel 10 neu (Geschaeftsprozess, 18 Seitenabschnitte, Glossar 21 Begriffe), Word neu, deployed</t>
+        </is>
+      </c>
+      <c r="K109" s="57" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+      <c r="L109" s="57" t="inlineStr"/>
+      <c r="M109" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M108"/>
+  <autoFilter ref="A1:M109"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
Handbook: operations quick overview with process graphic (Trafag CI), image lines in tab and Word; shopfloor SAP quantities live (P76 verified, first run)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9687,7 +9687,7 @@
       <c r="I108" s="57" t="inlineStr"/>
       <c r="J108" s="57" t="inlineStr">
         <is>
-          <t>16.10.: produktiv 07:06 (b2103a4, 1240/1240), im Browser geprueft (Lieferzeiten, Ampel, Forecast DS, DW1 ohne Abteilung). ZD05 seit 16.10. um 04:00 und 12:45 (a285009). Speichertest Ampel produktiv ok. 16.10.: J5 Logistik, J8 SEH/TR5, J11 FPY SEH gebaut (ShopRmSet/ShopProdSet T76, gegen ZC27 gleich; Cockpit 2bc54bd, Schreiben aus). Offen: Ingo transportiert T76K912740 + T76K912738, dann Abgleich P76 und einschalten; J2/J3 Verkauf (KEA0), J6 Auftragsvorrat, Lieferzeit-Ziele Daniel Tobler. Ampel seit 07:37 loeschbar, planned_source aus Fabios Paketen wird gelesen (e6c007f)</t>
+          <t>16.10.: produktiv 07:06 (b2103a4, 1240/1240), im Browser geprueft (Lieferzeiten, Ampel, Forecast DS, DW1 ohne Abteilung). ZD05 seit 16.10. um 04:00 und 12:45 (a285009). Speichertest Ampel produktiv ok. 16.10.: J5 Logistik, J8 SEH/TR5, J11 FPY SEH gebaut (ShopRmSet/ShopProdSet T76, gegen ZC27 gleich; Cockpit 2bc54bd, Schreiben aus). P76 importiert, Vorschau gleich Kontrollwerten, seit 09:51 live (9d6b5d2). Offen: J2/J3 Verkauf (KEA0), J6 Auftragsvorrat, Lieferzeit-Ziele Daniel Tobler. Ampel seit 07:37 loeschbar, planned_source aus Fabios Paketen wird gelesen (e6c007f)</t>
         </is>
       </c>
       <c r="K108" s="57" t="inlineStr"/>
@@ -9734,7 +9734,7 @@
       <c r="I109" s="57" t="inlineStr"/>
       <c r="J109" s="57" t="inlineStr">
         <is>
-          <t>16.10.: Kapitel 10 neu (Geschaeftsprozess, 18 Seitenabschnitte, Glossar 21 Begriffe), Word neu, deployed</t>
+          <t>16.10.: Kapitel 10 neu (Geschaeftsprozess, 18 Seitenabschnitte, Glossar 21 Begriffe), Word neu, deployed; Schnellueberblick mit Prozessgrafik (Trafag CI) ergaenzt</t>
         </is>
       </c>
       <c r="K109" s="57" t="inlineStr">

</xml_diff>

<commit_message>
Docs: BOM brain (handbook Einkauf section, Fachdoku, router, baum, Wochen_Todo 109, deploy 10:48, learnings)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$110</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3356,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M109"/>
+  <dimension ref="A1:M110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="47" min="1" max="1"/>
@@ -9745,8 +9745,59 @@
       <c r="L109" s="57" t="inlineStr"/>
       <c r="M109" s="57" t="inlineStr"/>
     </row>
+    <row r="110">
+      <c r="A110" s="57" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="B110" s="57" t="inlineStr">
+        <is>
+          <t>Umsetzung</t>
+        </is>
+      </c>
+      <c r="C110" s="57" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D110" s="57" t="inlineStr"/>
+      <c r="E110" s="57" t="inlineStr">
+        <is>
+          <t>Stücklisten-Netz „Gehirn“ im Spend-Aufriss (Prototyp, WebGL, Farbe umschaltbar)</t>
+        </is>
+      </c>
+      <c r="F110" s="57" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G110" s="57" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="H110" s="58" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="I110" s="57" t="inlineStr"/>
+      <c r="J110" s="57" t="inlineStr">
+        <is>
+          <t>16.10.: live 10:48 (d6ca646), 11'005 Materialien, 24'979 Stränge; später ganze Stückliste aus SAP</t>
+        </is>
+      </c>
+      <c r="K110" s="57" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+      <c r="L110" s="57" t="inlineStr"/>
+      <c r="M110" s="57" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M109"/>
+  <autoFilter ref="A1:M110"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>

</xml_diff>

<commit_message>
ZLO03 docs: wording 'mechanism proven, case proof after import'; ABAP before/after FIX 12 versioned; row-order candidate for time-of-day issue (Wochen_Todo 94); baseline test step
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -3965,7 +3965,7 @@
       <c r="I10" s="57" t="inlineStr"/>
       <c r="J10" s="57" t="inlineStr">
         <is>
-          <t>16.10.: Ursache MK-Abweichung B63485 in P76 belegt (Textpositionen in 46123/24/26/28, Kennzahlen nur beim ersten Treffer). FIX 12 in Z_ZLO03_TURBO2 T76 aktiv, Transport T76K912742: Ingo freigeben/importieren, dann in P76 testen und Ann-Katrin antworten. Fixes 10/11/15 weiter nur lokal. zlo03/MK_B63485_FIX12_2026-10-16.md | vorher: Diagnoselauf p_diag und Regressionstest, danach Transport nach B76</t>
+          <t>16.10.: Mechanismus MK-Abweichung B63485 in P76 belegt (Textpositionen in 46123/24/26/28, Kennzahlen nur beim ersten Treffer), Nachweis am Fall erst nach Import. FIX 12 in Z_ZLO03_TURBO2 T76 aktiv, Transport T76K912742: Ingo freigeben/importieren, dann in P76 testen und Ann-Katrin antworten. Fixes 10/11/15 weiter nur lokal. zlo03/MK_B63485_FIX12_2026-10-16.md | vorher: Diagnoselauf p_diag und Regressionstest, danach Transport nach B76</t>
         </is>
       </c>
       <c r="K10" s="57" t="inlineStr"/>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="J95" s="57" t="inlineStr">
         <is>
-          <t>13.10.: Batch-Jobs enden laut SM37 um etwa 06:32 und erklären die Unterschiede am Nachmittag nicht. Nur lesend prüfen: ZM_LZCODES20_BG/ZM_LZCODE20_BG (ZLO03N/NN), Z_ZLO03_TURBO2, Job-Schritte (TBTCP), SM37 ohne Benutzerfilter; Ann-Katrin fragen, ob der Effekt noch auftritt. zlo03/TAGESZEIT_ABHAENGIGKEIT_2026-10-13.md</t>
+          <t>16.10.: neuer Kandidat Satzreihenfolge/Textposition (Bottom-Up loescht VKNR mit leerem Text), passt zu B64404; P76 lesen KOMPNR=B64404, POSTYP. FIX 12 in T76 (T76K912742). | 13.10.: Batch-Jobs enden laut SM37 um etwa 06:32 und erklären die Unterschiede am Nachmittag nicht. Nur lesend prüfen: ZM_LZCODES20_BG/ZM_LZCODE20_BG (ZLO03N/NN), Z_ZLO03_TURBO2, Job-Schritte (TBTCP), SM37 ohne Benutzerfilter; Ann-Katrin fragen, ob der Effekt noch auftritt. zlo03/TAGESZEIT_ABHAENGIGKEIT_2026-10-13.md</t>
         </is>
       </c>
       <c r="K95" s="57" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: closing round dashboard/data lake in lastchange and PROJEKTSTATUS (PM-10, PM-12), PM-11 aligned with HERMES (done 13.10.), new PM-13 SAP PS, PS addendum (external costs, P76, slides 11-16)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -2889,7 +2889,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="68" customHeight="1" s="62">
+    <row r="19" ht="83" customHeight="1" s="62">
       <c r="A19" s="126" t="inlineStr">
         <is>
           <t>PM-12</t>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="K19" s="133" t="inlineStr">
         <is>
-          <t>Neu aufgenommen am 29.09.2026; die Liste der Dashboards und ihre Zuordnung zu Fachbereichen fehlt noch.</t>
+          <t>Neu aufgenommen am 29.09.2026; die Liste der Dashboards und ihre Zuordnung zu Fachbereichen fehlt noch. Am 20.10.2026 zur Abschlussrunde mit allen Bereichen eingeladen, Datenverantwortung ist dort Agendapunkt.</t>
         </is>
       </c>
       <c r="L19" s="133" t="inlineStr">

</xml_diff>

<commit_message>
ZLO03: transport T76K912742 released by Ingo (FIX 12, 19 incl. RoHS, 20); FIX 21 real .xlsx export (CL_ABAP_ZIP, OOXML, formulas kept) prepared in repo only, prototype cell-identical to text import (126x182 and 331x2097), needs new transport
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -10210,7 +10210,7 @@
       <c r="I115" s="7" t="inlineStr"/>
       <c r="J115" s="7" t="inlineStr">
         <is>
-          <t>20.10.: FIX 19 (REACH, SVHC, PFAS-Gehalt aus Z_PACK_REGULATION) in T76 aktiv, in T76K912742; Lauf fehlerfrei, Spalten leer (T76 ohne Werte). Offen: Test mit Werten (Testklassifizierung T76 oder nach Import P76), RoHS-Merkmal durch Adil (Vorschlag ROHSCOM). 22.10.: Adil hat Merkmal ROHS angelegt, Spalte RoHS (vor REACH) in T76 aktiv, gleicher Auftrag; ob ROHS in P76 existiert, ungeprueft. Offen: Test mit Werten, Import P76 (Ingo). zlo03/FIX19_STOFFCOMPLIANCE_SPALTEN_2026-10-20.md</t>
+          <t>20.10.: FIX 19 (REACH, SVHC, PFAS-Gehalt aus Z_PACK_REGULATION) in T76 aktiv, in T76K912742; Lauf fehlerfrei, Spalten leer (T76 ohne Werte). Offen: Test mit Werten (Testklassifizierung T76 oder nach Import P76), RoHS-Merkmal durch Adil (Vorschlag ROHSCOM). 22.10.: Adil hat Merkmal ROHS angelegt, Spalte RoHS (vor REACH) in T76 aktiv, gleicher Auftrag; ob ROHS in P76 existiert, ungeprueft. Offen: Test mit Werten, Import P76 (Ingo; T76K912742 am 22.10. freigegeben). zlo03/FIX19_STOFFCOMPLIANCE_SPALTEN_2026-10-20.md</t>
         </is>
       </c>
       <c r="K115" s="7" t="inlineStr"/>
@@ -10445,7 +10445,7 @@
       <c r="I120" s="7" t="inlineStr"/>
       <c r="J120" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Ursache Gruppenrichtlinie ExtensionHardening = 2, Datei selbst korrekt (als .txt lesbar). FIX 20 (Download .txt, Oeffnen mit Excel) in T76 aktiv, in T76K912742. Sofortloesung: Datei in .txt umbenennen. Offen: Programm hinter ZLO03 in P76 pruefen, Import P76, Benutzer informieren. zlo03/FIX20_DOWNLOAD_TXT_2026-10-22.md</t>
+          <t>22.10.: Ursache Gruppenrichtlinie ExtensionHardening = 2, Datei selbst korrekt (als .txt lesbar). FIX 20 (Download .txt, Oeffnen mit Excel) in T76 aktiv, in T76K912742. Sofortloesung: Datei in .txt umbenennen. Offen: Programm hinter ZLO03 in P76 pruefen, Import P76, Benutzer informieren. 22.10.: T76K912742 von Ingo freigegeben. Auf Wunsch Ingo FIX 21 (echtes .xlsx) vorbereitet, Prototyp zellgleich; braucht neuen Auftrag (Entscheid Ingo). zlo03/FIX20_DOWNLOAD_TXT_2026-10-22.md</t>
         </is>
       </c>
       <c r="K120" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Handbestellwesen: analysis of legacy PHP order app and concept for replacement as dashboard module (decisions Ingo: module, migrate data from dump, master data local then SAP, GUI like PHP); legacy folder gitignored (plaintext passwords); docs, Wochen_Todo 120
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$121</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M120"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="62" min="1" max="1"/>
@@ -10452,8 +10452,55 @@
       <c r="L120" s="7" t="inlineStr"/>
       <c r="M120" s="7" t="inlineStr"/>
     </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr"/>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Handbestellwesen: PHP-Anwendung (Student, privater Hoster) durch Modul im Dashboard abloesen</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
+        <is>
+          <t>Wartet auf Input</t>
+        </is>
+      </c>
+      <c r="I121" s="7" t="inlineStr"/>
+      <c r="J121" s="7" t="inlineStr">
+        <is>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP. Naechster Schritt: MySQL-Dump von Ingo, Owner/Freigabe Fachabteilung klaeren. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
+        </is>
+      </c>
+      <c r="K121" s="7" t="inlineStr"/>
+      <c r="L121" s="7" t="inlineStr"/>
+      <c r="M121" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M120">
+  <autoFilter ref="A1:M121">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Einkauf"/>

</xml_diff>

<commit_message>
Handbestellwesen concept: answers Ingo (hosted locally at Trafag, users without SAP account, plugin/KISS, AD, later SAP write with indirect-use licence question), no dump in folder; Wochen_Todo 98 closed (Einkauf delta 14.10 succeeded, checked read-only in PurchasingSyncState)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -9390,7 +9390,7 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>Heute</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -9414,18 +9414,22 @@
           <t>Hoch</t>
         </is>
       </c>
-      <c r="H99" s="155" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="H99" s="151" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="I99" s="7" t="inlineStr"/>
       <c r="J99" s="7" t="inlineStr">
         <is>
-          <t>Auf /einkauf/ideen/datenservice nachsehen, ob ein Lauf „beim Start abgebrochen“ ist, und ihn bei Bedarf neu starten. Ursache und Regel in docs/rag/LEARNINGS.md (2026-10-14).</t>
-        </is>
-      </c>
-      <c r="K99" s="7" t="inlineStr"/>
+          <t>22.10.: In PurchasingSyncState geprueft (Produktiv-DB nur lesend): Delta 14.10. erfolgreich (11:12 UTC), Lauf 15.10. abgebrochen und sofort erfolgreich wiederholt; seither taeglich erfolgreich, zuletzt 21.10. 12:29-13:12.</t>
+        </is>
+      </c>
+      <c r="K99" s="7" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
       <c r="L99" s="7" t="inlineStr"/>
       <c r="M99" s="7" t="inlineStr"/>
     </row>
@@ -10471,7 +10475,7 @@
       <c r="D121" s="7" t="inlineStr"/>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>Handbestellwesen: PHP-Anwendung (Student, privater Hoster) durch Modul im Dashboard abloesen</t>
+          <t>Handbestellwesen: PHP-Anwendung (Student, lokal bei Trafag) durch Plugin-Modul im Dashboard abloesen</t>
         </is>
       </c>
       <c r="F121" s="7" t="inlineStr">
@@ -10492,7 +10496,7 @@
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP. Naechster Schritt: MySQL-Dump von Ingo, Owner/Freigabe Fachabteilung klaeren. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). Naechster Schritt: MySQL-Dump von Ingo, Owner/Freigabe Fachabteilung klaeren. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Handbestellwesen phase 1: new top-level tab /handbestellwesen as plugin module (own SQLite DB with backup, GUI like the PHP app, limit/approval/goods receipt/delete checked server-side, per-(year, cost centre) counter in a transaction, audit log); 9 tests, suite 1274/1274; not deployed; gitignore anchored to root; docs, learnings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -10490,13 +10490,13 @@
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>Wartet auf Input</t>
+          <t>In Arbeit</t>
         </is>
       </c>
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). Naechster Schritt: MySQL-Dump von Ingo, Owner/Freigabe Fachabteilung klaeren. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: Einkauf meeting 2026-10-22 (dashboard stabilise until 28.10, feedback list, new supplier evaluation request, Handbestellwesen shutdown vs replacement open); Wochen_Todo 120 updated, 121/122 new
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$123</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M123"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="62" min="1" max="1"/>
@@ -10490,21 +10490,119 @@
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Wartet auf Entscheid</t>
         </is>
       </c>
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>
       <c r="L121" s="7" t="inlineStr"/>
       <c r="M121" s="7" t="inlineStr"/>
     </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr"/>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Einkaufs-Dashboard: Zwischenstand bis 28.10. stabilisieren, Feedbackliste Erich/Sandro/Marco abarbeiten</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H122" s="7" t="inlineStr">
+        <is>
+          <t>Wartet auf Input</t>
+        </is>
+      </c>
+      <c r="I122" s="7" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="J122" s="7" t="inlineStr">
+        <is>
+          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md</t>
+        </is>
+      </c>
+      <c r="K122" s="7" t="inlineStr"/>
+      <c r="L122" s="7" t="inlineStr"/>
+      <c r="M122" s="7" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>Nur terminieren</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr"/>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>Lieferantenbewertung und -entwicklung im Dashboard (SAP-Kennzahlen plus Eingaben: Zertifikate ISO 9001, Massnahmen, Zusatzfragen, Audits)</t>
+        </is>
+      </c>
+      <c r="F123" s="7" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="G123" s="7" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H123" s="7" t="inlineStr">
+        <is>
+          <t>Wartet auf Input</t>
+        </is>
+      </c>
+      <c r="I123" s="7" t="inlineStr"/>
+      <c r="J123" s="7" t="inlineStr">
+        <is>
+          <t>Sitzung 22.10.: Einkauf schickt Word-Dokument und Dashboard-Entwurf, nennt Datenquellen (SAP-Tabellen/Transaktionen); Fiori-Parametrisierung der neuen Lieferantenbewertung ist Voraussetzung (eigene Aufgabe, NTT). Danach kleiner Pilot; Eingaben mit Schreibrecht nur fuer Berechtigte. docs/EINKAUF_SITZUNG_2026-10-22.md</t>
+        </is>
+      </c>
+      <c r="K123" s="7" t="inlineStr"/>
+      <c r="L123" s="7" t="inlineStr"/>
+      <c r="M123" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M121">
+  <autoFilter ref="A1:M123">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Einkauf"/>

</xml_diff>

<commit_message>
Handbestellwesen: decision Ingo 22.10 keep it running but record usage; page visits once per account and day, admin tile Nutzung with orders/CHF/visits per person, cost centre and month (deleted excluded); test, suite 1275/1275; docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -10490,13 +10490,13 @@
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>Wartet auf Entscheid</t>
+          <t>In Arbeit</t>
         </is>
       </c>
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md Entscheid 22.10. (Ingo): lebt weiter, Nutzung festhalten (wer/wann/wie viel) -&gt; umgesetzt (Aufrufe je Tag, Kachel Nutzung, Suite 1275/1275). Naechster Schritt: Dump von Tobias, Deploy-Entscheid.</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Einkauf feedback Erich/Sandro/Marco 22.10: superseded contract items (never called off, sibling fully called off) excluded from open value and listed separately; expired-only filter; legacy text items (due > 1 year) no longer open/overdue; applied-period label, not-applied warning, calculating ring; stock value by MRP controller; drop top-spend row; hide coverage, material dependency, interactive once; BOM brain collapsed; Handbestellwesen tab seeded hidden; translations; tests, suite 1279/1279; docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -8314,7 +8314,7 @@
       <c r="I79" s="7" t="inlineStr"/>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>Einkauf informieren, dass endgelieferte Positionen seit 06.10. nicht mehr als offen zählen (ISS-031).</t>
+          <t>Einkauf informieren, dass endgelieferte Positionen seit 06.10. nicht mehr als offen zählen (ISS-031). 22.10.: zusaetzlich zaehlen alte Textpositionen (Termin &gt; 1 Jahr vorbei, 168 Pos. CHF 3,1 Mio.) nicht mehr als offen/ueberfaellig; beides dem Einkauf mitteilen.</t>
         </is>
       </c>
       <c r="K79" s="7" t="inlineStr"/>
@@ -8904,7 +8904,7 @@
       <c r="I89" s="7" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>T76K912724 und T76K912718 am 09.10. in P76, Caches geleert, Delta 09.10. 12:27 erfolgreich: 1'262 Kontraktpositionen, 35'042 LZ-Codes, offener Kontraktwert CHF 18,67 Mio. inkl. abgelaufener Kontrakte. Offen mit Armin: Abweichung zu ME3L (16–17 Mio.), nur Bsart MK?</t>
+          <t>T76K912724 und T76K912718 am 09.10. in P76, Caches geleert, Delta 09.10. 12:27 erfolgreich: 1'262 Kontraktpositionen, 35'042 LZ-Codes, offener Kontraktwert CHF 18,67 Mio. inkl. abgelaufener Kontrakte. Offen mit Armin: Abweichung zu ME3L (16–17 Mio.), nur Bsart MK? 22.10.: Teil der Abweichung gefunden: nie abgerufene, durch eine andere Position ersetzte Kontraktpositionen (46009671 Pos. 10 u. a., 4 Pos. CHF 1,29 Mio.) zaehlen nicht mehr; ME3L zeigt sie weiter offen -&gt; in SAP loeschen lassen.</t>
         </is>
       </c>
       <c r="K89" s="7" t="inlineStr"/>
@@ -10537,7 +10537,7 @@
       </c>
       <c r="H122" s="7" t="inlineStr">
         <is>
-          <t>Wartet auf Input</t>
+          <t>In Arbeit</t>
         </is>
       </c>
       <c r="I122" s="7" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md</t>
+          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md 22.10.: Feedbackliste erhalten und umgesetzt (Kontrakt-Ersetzung, Filter abgelaufene, Altposten Textpositionen, Hinweis Zeitraum, Lagerwert je Disponent, Ausblendungen). Offen: Deploy, Rueckfrage Sandro Zeitraum. PURCHASING_DASHBOARD Nachtrag 2026-10-22.</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: deploy 2026-10-22 13:38 (77778a5, Einkauf feedback + Handbestellwesen module, tab hidden), weekly backup; Handbestellwesen dump (8 tables) and latest PHP files received, findings (central db_config, htaccess without dot so Basic Auth inactive)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -10496,7 +10496,7 @@
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md Entscheid 22.10. (Ingo): lebt weiter, Nutzung festhalten (wer/wann/wie viel) -&gt; umgesetzt (Aufrufe je Tag, Kachel Nutzung, Suite 1275/1275). Naechster Schritt: Dump von Tobias, Deploy-Entscheid.</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md Entscheid 22.10. (Ingo): lebt weiter, Nutzung festhalten (wer/wann/wie viel) -&gt; umgesetzt (Aufrufe je Tag, Kachel Nutzung, Suite 1275/1275). Naechster Schritt: Dump von Tobias, Deploy-Entscheid. 22.10. nachmittags: Modul deployed (Reiter unsichtbar), Dump (8 Tabellen) und neueste PHP-Dateien erhalten; Basic-Auth-Datei heisst htaccess ohne Punkt, Schutz nicht aktiv. Naechster Schritt: Import-Werkzeug.</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md 22.10.: Feedbackliste erhalten und umgesetzt (Kontrakt-Ersetzung, Filter abgelaufene, Altposten Textpositionen, Hinweis Zeitraum, Lagerwert je Disponent, Ausblendungen). Offen: Deploy, Rueckfrage Sandro Zeitraum. PURCHASING_DASHBOARD Nachtrag 2026-10-22.</t>
+          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md 22.10.: Feedbackliste erhalten und umgesetzt (Kontrakt-Ersetzung, Filter abgelaufene, Altposten Textpositionen, Hinweis Zeitraum, Lagerwert je Disponent, Ausblendungen). Offen: Deploy, Rueckfrage Sandro Zeitraum. PURCHASING_DASHBOARD Nachtrag 2026-10-22. Deployed 22.10. 13:38 (77778a5).</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: Wochen_Todo nachgefuehrt (Handbestellwesen AD/Altbestand, Einkauf 27.10.), mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -10496,7 +10496,7 @@
       <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md Entscheid 22.10. (Ingo): lebt weiter, Nutzung festhalten (wer/wann/wie viel) -&gt; umgesetzt (Aufrufe je Tag, Kachel Nutzung, Suite 1275/1275). Naechster Schritt: Dump von Tobias, Deploy-Entscheid. 22.10. nachmittags: Modul deployed (Reiter unsichtbar), Dump (8 Tabellen) und neueste PHP-Dateien erhalten; Basic-Auth-Datei heisst htaccess ohne Punkt, Schutz nicht aktiv. Naechster Schritt: Import-Werkzeug. Import gebaut (Admin-Kachel Altdaten-Import, Fehler korrigiert statt uebernommen), Probelauf 12629 Bestellungen; 930 offene aelter als 1 Jahr -&gt; Entscheid Ingo. Import produktiv 14:27 (Ingo); Datenpruefung: keine doppelten Nummern, 25 Doppelklick-Doubletten, ~930 alte offene; Bereinigung als Admin-Funktion deployed, Knoepfe drueckt Ingo. 27.10.: PHP abgeschaltet (PHP-Luecke), Reiter sichtbar, Link klassisch -&gt; neue Version, Freigabe wie PHP (umschaltbar auf gleiche KoSt), a0030e8; offen: Zugriff, Grundtests durch Anwender, Rechnungsbetrag/Mail. Stammdaten loeschen + AD-Uebernahme (a8e9eec).</t>
+          <t>22.10.: Analyse (SQL-Injection, Passwoerter im Code, Limit nur im Browser, Nummernkollision 87/875) und Konzept; Entscheide Ingo: Modul im Dashboard, Altdaten uebernehmen, Stammdaten zuerst lokal dann SAP, Oberflaeche wie im PHP, AD-Benutzer, KISS/Plugin, spaeter Schreiben nach SAP (Lizenzfrage indirekte Nutzung klaeren, Benutzer ohne SAP-Konto). 22.10. Phase 1 programmiert (Reiter /handbestellwesen, eigene DB, Pruefungen auf dem Server, 9 Tests, Suite 1274/1274), nicht deployed. Naechster Schritt: MySQL-Dump von Tobias (Import), Owner/Freigabe Fachabteilung, Entscheid Deploy. docs/HANDBESTELLWESEN_KONZEPT_2026-10-22.md Sitzung Einkauf 22.10.: Abschalten statt Abloesen steht im Raum (Anlass Vorfall 21.10.); Inbetriebnahme erst nach Grundsatzentscheid, Entscheidungstraeger offen. docs/EINKAUF_SITZUNG_2026-10-22.md Entscheid 22.10. (Ingo): lebt weiter, Nutzung festhalten (wer/wann/wie viel) -&gt; umgesetzt (Aufrufe je Tag, Kachel Nutzung, Suite 1275/1275). Naechster Schritt: Dump von Tobias, Deploy-Entscheid. 22.10. nachmittags: Modul deployed (Reiter unsichtbar), Dump (8 Tabellen) und neueste PHP-Dateien erhalten; Basic-Auth-Datei heisst htaccess ohne Punkt, Schutz nicht aktiv. Naechster Schritt: Import-Werkzeug. Import gebaut (Admin-Kachel Altdaten-Import, Fehler korrigiert statt uebernommen), Probelauf 12629 Bestellungen; 930 offene aelter als 1 Jahr -&gt; Entscheid Ingo. Import produktiv 14:27 (Ingo); Datenpruefung: keine doppelten Nummern, 25 Doppelklick-Doubletten, ~930 alte offene; Bereinigung als Admin-Funktion deployed, Knoepfe drueckt Ingo. 27.10.: PHP abgeschaltet (PHP-Luecke), Reiter sichtbar, Link klassisch -&gt; neue Version, Freigabe wie PHP (umschaltbar auf gleiche KoSt), a0030e8; offen: Zugriff, Grundtests durch Anwender, Rechnungsbetrag/Mail. Stammdaten loeschen + AD-Uebernahme (a8e9eec). Neue Mitarbeitende nur aus dem AD, AD-Eintraege gesperrt mit "Aus AD aktualisieren", Altbestand voll pflegbar (3ff16f5, Deploy ausstehend). Offen: Deploy 3ff16f5, Push, Pruefung AD-Suche auf dem Server, Rueckfrage PHP-Bestellungen 22.10. bis Abschaltung, Pflege durch IT ohne Admin?, Rechnungsbetrag/Mail, Bereinigungsknoepfe (Ingo).</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr"/>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md 22.10.: Feedbackliste erhalten und umgesetzt (Kontrakt-Ersetzung, Filter abgelaufene, Altposten Textpositionen, Hinweis Zeitraum, Lagerwert je Disponent, Ausblendungen). Offen: Deploy, Rueckfrage Sandro Zeitraum. PURCHASING_DASHBOARD Nachtrag 2026-10-22. Deployed 22.10. 13:38 (77778a5).</t>
+          <t>Sitzung 22.10.: bis 28.10. nichts Neues, Bestehendes zum Laufen bringen (Zwischenstand, Weiterarbeit danach moeglich). Einkauf teilt die Feedbackliste mit Quelle je Punkt; Rueckfragen direkt an die Person. docs/EINKAUF_SITZUNG_2026-10-22.md 22.10.: Feedbackliste erhalten und umgesetzt (Kontrakt-Ersetzung, Filter abgelaufene, Altposten Textpositionen, Hinweis Zeitraum, Lagerwert je Disponent, Ausblendungen). Offen: Deploy, Rueckfrage Sandro Zeitraum. PURCHASING_DASHBOARD Nachtrag 2026-10-22. Deployed 22.10. 13:38 (77778a5). 27.10.: Spend-Schalter Einkaufsteile (Disponent 001-005) deployed 08:26 (c3147e1); Produktgruppe zeigt nur noch SAP-Text, z. B. FP_DICHTEWAECH statt "D2 - FP_DICHTEWAECH", deployed 11:05 (0917d9e). Offen: SAP-Bereinigung Dubletten DS1/DS2/016 in ZDISPO_GRP.</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Docs: Sitzung SAP PS und Projektmanagement-Werkzeug 29.10. zusammengefasst (Router, baum, PROJEKTSTATUS PM-10/PM-13, Wochen_Todo 126), mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$127</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="62" min="1" max="1"/>
@@ -6197,7 +6197,7 @@
       <c r="I44" s="7" t="inlineStr"/>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>Projektauftrag in der Initialisierung schreiben (Vorlage im Blatt Vorlage Projektauftrag), Stufe nach Aufwandschätzung festlegen, Abgleich mit dem Project-Power-Pack-Test von Philip Steiger.</t>
+          <t>29.10.: Sitzung SAP PS/PPP: Philip fuehrt den Test des Project Power Pack weiter (Entscheid offen); Trafag Projekte bekommt Smartsheet-Modus (Bau ab 29.10.), vor breiter Ankuendigung mit Philip/Oskar abstimmen. docs/SITZUNG_SAP_PS_PROJEKTMANAGEMENT_2026-10-29.md | Projektauftrag in der Initialisierung schreiben (Vorlage im Blatt Vorlage Projektauftrag), Stufe nach Aufwandschätzung festlegen, Abgleich mit dem Project-Power-Pack-Test von Philip Steiger.</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr"/>
@@ -10758,8 +10758,67 @@
       <c r="L126" s="7" t="inlineStr"/>
       <c r="M126" s="7" t="inlineStr"/>
     </row>
+    <row r="127">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>PM-13</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>SAP PS: Sitzung 29.10. mit Philip, Oskar, Lucas (zwei Ebenen PPP/PS, Schnittstelle Projektstrukturplan)</t>
+        </is>
+      </c>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>Lucas / Philip / Ingo</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H127" s="153" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I127" s="7" t="inlineStr"/>
+      <c r="J127" s="7" t="inlineStr">
+        <is>
+          <t>29.10.: Lucas fragt bei NTT Data Offerte/Einfuehrung PS an; Philip liefert Testprojekte 133.2 und 103.46 plus Vorlage Produktentwicklung; beide in PS (T76) abbilden; danach Finance. Offene Fragen: WBS-Aenderung nach Buchung, CAPEX/OPEX, Zeiterfassung wo, Risiken finanziell. docs/SITZUNG_SAP_PS_PROJEKTMANAGEMENT_2026-10-29.md</t>
+        </is>
+      </c>
+      <c r="K127" s="7" t="inlineStr"/>
+      <c r="L127" s="7" t="inlineStr">
+        <is>
+          <t>PM-13</t>
+        </is>
+      </c>
+      <c r="M127" s="156" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M126">
+  <autoFilter ref="A1:M127">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Einkauf"/>

</xml_diff>

<commit_message>
Docs: Deploy 1e3300d Trafag Projekte (Smartsheet-Ansicht, Risiken, PMO, Vorhaben), LEARNINGS, Router, Wochen_Todo 127, Koordination abgeschlossen, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$128</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="J17" s="132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" s="133" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M127"/>
+  <dimension ref="A1:M128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="62" min="1" max="1"/>
@@ -10817,8 +10817,67 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t>Diese Woche</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>Projekte</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t>PM-10</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>Trafag Projekte: Smartsheet-Ansicht, Risiken mit Franken, Projektstrukturplan, Decision Log, Vorlagen, Uebernahme Vorhaben (Auftrag Ingo 29.10.)</t>
+        </is>
+      </c>
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G128" s="7" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="H128" s="153" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="I128" s="7" t="inlineStr"/>
+      <c r="J128" s="7" t="inlineStr">
+        <is>
+          <t>29.10.: Phase 1 und PMO produktiv seit 12:23 (1e3300d, 1311/1311). Offen: Sichtpruefung und einmal Balken ziehen produktiv (Ingo); Vorhaben einmal hochladen (Vorhaben_HERMES.tsv + Wochen_Todo.tsv); Abstimmung mit Philip/Oskar vor breiter Ankuendigung; Phase 2 Guide, Phase 3 Auslastung/Automatisierungen/Formulare. docs/TRAFAG_PROJEKTE_2026-10-09.md</t>
+        </is>
+      </c>
+      <c r="K128" s="7" t="inlineStr"/>
+      <c r="L128" s="7" t="inlineStr">
+        <is>
+          <t>PM-10</t>
+        </is>
+      </c>
+      <c r="M128" s="156" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M127">
+  <autoFilter ref="A1:M128">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Einkauf"/>

</xml_diff>

<commit_message>
Docs: ZLO03 Top-Down-Befunde fuer FIX 24 notiert (zlo03/CLAUDE.md G, Wochen_Todo 129), mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Wochen_Todo.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HERMES Übersicht'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'HERMES Übersicht'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wochen-Todo'!$A$1:$M$130</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Wochen-Todo'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Wochen-Todo'!$A$1:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Erläuterungen'!$1:$4</definedName>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="J8" s="124" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" s="125" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="62" min="1" max="1"/>
@@ -10935,8 +10935,67 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Später</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>SAP ZLO03</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>ZLO03 Top-Down: weitere Befunde fuer FIX 24 (Rundung Stueckkosten bei PEINH&gt;1, p_days wirkungslos, Textpositionen im Bedarf, Verdacht Mehrstufigkeit)</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="H130" s="155" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I130" s="7" t="inlineStr"/>
+      <c r="J130" s="7" t="inlineStr">
+        <is>
+          <t>29.10.: notiert, nicht umgesetzt (Ingo transportiert zuerst FIX 12 bis 23). Details zlo03/CLAUDE.md Offene Punkte G; Mehrstufigkeit erst gegen CS12 fuer 41019 pruefen.</t>
+        </is>
+      </c>
+      <c r="K130" s="7" t="inlineStr"/>
+      <c r="L130" s="7" t="inlineStr">
+        <is>
+          <t>PM-01</t>
+        </is>
+      </c>
+      <c r="M130" s="156" t="inlineStr">
+        <is>
+          <t>Vorhaben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M129">
+  <autoFilter ref="A1:M130">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Einkauf"/>

</xml_diff>